<commit_message>
18th Commit : Autoride Lifecycle Test Sutite Initated
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,17 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8B528C-B7DA-4F25-926E-8D3EAB7F5DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7556EA-947F-46E7-B25D-CE21925CDC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
-    <sheet name="HybridTestFlow" sheetId="31" r:id="rId2"/>
-    <sheet name="AddCustomer" sheetId="13" r:id="rId3"/>
-    <sheet name="AddCityArea" sheetId="1" r:id="rId4"/>
-    <sheet name="AddCityAdmin" sheetId="2" r:id="rId5"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId6"/>
+    <sheet name="HybridTestFlow" sheetId="31" r:id="rId1"/>
+    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId2"/>
+    <sheet name="AddAutoDriver" sheetId="32" r:id="rId3"/>
+    <sheet name="AutoRideLifecycleTest" sheetId="33" r:id="rId4"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,10 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="42">
-  <si>
-    <t>City Area</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -65,22 +61,13 @@
     <t>SA_TS_1</t>
   </si>
   <si>
-    <t>CityAdmin</t>
-  </si>
-  <si>
     <t>SA_TS_3</t>
   </si>
   <si>
     <t>SA_TS_4</t>
   </si>
   <si>
-    <t>SA_TS_5</t>
-  </si>
-  <si>
     <t>SA_TS_0</t>
-  </si>
-  <si>
-    <t>TC_CA_00_super_admin_login</t>
   </si>
   <si>
     <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
@@ -92,12 +79,6 @@
     <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation.</t>
   </si>
   <si>
-    <t>Validate the end-to-end creation of a City Area, including status configuration and polygon mapping. Verify data persistence by ensuring the new area is correctly listed and available for selection in 'City Wise Manage Services' in ' Transport Service ' and 'City Admin' modules.</t>
-  </si>
-  <si>
-    <t>To verify that the Super Admin can successfully create a new City Admin account by providing valid personal details, associating them with a specific city, and granting multiple service and module-level permissions.</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -188,191 +169,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The AddCityArea test suite must be always executed before this test. This is critical because the AddCityAdmin process utilizes the dynamic {areaName} variable generated and stored during the AddCityArea creation phase.
-RunSheet: AddCityArea</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>System State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-RunSheet: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SuperAdminLogin</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
-    </r>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>Validate the end-to-end creation of a Customer.</t>
-  </si>
-  <si>
     <t>Clean The Test Data Created During Test Run</t>
   </si>
   <si>
@@ -495,167 +291,6 @@
       <t xml:space="preserve">
 </t>
     </r>
-  </si>
-  <si>
-    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
-3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
-4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
-5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
-6.Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
-7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
-8.Open Gender,click,,"//span[@aria-label='select gender']"
-9.Select Male,click,,"//li[@aria-label='Male']"
-10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
-11.Click Submit, click, , "//button[normalize-space()='Submit']"
-12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-15.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-18.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-19.Click Edit Icon ,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-20.Click Close, click, , "//button[normalize-space()='Close']"
-21.Click Wallet Icon ,click,,"//i[@title='Wallet']"
-22.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-23.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-24.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-25.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-26.Click Submit, click, , "//button[normalize-space()='Submit']"
-27.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-28.Click Add Money ,click,,"//button[normalize-space()='Add Money']"
-29.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-30.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-31.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-32.Click Submit, click, , "//button[normalize-space()='Submit']"
-33.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-34. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-35. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-36.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-37. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-38.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-39.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-40.Click Loyalty Points Icon,click,,"//i[@title='Loyalty Points']"
-41.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-42.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-43.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-44.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-45.Select Add Points,click,,"//li[@role='option'][contains(.,'Add Points')]"
-46.Enter Points, type, 30, "//input[@placeholder='Enter Points']"
-47.Click Submit, click, , "//button[normalize-space()='Submit']"
-48.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-49.Click Manage Loyality Points, click, , "//button[normalize-space()='Manage Loyalty Points']"
-50.Open Service Dropdown,click,,"//label[contains(.,'Service')]/following-sibling::p-dropdown/div"
-51.Select Bike Ride,click,,"//li[@role='option'][contains(.,'Bike Ride')]"
-52.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-53.Select Deduct Points,click,,"//li[@role='option'][contains(.,'Deduct Points')]"
-54.Enter Points, type, 10, "//input[@placeholder='Enter Points']"
-55.Click Submit, click, , "//button[normalize-space()='Submit']"
-56.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-57. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-58. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-59.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-60. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-61.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-62.Scroll Grid, tab, 7, "//input[@aria-label='Customer Name Filter Input']"
-63.Click Disable  Icon,click,,"//i[@title='Block']"
-64.Click Disable  User  Yes,click,,"//button[normalize-space()='Yes']"
-65.Disable Reason,type,Client Complaints,"//textarea[@id='swal2-textarea']"
-66.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-67.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-68. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-69. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-70.Click  Blocked Customers,click,,"//span[normalize-space()='Blocked Customers']"
-71.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-72.Scroll Grid, tab, 10, "//input[@aria-label='Customer Name Filter Input']"
-73.Click Enable  Icon,click,,"//i[@title='Status']"
-74.Click Enable  Yes,click,,"//button[normalize-space()='Yes']"
-75. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-76. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-77.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-78. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-79.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-80.wait,1000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click City area menu,click,,"//span[normalize-space()='City Area']"
-3. Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-4. Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-5. Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-6. Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-7. Open Status Dropdown,click,,"//span[@aria-label='select status']"
-8. Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-9.Enter City Area, type, triplicane, "//input[@placeholder='Search location']"
-10.wait,1000,,
-11.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-12.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-13.wait,1000,,
-14. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-15. Click Submit,click,,"//button[normalize-space()='Submit']"
-16. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-17. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-18. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-19. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-20. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-21. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-22. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-23. Click close,click,,"//button[normalize-space()='Close']"
-19. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-24. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-25. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-26. Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-27. Open Select City Dropdown,click,,"//select[@id='cityId']"
-28. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-29. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
-5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Select Name field,click ,, "//input[@id='name']"
-8. Enter Admin Name, type, faizal{randomAlpha} &gt;&gt; adminName, "//input[@id='name']"
-9.Select Email field,click,, "//input[@id='email']"
-10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.select the password field,click,, "//input[@id='password']"
-12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Open Select City Dropdown,click,,"//select[@id='cityId']"
-14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
-18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
-22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
-39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
-40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-41.Click on the "Add City Admin" button. "//button[@type='submit']"
-42. Verify Success Message,verify,,"//div[@aria-label='Info']"
-43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
-</t>
   </si>
   <si>
     <t>Super Admin Login</t>
@@ -767,25 +402,388 @@
 </t>
   </si>
   <si>
-    <t>TC_CA_02_add_customer</t>
-  </si>
-  <si>
-    <t>TC_CA_03_add_city_area</t>
-  </si>
-  <si>
-    <t>TC_CA_04_add_city_admin</t>
-  </si>
-  <si>
-    <t>TC_CA_05_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>TC_CA_01_Hybrid_Test_Flow</t>
-  </si>
-  <si>
     <t>HybridFlow</t>
   </si>
   <si>
-    <t>HybridFlow for mobile and web Integrated work flow</t>
+    <t>Auto Driver Registration</t>
+  </si>
+  <si>
+    <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list .</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>TC_CA_00_Hybrid_Test_Flow</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Nill</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>This is just an hybrid test flow that  validates the cross-platform orchestration capabilities of the ABCD Automation Framework by shifting execution seamlessly among three separate driver contexts: Web Admin, User App, and Driver App. The script initiates with a standard login and dashboard verification on the web portal, transitions to the Appium-driven User and Driver emulators to verify basic native touch and configuration steps sequentially, and then returns control back to the web context.</t>
+  </si>
+  <si>
+    <t>TC_CA_01_super_admin_login</t>
+  </si>
+  <si>
+    <t>TC_CA_02_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_04_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>Auto Ride Complete Life Cycle Test</t>
+  </si>
+  <si>
+    <t>TC_CA_03_Autoride_Lifecycle_Test</t>
+  </si>
+  <si>
+    <t>This comprehensive end-to-end hybrid test validates the multi-platform orchestration and transactional workflow of the ABCD Framework by simulating a complete ride lifecycle across Web Admin, Driver, and User contexts. The execution flows sequentially from the Web Admin portal to register a new auto driver, switches to the Appium-driven Driver App to submit verification documents, and transitions back to Web Admin for regulatory approval and onboarding. The test then establishes parallel operations, shifting to the Driver App to go online, moving to the User App to dynamically book a ride, routing back to the Driver App to accept and complete the trip, and concludes with payment processing, data lifecycle validation, and transactional integrity verification across all application touchpoints.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin,AddAutoDriver
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+26. Click Submit, click, , "//button[contains(.,'Submit')]"
+27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+28. Wait for Toast to hide, wait, 1000,
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.wait,1000,,
+34.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+35.wait,1000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.wait,3000,,
+2.Load User App,switch_to,user,
+3.wait,2000,,
+4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+8.wait,2000,,
+9.Load Driver App,switch_to,driver,
+10.wait,2000,,
+11.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+12.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+13.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+14.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+15.wait,1000,,
+16.Load  Super Admin,switch_to,web,
+17.wait,2000,,
+</t>
   </si>
 </sst>
 </file>
@@ -851,7 +849,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -874,6 +872,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1154,64 +1155,64 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F96D9-3311-4A18-82B5-F5729925CB8A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1717BC20-9348-4B52-9588-34F52BC8B75D}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="36.88671875" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="57.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
     <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1230,7 +1231,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1717BC20-9348-4B52-9588-34F52BC8B75D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F96D9-3311-4A18-82B5-F5729925CB8A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1246,48 +1247,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1306,64 +1307,63 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECEE02-404F-4AF1-8311-95653C3B218B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC812CD8-667D-4888-8684-24E9CC12973D}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1371,10 +1371,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="E3" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1382,64 +1379,64 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E73811-1019-42A7-934A-5E2FAE40D576}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="57.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
     <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1458,71 +1455,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9466ABF-463D-46B5-A321-4AC4765F1CE7}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.33203125" customWidth="1"/>
-    <col min="2" max="2" width="19.88671875" customWidth="1"/>
-    <col min="3" max="3" width="25.44140625" customWidth="1"/>
-    <col min="4" max="4" width="34.77734375" customWidth="1"/>
-    <col min="5" max="5" width="64" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1538,48 +1470,48 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
19th Commit : Autoride Lifecycle Test Sutite Updated
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7556EA-947F-46E7-B25D-CE21925CDC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5BE3ED-FC6D-434D-9BEC-04E7DF7BE45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HybridTestFlow" sheetId="31" r:id="rId1"/>
@@ -729,6 +729,26 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">1.wait,3000,,
+2.Load User App,switch_to,user,
+3.wait,2000,,
+4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+8.wait,2000,,
+9.Load Driver App,switch_to,driver,
+10.wait,2000,,
+11.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+12.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+13.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+14.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+15.wait,1000,,
+16.Load  Super Admin,switch_to,web,
+17.wait,2000,,
+</t>
+  </si>
+  <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
@@ -737,11 +757,11 @@
 6. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
 7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
 8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-9. Enter Contact Number, type, {randomPhone}, "//input[@type='tel']"
+9. Enter Contact Number, type, {randomPhone}&gt;&gt;autoMobile, "//input[@type='tel']"
 10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
 11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
 12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+13.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
 14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
 15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
 16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
@@ -764,26 +784,6 @@
 33.wait,1000,,
 34.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
 35.wait,1000,,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.wait,3000,,
-2.Load User App,switch_to,user,
-3.wait,2000,,
-4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-8.wait,2000,,
-9.Load Driver App,switch_to,driver,
-10.wait,2000,,
-11.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-12.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-13.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-14.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-15.wait,1000,,
-16.Load  Super Admin,switch_to,web,
-17.wait,2000,,
-</t>
   </si>
 </sst>
 </file>
@@ -1360,7 +1360,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>25</v>
@@ -1433,7 +1433,7 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
20th Commit : Rebooter and Mobile Type Action Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D5BE3ED-FC6D-434D-9BEC-04E7DF7BE45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A848314F-AC2D-41C6-AFB5-AFDD1888E438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="HybridTestFlow" sheetId="31" r:id="rId1"/>
+    <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId2"/>
     <sheet name="AddAutoDriver" sheetId="32" r:id="rId3"/>
     <sheet name="AutoRideLifecycleTest" sheetId="33" r:id="rId4"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -65,9 +65,6 @@
   </si>
   <si>
     <t>SA_TS_4</t>
-  </si>
-  <si>
-    <t>SA_TS_0</t>
   </si>
   <si>
     <t>1. Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
@@ -349,62 +346,6 @@
 51.wait,2000,,</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Load Site,navigate,https://dev.we1.co/#/login,
-2.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-3.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-4.Click Login,click,,"//button[@type='submit']"
-5.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
-6.wait,5000,,
-7.Load User App,switch_to,user,
-8.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-9.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-10.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-11.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-12.wait,1000,,
-13.Load Driver App,switch_to,driver,
-14.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-15.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-16.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-17.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-18.wait,1000,,
-19.Load  Super Admn,switch_to,web,
-20.wait,1000,,
-21. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-22.Click City area menu,click,,"//span[normalize-space()='City Area']"
-23.Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-24.Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-25.Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-26.Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-27.Open Status Dropdown,click,,"//span[@aria-label='select status']"
-28.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-29.Enter City Area, type, triplicane, "//input[@placeholder='Search location']"
-30.wait,1000,,
-31.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-32.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-33.wait,1000,,
-34. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-35. Click Submit,click,,"//button[normalize-space()='Submit']"
-36. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-37. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-38. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-39. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-40. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-41. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-42. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-43. Click close,click,,"//button[normalize-space()='Close']"
-44. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-45. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-46. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-47.Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-48. Open Select City Dropdown,click,,"//select[@id='cityId']"
-49. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-50. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
-  </si>
-  <si>
-    <t>HybridFlow</t>
-  </si>
-  <si>
     <t>Auto Driver Registration</t>
   </si>
   <si>
@@ -500,102 +441,6 @@
       <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
 </t>
     </r>
-  </si>
-  <si>
-    <t>TC_CA_00_Hybrid_Test_Flow</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Nill</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
-  </si>
-  <si>
-    <t>This is just an hybrid test flow that  validates the cross-platform orchestration capabilities of the ABCD Automation Framework by shifting execution seamlessly among three separate driver contexts: Web Admin, User App, and Driver App. The script initiates with a standard login and dashboard verification on the web portal, transitions to the Appium-driven User and Driver emulators to verify basic native touch and configuration steps sequentially, and then returns control back to the web context.</t>
   </si>
   <si>
     <t>TC_CA_01_super_admin_login</t>
@@ -784,6 +629,30 @@
 33.wait,1000,,
 34.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
 35.wait,1000,,</t>
+  </si>
+  <si>
+    <t>SA_TS_00</t>
+  </si>
+  <si>
+    <t>Reboot Test</t>
+  </si>
+  <si>
+    <t>TC_CA_00_Reboot_Test</t>
+  </si>
+  <si>
+    <t>If in case emulators crashes wipe data and  cold reboot all emulators and run this test to make the emultators and web browser into initial state before running other tests</t>
+  </si>
+  <si>
+    <t>1.wait,3000,,
+2.Load Driver App,switch_to,driver,
+3.wait,2000,,
+4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+8.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+9.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+10.wait,3000,,</t>
   </si>
 </sst>
 </file>
@@ -1155,7 +1024,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1717BC20-9348-4B52-9588-34F52BC8B75D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5AE23A-69EB-46F0-86E8-8B9CD1BA86DE}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1197,22 +1066,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1276,19 +1145,19 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1351,19 +1220,19 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1424,19 +1293,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1499,19 +1368,19 @@
         <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
21th Commit : OTP Entering Mobile Type Action Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A848314F-AC2D-41C6-AFB5-AFDD1888E438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBC3F74-F9B5-4905-8275-F7F4F4840F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -652,7 +652,8 @@
 7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
 8.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
 9.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-10.wait,3000,,</t>
+10.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+10.wait,5000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
26th Commit : Working Code With Delay
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65658657-9CC7-4EB3-AF38-87F7C3562535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F00E4C1B-6259-4E99-83C4-0949878AABDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -626,38 +626,6 @@
     <t>c</t>
   </si>
   <si>
-    <t xml:space="preserve">1.wait,2000,,
-2.Load Driver App,switch_to,driver,
-3.wait,2000,,
-4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-15.wait,20000,,
-16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-19.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-21.Drag Page Layout Upward,swipe,up,
-22.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-23.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-25.wait,3000,,
-26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-27.wait,10000,,
-28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-29.wait,10000,,
-</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -794,6 +762,39 @@
 22.Load  Super Admin,switch_to,web,
 23.wait,2000,,
 </t>
+  </si>
+  <si>
+    <t>1.wait,2000,,
+2.Load Driver App,switch_to,driver,
+3.wait,2000,,
+4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+15.wait,10000,,
+16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+19.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+21.Drag Page Layout Upward,swipe,up,
+22.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+23.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+25.wait,3000,,
+26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+27.wait,10000,,
+28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+29.wait,15000,,
+30.Click Agree,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+31.wait,10000,,</t>
   </si>
 </sst>
 </file>
@@ -1219,10 +1220,10 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1443,7 +1444,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
27th Commit : Transistion Error Fixed
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F00E4C1B-6259-4E99-83C4-0949878AABDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54AF31BF-F297-40B1-97AC-0DBCB712849E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId2"/>
     <sheet name="AddAutoDriver" sheetId="32" r:id="rId3"/>
-    <sheet name="AutoRideLifecycleTest" sheetId="33" r:id="rId4"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId5"/>
+    <sheet name="TestRun" sheetId="33" r:id="rId4"/>
+    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId5"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="40">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -777,6 +778,31 @@
 11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
 12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
 13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+14.wait,4000
+15.Load User App,switch_to,user,
+16.wait,2000,,
+17.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+18.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+19.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+20.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+21.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+22.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+23.wait,2000,,</t>
+  </si>
+  <si>
+    <t>1.wait,2000,,
+2.Load Driver App,switch_to,driver,
+3.wait,2000,,
+4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
 15.wait,10000,,
 16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
@@ -793,8 +819,9 @@
 27.wait,10000,,
 28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 29.wait,15000,,
-30.Click Agree,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-31.wait,10000,,</t>
+30.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+31.Click Document,tap,,"//android.view.View[@content-desc="Documents"]"
+32.wait,10000,,</t>
   </si>
 </sst>
 </file>
@@ -1468,6 +1495,84 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79BE6A4-9FA5-4B28-B734-40C3B7520402}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
28th Commit : Explicit Wait Increased To Prevent Network Lag Crash
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54AF31BF-F297-40B1-97AC-0DBCB712849E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C264F89-23E1-45E2-80DB-843F929808FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -804,7 +804,7 @@
 12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
 13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-15.wait,10000,,
+15.wait,20000,,
 16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
 18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
@@ -816,7 +816,7 @@
 24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
 25.wait,3000,,
 26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-27.wait,10000,,
+27.wait,20000,,
 28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 29.wait,15000,,
 30.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"

</xml_diff>

<commit_message>
29th Commit :Mobile Image Upload Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C264F89-23E1-45E2-80DB-843F929808FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2886B7F1-F7D3-472E-B344-AF4802A6EDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -804,7 +804,7 @@
 12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
 13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-15.wait,20000,,
+15.wait,10000,,
 16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
 18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
@@ -816,12 +816,15 @@
 24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
 25.wait,3000,,
 26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-27.wait,20000,,
+27.wait,10000,,
 28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-29.wait,15000,,
+29.wait,10000,,
 30.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-31.Click Document,tap,,"//android.view.View[@content-desc="Documents"]"
-32.wait,10000,,</t>
+31.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
+32.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
+33.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
+34..Click License,tap,,"//*[contains(@text, 'license.JPG')] or //*[@text='license.JPG']"
+35.wait,10000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
32th Commit :Driver Approval Finished
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A39F430-5D35-4615-AE63-96A0FD90CF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ABCA96B-D77A-401F-AB90-B1B3108B7ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -834,7 +834,27 @@
 42.Click Upload,tap,,"//android.widget.Button[@content-desc="Upload Documents"]"
 43.wait,4000,,
 44.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-45.wait,10000,,</t>
+45.wait,5000,,
+46.Load Admin App,switch_to,web,
+47.wait,3000,,
+48. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+50.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+51.wait,1000,
+52.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+53.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+54.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+55.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+56.wait,1000,
+57.Click Approve Driver,click,,"//i[@title='Approve']"
+58.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+59.wait,3000,,
+60.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+61.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+62.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+63.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+64.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+65.wait,3000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
33th Commit :Wait For Visible Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ABCA96B-D77A-401F-AB90-B1B3108B7ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A6AD74-5AAB-4580-A9C0-2D6F53D8B1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -792,19 +792,23 @@
   <si>
     <t>1.wait,2000,,
 2.Load Driver App,switch_to,driver,
-3.wait,2000,,
+3.Wait For Notification,wait_until_visible,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
 4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
 5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
 6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
 7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
 8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+8.1.wait,4000,,
 9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+9.1.wait,4000,,
 10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+10.1.wait,4000,,
 11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+11.1.wait,4000,,
 12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
 13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-15.wait,10000,,
+15.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
 18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
@@ -816,11 +820,12 @@
 24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
 25.wait,3000,,
 26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-27.wait,10000,,
+27.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-29.wait,10000,,
+29.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
 30.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
 31.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
+31.1Wait For Upload,wait_until_visible,,"//android.widget.Button[@content-desc='Upload']"
 32.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
 33.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
 34.Click Sort,tap,,"//android.widget.TextView[@resource-id="com.google.android.documentsui:id/title" and @text="Sort by..."]"
@@ -854,7 +859,31 @@
 62.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 63.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
 64.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-65.wait,3000,,</t>
+65.wait,3000,,
+67.Load Driver App,switch_to,driver,
+68.wait,4000,,
+69.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
+70.wait,2000,,
+71.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+72.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+73.Click Online,tap,,"//android.view.View[@content-desc="autodriverHFRTSY Offline Ride Service Pink Auto"]"
+74.wait,5000,,
+75.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+76.Click Wallet,tap,,"//android.view.View[@content-desc="Wallet"]"
+77.wait,5000,,
+78.Click Topup,tap,,"//android.view.View[@content-desc="TopUp"]"
+79.Click Hundered,tap,,"//android.view.View[@content-desc="₹ 100.00"]"
+80.Click Proceed,tap,,"//android.widget.Button[@content-desc="Proceed"]"
+81.wait,10000,,
+82.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+83.Click Netbanking,tap,,"//android.view.View[@resource-id="mobile-nav"]/android.view.View/android.view.View/android.view.View[3]/android.view.View/android.widget.Image"
+84.Click Bob,tap,,"//android.widget.Button[@text="BOB BOB"]"
+85.wait,5000,,
+85.Click Success,tap,,"//android.widget.Button[@text="Success"]"
+86.wait,5000,,
+87.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+88.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+89.wait,5000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
34th Commit :Tap Cordinate Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A6AD74-5AAB-4580-A9C0-2D6F53D8B1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6637192A-677F-4FF9-B1E1-F5C98822756E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -790,100 +790,97 @@
 23.wait,2000,,</t>
   </si>
   <si>
-    <t>1.wait,2000,,
-2.Load Driver App,switch_to,driver,
-3.Wait For Notification,wait_until_visible,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-8.1.wait,4000,,
+    <t>1.Load Driver App,switch_to,driver,
+2.Wait For Notification,wait_until_visible,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+3.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+4.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+5.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+6.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+7.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+8.Wait for Mobile Number,wait_until_visible,,"//android.widget.Button[@content-desc="Mobile Number"]"
 9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-9.1.wait,4000,,
-10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-10.1.wait,4000,,
-11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-11.1.wait,4000,,
-12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-15.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-19.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-21.Drag Page Layout Upward,swipe,up,
-22.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-23.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-25.wait,3000,,
-26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-27.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-29.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-30.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-31.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
-31.1Wait For Upload,wait_until_visible,,"//android.widget.Button[@content-desc='Upload']"
-32.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
-33.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
-34.Click Sort,tap,,"//android.widget.TextView[@resource-id="com.google.android.documentsui:id/title" and @text="Sort by..."]"
-35.Click Modified,tap,,"//android.widget.CheckedTextView[@resource-id="android:id/text1" and @text="Modified (newest first)"]"
-36.Click License,tap,,"//android.widget.ImageView[@resource-id="com.google.android.documentsui:id/icon_thumb"]"
-37.Click Crop,tap,,"//android.widget.Button[@content-desc="Crop"]"
-38.Click Calender,tap,,"//android.widget.ImageView[contains(@content-desc, 'Driving Licence')]/android.view.View[2]/android.view.View"
-39.Click Month,tap,"//android.widget.Button[@content-desc="Next month"]"
-40.Click Date,tap,,"//android.widget.Button[contains(@content-desc, '25')]"
-41. Click Ok,tap,,"//android.widget.Button[@content-desc="OK"]"
-42.Click Upload,tap,,"//android.widget.Button[@content-desc="Upload Documents"]"
-43.wait,4000,,
-44.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-45.wait,5000,,
-46.Load Admin App,switch_to,web,
-47.wait,3000,,
-48. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-50.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-51.wait,1000,
-52.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-53.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-54.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-55.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-56.wait,1000,
-57.Click Approve Driver,click,,"//i[@title='Approve']"
-58.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-59.wait,3000,,
-60.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-61.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-62.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-63.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-64.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-65.wait,3000,,
+10.Wait for Close,wait_until_visible,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+12.Wait for Mobile Number,wait_until_visible,,"//android.widget.EditText"
+13.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+14.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+15.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+16.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+17.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+18.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+19.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+20.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+21.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+22.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+23.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+24.Drag Page Layout Upward,swipe,up,
+25.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+26.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+27.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+28.Wait For Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+29.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+30.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+31.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+32.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+33.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+34.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
+35.Wait For Upload,wait_until_visible,,"//android.widget.Button[@content-desc='Upload']"
+36.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
+37.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
+38.Click Sort,tap,,"//android.widget.TextView[@resource-id="com.google.android.documentsui:id/title" and @text="Sort by..."]"
+39.Click Modified,tap,,"//android.widget.CheckedTextView[@resource-id="android:id/text1" and @text="Modified (newest first)"]"
+40.Click License,tap,,"//android.widget.ImageView[@resource-id="com.google.android.documentsui:id/icon_thumb"]"
+41.Click Crop,tap,,"//android.widget.Button[@content-desc="Crop"]"
+42.Click Calender,tap,,"//android.widget.ImageView[contains(@content-desc, 'Driving Licence')]/android.view.View[2]/android.view.View"
+43.Click Month,tap,"//android.widget.Button[@content-desc="Next month"]"
+44.Click Date,tap,,"//android.widget.Button[contains(@content-desc, '25')]"
+45. Click Ok,tap,,"//android.widget.Button[@content-desc="OK"]"
+46.Click Upload,tap,,"//android.widget.Button[@content-desc="Upload Documents"]"
+47.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
+48.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+49.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+50.Load Admin App,switch_to,web,
+51.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+52.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+53.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+54.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+55.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+56.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+57.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+58.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+59.Click Approve Driver,click,,"//i[@title='Approve']"
+60.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+61.wait,3000,,
+62.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+63.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+64.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+65.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+66.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
 67.Load Driver App,switch_to,driver,
-68.wait,4000,,
+68.Wait For Document,wait_until_visible,,"//android.view.View[@content-desc='Documents']"
 69.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
-70.wait,2000,,
+70.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
 71.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
 72.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-73.Click Online,tap,,"//android.view.View[@content-desc="autodriverHFRTSY Offline Ride Service Pink Auto"]"
-74.wait,5000,,
-75.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-76.Click Wallet,tap,,"//android.view.View[@content-desc="Wallet"]"
-77.wait,5000,,
-78.Click Topup,tap,,"//android.view.View[@content-desc="TopUp"]"
-79.Click Hundered,tap,,"//android.view.View[@content-desc="₹ 100.00"]"
-80.Click Proceed,tap,,"//android.widget.Button[@content-desc="Proceed"]"
-81.wait,10000,,
-82.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-83.Click Netbanking,tap,,"//android.view.View[@resource-id="mobile-nav"]/android.view.View/android.view.View/android.view.View[3]/android.view.View/android.widget.Image"
-84.Click Bob,tap,,"//android.widget.Button[@text="BOB BOB"]"
-85.wait,5000,,
-85.Click Success,tap,,"//android.widget.Button[@text="Success"]"
-86.wait,5000,,
-87.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-88.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-89.wait,5000,,</t>
+73.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+74.Wait For Offline,wait_until_visible,,"//android.view.View[contains(@content-desc, 'Offline')]"
+75.Click Online,tap_coordinate,989:2045,
+76.wait,2000,,
+77.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+78.Click Wallet,tap,,"//android.view.View[@content-desc="Wallet"]"
+79.Wait For Topup,wait_until_visible,,"//android.view.View[@content-desc="TopUp"]"
+80.Click Topup,tap,,"//android.view.View[@content-desc="TopUp"]"
+81.Click Hundered,tap,,"//android.view.View[@content-desc="₹ 100.00"]"
+82.Click Proceed,tap,,"//android.widget.Button[@content-desc="Proceed"]"
+83.Wait For Mobile,wait_until_visible,,"//android.widget.EditText"
+84.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+85.Click Netbanking,tap,,"//android.widget.RadioButton[contains(@text,'Netbanking')]"
+86.Click Bob,tap,,"//android.widget.Button[@text="BOB BOB"]"
+87.Wait For Success,wait_until_visible,,"//android.widget.Button[@text="Success"]"
+88.Click Success,tap,,"//android.widget.Button[@text="Success"]"
+89.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
+90.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+91.Click Back,tap,,"//android.view.View[@content-desc="Back"]"</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
35th Commit :Regression Test Suite Updated
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6637192A-677F-4FF9-B1E1-F5C98822756E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6230F09-D273-4861-A963-A545640E533E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -817,7 +817,7 @@
 25.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
 26.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
 27.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-28.Wait For Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+28.wait,3000,,
 29.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
 30.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
 31.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
@@ -880,7 +880,8 @@
 88.Click Success,tap,,"//android.widget.Button[@text="Success"]"
 89.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
 90.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-91.Click Back,tap,,"//android.view.View[@content-desc="Back"]"</t>
+91.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+92.wait,3000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
36th Commit :Tap Cordinate Mobile Action Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6230F09-D273-4861-A963-A545640E533E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7173322F-1D68-4EF4-B364-BE6C38CCFA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId2"/>
     <sheet name="AddAutoDriver" sheetId="32" r:id="rId3"/>
-    <sheet name="TestRun" sheetId="33" r:id="rId4"/>
-    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId5"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId6"/>
+    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId4"/>
+    <sheet name="AddCustomer" sheetId="36" r:id="rId5"/>
+    <sheet name="ApprovedAutoDriver" sheetId="38" r:id="rId6"/>
+    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId7"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="48">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -763,31 +765,6 @@
 22.Load  Super Admin,switch_to,web,
 23.wait,2000,,
 </t>
-  </si>
-  <si>
-    <t>1.wait,2000,,
-2.Load Driver App,switch_to,driver,
-3.wait,2000,,
-4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-14.wait,4000
-15.Load User App,switch_to,user,
-16.wait,2000,,
-17.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-18.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-19.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-20.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-21.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-22.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-23.wait,2000,,</t>
   </si>
   <si>
     <t>1.Load Driver App,switch_to,driver,
@@ -881,7 +858,427 @@
 89.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
 90.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
 91.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-92.wait,3000,,</t>
+92.wait,3000,,
+93.Load User App,switch_to,user,
+94.wait,2000,,
+95.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+96.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+97.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+98.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+99.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+100.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+101.Enter Auto Mobile,type,{randomPhone}&gt;&gt;autoMobile,"//android.widget.EditText"
+102.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+103.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+104.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+105.Wait for Customer Form,wait_until_visible,,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[1]"
+106.Enter Name,type,user{randomAlpha} &gt;&gt; userName,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[1]"
+107.Enter Email,type,user_{timestamp}@gmail.com&gt;&gt;userEmail,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[2]"
+108.Click Agree,tap,,"//android.widget.CheckBox"
+109.wait,2000,,
+110.Click Signup,tap,,"//android.widget.Button[@content-desc="Sign Up"]"
+111.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+112.Click Auto Ride,tap,,"//android.widget.ImageView[@content-desc="Auto Ride"]"
+113..Enter Destination, type, Parsn Manare, "//android.view.View[contains(@content-desc, 'What type of vehicle would you like to book?')]/descendant::android.widget.EditText"
+114.wait,1000,,
+115.Select Destination Option,tap,,"//android.widget.Button[@content-desc="1 m Parsn Manere, Gangai Karai Puram, Anna Salai, Chennai, Tamil Nadu, India Gangai Karai Puram, Anna Salai, Chennai, Tamil Nadu, India"]"
+116.Click Confirm,tap,,"//android.widget.Button[@content-desc="Confirm"]"
+117.Wait for Ride,wait_until_visible,,"//android.widget.Button[@content-desc="Schedule Ride"]"
+118.Click Pink Auto,tap,,"//android.widget.ImageView[@content-desc="Pink Auto 0 Min Away ₹ 70.00"]"
+119.Click Ride Now,tap,,"//android.widget.Button[@content-desc="Ride Now"]"
+120.Load Driver App,switch_to,driver,
+121.wait,2000,,
+122.Click Accept,tap,,"//android.view.View[@content-desc="Accept Accept"]"
+123.wait,3000,,
+124.Load User App,switch_to,user,
+125.wait,2000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLogin</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a Customer.</t>
+  </si>
+  <si>
+    <t>TC_CA_01_add_customer</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
+3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
+4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
+5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
+6.Enter Contact Number, type, {randomPhone}&gt;&gt;userPhone,"//input[@type='tel']"
+7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
+8.Open Gender,click,,"//span[@aria-label='select gender']"
+9.Select Male,click,,"//li[@aria-label='Male']"
+10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
+11.Click Submit, click, , "//button[normalize-space()='Submit']"
+12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+15.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+18.wait,1000,,</t>
+  </si>
+  <si>
+    <t>TC_CA_04_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin,AddCustomer,ApprovedAutoDriver
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+9. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
+14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+26. Click Submit, click, , "//button[contains(.,'Submit')]"
+27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+28. Wait for Toast to hide, wait, 1000,
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+37.Add Driving License,click,,"//i[@title='Edit']"
+38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+48.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@title='Document']"
+51.Click Eye Icon,click,,"//i[@title='View']"
+52.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Driver subscription plan,click,,"//span[normalize-space()='Driver Subscription Plan']"
+4.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
+5.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
+6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+7.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
+8.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
+9.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+10.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
+11.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
+12.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
+13.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
+14.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+15.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+16.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
+17.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
+18.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
+19.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+20.Select On,click,,"//li[@aria-label='on']"
+21.Click Submit ,click,,"//button[normalize-space()='Submit']"
+22.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+23.wait,2000,,
+24.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+25.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+26.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
+27.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
+28.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+29.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+30.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+31.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "//input[@placeholder='Plan Name']"
+32.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+33.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+34.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+35.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+36.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
+37.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+38.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+39.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+40.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+41.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+42.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+43.Select On,click,,"//li[@aria-label='on']"
+44.Click Submit ,click,,"//button[normalize-space()='Submit']"
+45.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+46.wait,3000,,
+47.Load User App,switch_to,user,
+48.wait,2000,,
+49.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+50.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+51.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+52.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+53.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+54.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+55.wait,2000,,
+56.Enter Mobile Number,type,{userPhone},"//android.widget.EditText"
+57.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+58.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+59.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+60.Click Finish,tap,,"//android.widget.Button[@content-desc="Finish"]"
+61.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+62.Profile, tap_coordinate ,978:2224,COORDINATE_MODE
+63.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
+64.wait,5000,,
+65.Load Driver App,switch_to,driver,
+66.wait,2000,,
+67.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+68.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+69.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+70.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+71.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+72.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+73.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+74.Enter Mobile Number,type,{autoPhone},"//android.widget.EditText"
+75.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+76.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+77.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+78.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+79.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+80.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+81.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+82.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+83.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+84.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+85.Drag Page Layout Upward,swipe,up,
+86.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+87.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+88.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+89.wait,3000,,
+90.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+91.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+92.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+93.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+94.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+95.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
+96.wait,5000,,</t>
   </si>
 </sst>
 </file>
@@ -1477,84 +1874,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60E73811-1019-42A7-934A-5E2FAE40D576}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79BE6A4-9FA5-4B28-B734-40C3B7520402}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1609,7 +1928,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>
@@ -1632,7 +1951,233 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AFDAE34-EFC2-4F6C-B8AA-8F3D7C9C3718}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF6BCA45-0614-4137-B63C-BCC5F13F9786}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
38th Commit :Power Tap Implemented To Pass Tests
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83576BE-DB8E-41F7-9603-AD31B4AFB240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F89FA9-B536-4BE2-A320-55E0610CB0EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="52">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -986,9 +986,6 @@
     <t>Validate the end-to-end creation of a Customer.</t>
   </si>
   <si>
-    <t>TC_CA_01_add_customer</t>
-  </si>
-  <si>
     <t>Customer</t>
   </si>
   <si>
@@ -1010,122 +1007,6 @@
 16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
 17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
 18.wait,1000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_04_add_verify_auto_driver</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">SuperAdminLogin,AddCustomer,ApprovedAutoDriver
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
   </si>
   <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -1180,6 +1061,137 @@
 50.Click Doc Icon,click,,"//i[@title='Document']"
 51.Click Eye Icon,click,,"//i[@title='View']"
 52.wait,1000,,</t>
+  </si>
+  <si>
+    <t>TC_CA_04_add_customer</t>
+  </si>
+  <si>
+    <t>SA_TS_5</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_approved_auto_driver</t>
+  </si>
+  <si>
+    <t>SA_TS_7</t>
+  </si>
+  <si>
+    <t>TC_CA_07_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin, AddCustomer and ApprovedAutoDriver test sheets must always be executed prior to running this  test
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin,AddCustomer,ApprovedAutoDriver
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
@@ -1276,7 +1288,7 @@
 93.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
 94.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
 95.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
-96.wait,5000,,</t>
+96.wait,10000,,</t>
   </si>
 </sst>
 </file>
@@ -1992,19 +2004,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>40</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>39</v>
@@ -2067,19 +2079,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>22</v>
@@ -2140,22 +2152,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
39th Commit :Rebooter Modified
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27F89FA9-B536-4BE2-A320-55E0610CB0EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1DC461-CC63-49C6-9AE2-78C1CCFE914E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -740,158 +740,6 @@
       </rPr>
       <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">1.wait,3000,,
-2.Load User App,switch_to,user,
-3.wait,2000,,
-4.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-5.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-11.wait,2000,,
-12.Load Driver App,switch_to,driver,
-13.wait,2000,,
-14.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-15.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-16.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-17.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-18.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-19.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-20.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-21.wait,1000,,
-22.Load  Super Admin,switch_to,web,
-23.wait,2000,,
-</t>
-  </si>
-  <si>
-    <t>1.Load Driver App,switch_to,driver,
-2.Wait For Notification,wait_until_visible,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-3.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-4.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-5.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-6.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-7.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-8.Wait for Mobile Number,wait_until_visible,,"//android.widget.Button[@content-desc="Mobile Number"]"
-9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-10.Wait for Close,wait_until_visible,,"//android.widget.ImageView[@content-desc="Cancel"]"
-11.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-12.Wait for Mobile Number,wait_until_visible,,"//android.widget.EditText"
-13.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-14.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
-15.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-16.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-17.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-18.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-19.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-20.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-21.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-22.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-23.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-24.Drag Page Layout Upward,swipe,up,
-25.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-26.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-27.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-28.wait,3000,,
-29.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-30.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-31.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-32.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-33.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-34.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
-35.Wait For Upload,wait_until_visible,,"//android.widget.Button[@content-desc='Upload']"
-36.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
-37.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
-38.Click Sort,tap,,"//android.widget.TextView[@resource-id="com.google.android.documentsui:id/title" and @text="Sort by..."]"
-39.Click Modified,tap,,"//android.widget.CheckedTextView[@resource-id="android:id/text1" and @text="Modified (newest first)"]"
-40.Click License,tap,,"//android.widget.ImageView[@resource-id="com.google.android.documentsui:id/icon_thumb"]"
-41.Click Crop,tap,,"//android.widget.Button[@content-desc="Crop"]"
-42.Click Calender,tap,,"//android.widget.ImageView[contains(@content-desc, 'Driving Licence')]/android.view.View[2]/android.view.View"
-43.Click Month,tap,"//android.widget.Button[@content-desc="Next month"]"
-44.Click Date,tap,,"//android.widget.Button[contains(@content-desc, '25')]"
-45. Click Ok,tap,,"//android.widget.Button[@content-desc="OK"]"
-46.Click Upload,tap,,"//android.widget.Button[@content-desc="Upload Documents"]"
-47.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
-48.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-49.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-50.Load Admin App,switch_to,web,
-51.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-52.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-53.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-54.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-55.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-56.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-57.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-58.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-59.Click Approve Driver,click,,"//i[@title='Approve']"
-60.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-61.wait,3000,,
-62.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-63.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-64.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-65.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-66.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-67.Load Driver App,switch_to,driver,
-68.Wait For Document,wait_until_visible,,"//android.view.View[@content-desc='Documents']"
-69.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
-70.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
-71.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-72.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-73.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-74.Wait For Offline,wait_until_visible,,"//android.view.View[contains(@content-desc, 'Offline')]"
-75.Click Online,tap_coordinate,989:2045,
-76.wait,2000,,
-77.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-78.Click Wallet,tap,,"//android.view.View[@content-desc="Wallet"]"
-79.Wait For Topup,wait_until_visible,,"//android.view.View[@content-desc="TopUp"]"
-80.Click Topup,tap,,"//android.view.View[@content-desc="TopUp"]"
-81.Click Hundered,tap,,"//android.view.View[@content-desc="₹ 100.00"]"
-82.Click Proceed,tap,,"//android.widget.Button[@content-desc="Proceed"]"
-83.Wait For Mobile,wait_until_visible,,"//android.widget.EditText"
-84.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-85.Click Netbanking,tap,,"//android.widget.RadioButton[contains(@text,'Netbanking')]"
-86.Click Bob,tap,,"//android.widget.Button[@text="BOB BOB"]"
-87.Wait For Success,wait_until_visible,,"//android.widget.Button[@text="Success"]"
-88.Click Success,tap,,"//android.widget.Button[@text="Success"]"
-89.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
-90.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-91.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
-92.wait,3000,,
-93.Load User App,switch_to,user,
-94.wait,2000,,
-95.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-96.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-97.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-98.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-99.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-100.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-101.Enter Auto Mobile,type,{randomPhone}&gt;&gt;autoMobile,"//android.widget.EditText"
-102.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
-103.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-104.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-105.Wait for Customer Form,wait_until_visible,,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[1]"
-106.Enter Name,type,user{randomAlpha} &gt;&gt; userName,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[1]"
-107.Enter Email,type,user_{timestamp}@gmail.com&gt;&gt;userEmail,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[2]"
-108.Click Agree,tap,,"//android.widget.CheckBox"
-109.wait,2000,,
-110.Click Signup,tap,,"//android.widget.Button[@content-desc="Sign Up"]"
-111.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-112.Click Auto Ride,tap,,"//android.widget.ImageView[@content-desc="Auto Ride"]"
-113..Enter Destination, type, Parsn Manare, "//android.view.View[contains(@content-desc, 'What type of vehicle would you like to book?')]/descendant::android.widget.EditText"
-114.wait,1000,,
-115.Select Destination Option,tap,,"//android.widget.Button[@content-desc="1 m Parsn Manere, Gangai Karai Puram, Anna Salai, Chennai, Tamil Nadu, India Gangai Karai Puram, Anna Salai, Chennai, Tamil Nadu, India"]"
-116.Click Confirm,tap,,"//android.widget.Button[@content-desc="Confirm"]"
-117.Wait for Ride,wait_until_visible,,"//android.widget.Button[@content-desc="Schedule Ride"]"
-118.Click Pink Auto,tap,,"//android.widget.ImageView[@content-desc="Pink Auto 0 Min Away ₹ 70.00"]"
-119.Click Ride Now,tap,,"//android.widget.Button[@content-desc="Ride Now"]"
-120.Load Driver App,switch_to,driver,
-121.wait,2000,,
-122.Click Accept,tap,,"//android.view.View[@content-desc="Accept Accept"]"
-123.wait,3000,,
-124.Load User App,switch_to,user,
-125.wait,2000,,</t>
   </si>
   <si>
     <r>
@@ -1289,6 +1137,154 @@
 94.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
 95.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
 96.wait,10000,,</t>
+  </si>
+  <si>
+    <t>1.Load Driver App,switch_to,driver,
+2.Wait For Notification,wait_until_visible,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+3.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+4.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+5.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+7.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+8.Wait for Mobile Number,wait_until_visible,,"//android.widget.Button[@content-desc="Mobile Number"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Wait for Close,wait_until_visible,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+12.Wait for Mobile Number,wait_until_visible,,"//android.widget.EditText"
+13.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+14.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+15.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+16.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+17.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+18.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+19.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+20.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+21.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+22.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+23.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+24.Drag Page Layout Upward,swipe,up,
+25.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+26.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+27.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+28.wait,3000,,
+29.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+30.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+31.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+32.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+33.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+34.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
+35.Wait For Upload,wait_until_visible,,"//android.widget.Button[@content-desc='Upload']"
+36.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
+37.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
+38.Click Sort,tap,,"//android.widget.TextView[@resource-id="com.google.android.documentsui:id/title" and @text="Sort by..."]"
+39.Click Modified,tap,,"//android.widget.CheckedTextView[@resource-id="android:id/text1" and @text="Modified (newest first)"]"
+40.Click License,tap,,"//android.widget.ImageView[@resource-id="com.google.android.documentsui:id/icon_thumb"]"
+41.Click Crop,tap,,"//android.widget.Button[@content-desc="Crop"]"
+42.Click Calender,tap,,"//android.widget.ImageView[contains(@content-desc, 'Driving Licence')]/android.view.View[2]/android.view.View"
+43.Click Month,tap,"//android.widget.Button[@content-desc="Next month"]"
+44.Click Date,tap,,"//android.widget.Button[contains(@content-desc, '25')]"
+45. Click Ok,tap,,"//android.widget.Button[@content-desc="OK"]"
+46.Click Upload,tap,,"//android.widget.Button[@content-desc="Upload Documents"]"
+47.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
+48.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+49.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+50.Load Admin App,switch_to,web,
+51.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+52.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+53.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+54.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+55.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+56.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+57.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+58.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+59.Click Approve Driver,click,,"//i[@title='Approve']"
+60.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+61.wait,3000,,
+62.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+63.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+64.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+65.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+66.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+67.Load Driver App,switch_to,driver,
+68.Wait For Document,wait_until_visible,,"//android.view.View[@content-desc='Documents']"
+69.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
+70.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
+71.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+72.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+73.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+74.Wait For Offline,wait_until_visible,,"//android.view.View[contains(@content-desc, 'Offline')]"
+75.Click Online,tap_coordinate,989:2045,
+76.wait,2000,,
+77.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+78.Click Wallet,tap,,"//android.view.View[@content-desc="Wallet"]"
+79.Wait For Topup,wait_until_visible,,"//android.view.View[@content-desc="TopUp"]"
+80.Click Topup,tap,,"//android.view.View[@content-desc="TopUp"]"
+81.Click Hundered,tap,,"//android.view.View[@content-desc="₹ 100.00"]"
+82.Click Proceed,tap,,"//android.widget.Button[@content-desc="Proceed"]"
+83.Wait For Mobile,wait_until_visible,,"//android.widget.EditText"
+84.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+85.Click Netbanking,tap,,"//android.widget.RadioButton[contains(@text,'Netbanking')]"
+86.Click Bob,tap,,"//android.widget.Button[@text="BOB BOB"]"
+87.Wait For Success,wait_until_visible,,"//android.widget.Button[@text="Success"]"
+88.Click Success,tap,,"//android.widget.Button[@text="Success"]"
+89.Wait For Back,wait_until_visible,,"//android.view.View[@content-desc="Back"]"
+90.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+91.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+92.wait,3000,,
+93.Load User App,switch_to,user,
+94.wait,2000,,
+95.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+96.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+98.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+99.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+100.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+101.Enter Auto Mobile,type,{randomPhone}&gt;&gt;autoMobile,"//android.widget.EditText"
+102.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+103.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+104.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+105.Wait for Customer Form,wait_until_visible,,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[1]"
+106.Enter Name,type,user{randomAlpha} &gt;&gt; userName,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[1]"
+107.Enter Email,type,user_{timestamp}@gmail.com&gt;&gt;userEmail,"//android.widget.ImageView[@content-desc="Get started with I am "]/android.view.View[1]/android.widget.EditText[2]"
+108.Click Agree,tap,,"//android.widget.CheckBox"
+109.wait,2000,,
+110.Click Signup,tap,,"//android.widget.Button[@content-desc="Sign Up"]"
+111.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+112.Click Auto Ride,tap,,"//android.widget.ImageView[@content-desc="Auto Ride"]"
+113..Enter Destination, type, Parsn Manare, "//android.view.View[contains(@content-desc, 'What type of vehicle would you like to book?')]/descendant::android.widget.EditText"
+114.wait,1000,,
+115.Select Destination Option,tap,,"//android.widget.Button[@content-desc="1 m Parsn Manere, Gangai Karai Puram, Anna Salai, Chennai, Tamil Nadu, India Gangai Karai Puram, Anna Salai, Chennai, Tamil Nadu, India"]"
+116.Click Confirm,tap,,"//android.widget.Button[@content-desc="Confirm"]"
+117.Wait for Ride,wait_until_visible,,"//android.widget.Button[@content-desc="Schedule Ride"]"
+118.Click Pink Auto,tap,,"//android.widget.ImageView[@content-desc="Pink Auto 0 Min Away ₹ 70.00"]"
+119.Click Ride Now,tap,,"//android.widget.Button[@content-desc="Ride Now"]"
+120.Load Driver App,switch_to,driver,
+121.wait,2000,,
+122.Click Accept,tap,,"//android.view.View[@content-desc="Accept Accept"]"
+123.wait,3000,,
+124.Load User App,switch_to,user,
+125.wait,5000,,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.wait,3000,,
+2.Load User App,switch_to,user,
+3.wait,2000,,
+4.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+5.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+6.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+7.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+8.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+9.wait,2000,,
+10.Load Driver App,switch_to,driver,
+11.wait,2000,,
+12.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+13.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+14.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+15.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+16.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+17.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+18.wait,1000,,
+19.Load  Super Admin,switch_to,web,
+20.wait,2000,,
+</t>
   </si>
 </sst>
 </file>
@@ -1714,7 +1710,7 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>36</v>
@@ -1938,7 +1934,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>
@@ -2007,19 +2003,19 @@
         <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2079,19 +2075,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>22</v>
@@ -2152,22 +2148,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
44th Commit : Element access with accessibility id implemented for mobile automation
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BCDDE57-385F-4FDC-9E76-765FB7F5716B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BC08C6-E44E-444B-9C8A-CF70BE5A4623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
-    <sheet name="Rebooter" sheetId="34" r:id="rId2"/>
-    <sheet name="AddAutoDriver" sheetId="32" r:id="rId3"/>
-    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId4"/>
-    <sheet name="AddCustomer" sheetId="36" r:id="rId5"/>
-    <sheet name="ApprovedAutoDriver" sheetId="38" r:id="rId6"/>
-    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId7"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId8"/>
+    <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
+    <sheet name="RebooterAccess" sheetId="39" r:id="rId2"/>
+    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId3"/>
+    <sheet name="AddAutoDriver" sheetId="32" r:id="rId4"/>
+    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId5"/>
+    <sheet name="AddCustomer" sheetId="36" r:id="rId6"/>
+    <sheet name="ApprovedAutoDriver" sheetId="38" r:id="rId7"/>
+    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId8"/>
+    <sheet name="SubscriptionPlanAccess" sheetId="40" r:id="rId9"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="61">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -59,9 +61,6 @@
   </si>
   <si>
     <t>SA_TS_2</t>
-  </si>
-  <si>
-    <t>SA_TS_1</t>
   </si>
   <si>
     <t>SA_TS_3</t>
@@ -446,19 +445,7 @@
     </r>
   </si>
   <si>
-    <t>TC_CA_01_super_admin_login</t>
-  </si>
-  <si>
-    <t>TC_CA_02_add_verify_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_04_test_data_cleanup</t>
-  </si>
-  <si>
     <t>Auto Ride Complete Life Cycle Test</t>
-  </si>
-  <si>
-    <t>TC_CA_03_Autoride_Lifecycle_Test</t>
   </si>
   <si>
     <t>This comprehensive end-to-end hybrid test validates the multi-platform orchestration and transactional workflow of the ABCD Framework by simulating a complete ride lifecycle across Web Admin, Driver, and User contexts. The execution flows sequentially from the Web Admin portal to register a new auto driver, switches to the Appium-driven Driver App to submit verification documents, and transitions back to Web Admin for regulatory approval and onboarding. The test then establishes parallel operations, shifting to the Driver App to go online, moving to the User App to dynamically book a ride, routing back to the Driver App to accept and complete the trip, and concludes with payment processing, data lifecycle validation, and transactional integrity verification across all application touchpoints.</t>
@@ -837,13 +824,7 @@
     <t>Customer</t>
   </si>
   <si>
-    <t>TC_CA_04_add_customer</t>
-  </si>
-  <si>
     <t>SA_TS_5</t>
-  </si>
-  <si>
-    <t>TC_CA_05_add_approved_auto_driver</t>
   </si>
   <si>
     <t>SA_TS_7</t>
@@ -1238,13 +1219,71 @@
 19.wait,1000,,</t>
   </si>
   <si>
+    <t>SA_TS_01</t>
+  </si>
+  <si>
+    <t>Rebooter Access Test</t>
+  </si>
+  <si>
+    <t>TC_CA_01_Reboot_Access_Test</t>
+  </si>
+  <si>
+    <t>If in case emulators crashes wipe data and  cold reboot all emulators and run this test to make the emultators and web browser into initial state before running other tests.This test uses access id instead of xpath for mobile testing.</t>
+  </si>
+  <si>
+    <t>TC_CA_02_super_admin_login</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_04_Autoride_Lifecycle_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_customer</t>
+  </si>
+  <si>
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_approved_auto_driver</t>
+  </si>
+  <si>
+    <t>SA_TS_8</t>
+  </si>
+  <si>
+    <t>TC_CA_08_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>1.wait,3000,,
+2.Load User App,switch_to,user,
+3.wait,2000,,
+4.Click Get Started,tap,,"accessibility=Get Started"
+5.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+6.Click Next,tap,,"accessibility=Next"
+7.Click Mobile Number,tap,,"accessibility=Mobile Number"
+8.Click Close,tap,,"accessibility=Cancel"
+9.wait,2000,,
+10.Load Driver App,switch_to,driver,
+11.wait,2000,,
+12.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+13.Click Agree,tap,,"accessibility=Agree"
+14.Click Get Started,tap,,"accessibility=Get Started"
+15.Click Next,tap,,"accessibility=Next"
+16.Click Mobile Number,tap,,"accessibility=Mobile Number"
+17.Click Close,tap,,"accessibility=Cancel"
+18.wait,1000,,
+19.Load  Super Admin,switch_to,web,
+20.wait,2000,,</t>
+  </si>
+  <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
 4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
 5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.wait,5000,,
-7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox//input[@type='checkbox']"
+6.wait,3000,,
+7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
 8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
 9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
 10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
@@ -1252,49 +1291,152 @@
 12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
 13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
 14.Select Source,click,,"//span[@aria-label='Select Source']"
-15.Select Instagram,click,,"//span[normalize-space()='From Instagramj']"
+15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
 16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
 17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
 18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
 19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-20.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-24. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-25. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-26. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-27.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-28.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-29. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-30. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-31. Click Submit, click, , "//button[contains(.,'Submit')]"
-32. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-33. Wait for Toast to hide, wait, 1000,
-34.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-36.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-37.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-38.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-39.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-40. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-41.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-42.Add Driving License,click,,"//i[@title='Edit']"
-43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-45.Click Submit, click, , "//button[normalize-space()='Submit']"
+20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 1000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+38. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+40.Add Driving License,click,,"//i[@title='Edit']"
+41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+43.Click Submit, click, , "//button[normalize-space()='Submit']"
+44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+45.Click Approve Driver,click,,"//i[@title='Approve']"
 46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-47.Click Approve Driver,click,,"//i[@title='Approve']"
-48.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-49.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-50.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-51.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-52.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-53.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-54.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-55.Click Doc Icon,click,,"//i[@title='Document']"
-56.Click Eye Icon,click,,"//i[@title='View']"
-57.wait,1000,,</t>
+47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+52.Scroll Grid, tab, 10, "//input[@aria-label='Driver Name Filter Input']"
+53.Click Doc Icon,click,,"//i[@title='Document']"
+54.Click Eye Icon,click,,"//i[@title='View']"
+55.wait,1000,,</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Subscription_Plan_Access_Test</t>
+  </si>
+  <si>
+    <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.This test case uses accessibility id instead of xpath for mobile automation</t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+4.Click Driver subscription plan,click,,"//span[normalize-space()='Driver Subscription Plan']"
+5.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
+6.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
+7.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+8.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
+9.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
+10.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+11.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
+12.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
+13.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
+14.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
+15.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+16.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+17.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
+18.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
+19.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
+20.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+21.Select On,click,,"//li[@aria-label='on']"
+22.Click Submit ,click,,"//button[normalize-space()='Submit']"
+23.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+24.wait,2000,,
+25.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+26.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+27.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
+28.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
+29.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+30.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+31.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+32.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "//input[@placeholder='Plan Name']"
+33.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+34.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+35.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+36.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+37.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
+38.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+39.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+40.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+41.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+42.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+43.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+44.Select On,click,,"//li[@aria-label='on']"
+45.Click Submit ,click,,"//button[normalize-space()='Submit']"
+46.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+47.wait,3000,,
+48.Load User App,switch_to,user,
+49.wait,2000,,
+50.Click Get Started,tap,,"accessibility=Get Started"
+51.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+52.Click Next,tap,,"accessibility=Next"
+53.Click Mobile Number,tap,,"accessibility=Mobile Number"
+54.Click Close,tap,,"accessibility=Cancel"
+55.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+56.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+57.Click Continue,tap,,"accessibility=Continue"
+58.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+59.Click Finish,tap,,"accessibility=Finish"
+60.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+61.Profile, tap_coordinate ,978:2224,COORDINATE_MODE
+62.Click Subscription,tap,,"accessibility=Subscription"
+63.Wait Customer Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{customerSubscriptionName}")"
+64.Click Customer Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{customerSubscriptionName}")"
+65.wait,3000,,
+66.Load Driver App,switch_to,driver,
+67.wait,2000,,
+68.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+69.Click Agree,tap,,"accessibility=Agree"
+70.Click Get Started,tap,,"accessibility=Get Started"
+71.Click Next,tap,,"accessibility=Next"
+72.Click Mobile Number,tap,,"accessibility=Mobile Number"
+73.Click Close,tap,,"accessibility=Cancel"
+74.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+75.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+76.Click Continue,tap,,"accessibility=Continue"
+77.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+78.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+79.wait,3000,,
+80.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+81.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+82.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+83.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+84.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+85.Drag Page Layout Upward,swipe,up,
+86.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+87.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+88.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+89.wait,3000,,
+90.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+91.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+92.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+93.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+94.Click Subscription,tap,,"accessibility=Subscription"
+95.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
+96.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
+97.wait,5000,,</t>
   </si>
 </sst>
 </file>
@@ -1666,6 +1808,232 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5AE23A-69EB-46F0-86E8-8B9CD1BA86DE}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="57.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="7"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74DE6E4A-8100-4C1D-8A58-4E86A951B80B}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="57.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F96D9-3311-4A18-82B5-F5729925CB8A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1708,22 +2076,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1741,83 +2109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5AE23A-69EB-46F0-86E8-8B9CD1BA86DE}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="57.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC812CD8-667D-4888-8684-24E9CC12973D}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1859,22 +2151,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1889,7 +2181,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79BE6A4-9FA5-4B28-B734-40C3B7520402}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1935,19 +2227,19 @@
         <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1956,7 +2248,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1967,7 +2259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AFDAE34-EFC2-4F6C-B8AA-8F3D7C9C3718}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2010,22 +2302,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2043,7 +2335,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2085,22 +2377,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2115,7 +2407,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF6BCA45-0614-4137-B63C-BCC5F13F9786}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2158,22 +2450,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2182,7 +2474,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -2193,25 +2485,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5DCFAC-B912-41EA-9964-A3839A72D798}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -2233,36 +2526,39 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>25</v>
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+      <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
48th Commit : Auto Ride Booking Test Suite Completed
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B16D4C8-EA99-4011-9670-54DA1FA9F90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4414F07B-C8B7-49AB-822A-C16A3E0811A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1656,8 +1656,8 @@
 86.wait,2000,,
 87.Click Auto Ride,tap,,"accessibility=Auto Ride"
 88.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
-89.wait,3000,,
-90.Select Destination, tap ,, "automator=new UiSelector().description("0.1 km Parsn Manere, Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu")"
+89.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
+90.Select Destination,tap_coordinate,545:1299,
 91.Click Confirm,tap,,"accessibility=Confirm"
 92.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
 93.Ride Now,tap,,"accessibility=Ride Now"
@@ -1666,7 +1666,27 @@
 96.wait,2000,,
 97.Wait for Accept,wait_until_visible,,"automator=new UiSelector().description("Accept Accept")"
 98.Accept Ride,tap,,"automator=new UiSelector().description("Accept Accept")"
-99.wait,2000,,</t>
+99.wait,2000,,
+100.Ride Arrived,tap,,"accessibility=Arrived"
+101.Yes Arrived,tap,,"accessibility=Yes"
+102.Start Ride,tap,,"accessibility=Start Ride"
+103.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+104.Start Ride,tap,,"accessibility=Start"
+105.Complete Ride,tap,,"accessibility=Complete Ride"
+106.Collect Payment,tap,,"accessibility=Collect Payment"
+107.Confirm Payment,tap,,"accessibility=Yes"
+108.Give Rating,tap_coordinate,444:1642,
+109.Submit Rating,tap,,"accessibility=Submit"
+110.wait,3000,,
+111.Load User App,switch_to,user,
+112.wait,2000,,
+113.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+114.Pay Cash,tap,,"accessibility=Proceed To Pay"
+115.Give Review,tap,,"accessibility=Give Review"
+116.Give Rating,tap_coordinate,444:1642,
+117.Submit Rating,tap,,"accessibility=Submit"
+118.Trip Finished,tap,,"accessibility=Done"
+119.wait,3000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
50th Commit : Auto Ride Booking Test Suite Updated with Wait Visible
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7906DE6D-3D1C-44C1-81B6-7D72D2872048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C4FE79-6653-4227-948C-53F6EDA1D7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1581,7 +1581,7 @@
 11.Click Continue,tap,,"accessibility=Continue"
 12.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
 13.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-14.wait,3000,,
+14.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 15.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 16.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
 17.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
@@ -1591,102 +1591,110 @@
 21.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
 22.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
 23.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-24.wait,3000,,
+24.Wait for Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
 25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
 26.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
 27.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
 28.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-29.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+29.Click Hamburger,tap_coordinate ,75:209,COORDINATE_MODE
 30.Click Document,tap,,"accessibility=Documents"
-31.Click Upload,tap,,"accessibility=Upload"
-32.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
-33.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
-34.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
-35.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
-36.Click Crop,tap,,"accessibility=Crop"
-37.Click Calender,tap_coordinate ,123:1627,COORDINATE_MODE
-38..Click Month,tap,"accessibility=Next month"
-39.Click Date,tap_coordinate ,922:1381,COORDINATE_MODE
-40.Click Ok,tap,,"accessibility=OK"
-41.Click Upload,tap,,"accessibility=Upload Documents"
-42.Wait For Back,wait_until_visible,,"accessibility=Back"
-43.Click Back,tap,,"accessibility=Back"
+31.Wait For Upload,wait_until_visible,,"accessibility=Upload"
+32.Click Upload,tap,,"accessibility=Upload"
+33.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
+34.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
+35.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+36.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+37.Click Crop,tap,,"accessibility=Crop"
+38.Click Calender,tap_coordinate ,123:1627,COORDINATE_MODE
+39.Click Month,tap,"accessibility=Next month"
+40.Click Date,tap_coordinate ,922:1381,COORDINATE_MODE
+41.Click Ok,tap,,"accessibility=OK"
+42.Click Upload,tap,,"accessibility=Upload Documents"
+43.Wait For Back,wait_until_visible,,"accessibility=Back"
 44.Click Back,tap,,"accessibility=Back"
-45.Load Admin App,switch_to,web,
-46.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-48.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-49.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-50.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-51.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-52.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-53.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-54.Click Approve Driver,click,,"//i[@title='Approve']"
-55.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-56.wait,3000,,
-57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+45.Click Back,tap,,"accessibility=Back"
+46.Load Admin App,switch_to,web,
+47.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+50.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+51.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+52.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+53.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+54.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+55.Click Approve Driver,click,,"//i[@title='Approve']"
+56.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+57.wait,2000,,
 58.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-59.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-60.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-61.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-62.wait,2000,,
+59.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+60.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+61.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+62.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
 63.Load Driver App,switch_to,driver,
-64.wait,2000,,
-65.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-66.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-67.Click Document,tap,,"accessibility=Documents"
-68.Wait For Back,wait_until_visible,,"accessibility=Back"
+64.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+65.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+66.Click Document,tap,,"accessibility=Documents"
+67.Wait For Back,wait_until_visible,,"accessibility=Back"
+68.Click Back,tap,,"accessibility=Back"
 69.Click Back,tap,,"accessibility=Back"
-70.Click Back,tap,,"accessibility=Back"
-71.Click Online,tap_coordinate,989:2045,
-72.wait,3000,,
-73.Load User App,switch_to,user,
-74.wait,2000,,
-75.Click Get Started,tap,,"accessibility=Get Started"
-76.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-77.Click Next,tap,,"accessibility=Next"
-78.Click Mobile Number,tap,,"accessibility=Mobile Number"
-79.Click Close,tap,,"accessibility=Cancel"
-80.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
-81.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-82.Click Continue,tap,,"accessibility=Continue"
-83.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-84.Click Finish,tap,,"accessibility=Finish"
-85.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-86.wait,2000,,
-87.Click Auto Ride,tap,,"accessibility=Auto Ride"
-88.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
-89.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
-90.Select Destination,tap_coordinate,545:1299,
-91.Click Confirm,tap,,"accessibility=Confirm"
-92.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
-93.Ride Now,tap,,"accessibility=Ride Now"
-94.wait,2000,,
-95.Load Driver App,switch_to,driver,
-96.wait,2000,,
-97.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
-98.Accept Ride,tap,,"automator=new UiSelector().description("Accept Accept")"
-99.wait,2000,,
-100.Ride Arrived,tap,,"accessibility=Arrived"
-101.Yes Arrived,tap,,"accessibility=Yes"
+70.Click Online,tap_coordinate,989:2045,
+71.wait,2000,,
+72.Load User App,switch_to,user,
+73.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
+74.Click Get Started,tap,,"accessibility=Get Started"
+75.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+76.Click Next,tap,,"accessibility=Next"
+77.Click Mobile Number,tap,,"accessibility=Mobile Number"
+78.Click Close,tap,,"accessibility=Cancel"
+79.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+80.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+81.Click Continue,tap,,"accessibility=Continue"
+82.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+83.Click Finish,tap,,"accessibility=Finish"
+84.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+85.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
+86.Click Auto Ride,tap,,"accessibility=Auto Ride"
+87.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
+88.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
+89.Select Destination,tap_coordinate,545:1299,
+90.Click Confirm,tap,,"accessibility=Confirm"
+91.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+92.Ride Now,tap,,"accessibility=Ride Now"
+93.wait,2000,,
+94.Load Driver App,switch_to,driver,
+95.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
+96.Accept Ride,tap_coordinate,784:2224,
+97.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
+98.Ride Arrived,tap,,"accessibility=Arrived"
+99.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+100.Yes Arrived,tap,,"accessibility=Yes"
+101.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
 102.Start Ride,tap,,"accessibility=Start Ride"
-103.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
-104.Start Ride,tap,,"accessibility=Start"
-105.Complete Ride,tap,,"accessibility=Complete Ride"
-106.Collect Payment,tap,,"accessibility=Collect Payment"
-107.Confirm Payment,tap,,"accessibility=Yes"
-108.Give Rating,tap_coordinate,444:1642,
-109.Submit Rating,tap,,"accessibility=Submit"
-110.wait,3000,,
-111.Load User App,switch_to,user,
-112.wait,2000,,
-113.Proceed Payment,tap,,"accessibility=Proceed To Pay"
-114.Pay Cash,tap,,"accessibility=Proceed To Pay"
-115.Give Review,tap,,"accessibility=Give Review"
-116.Give Rating,tap_coordinate,444:1642,
-117.Submit Rating,tap,,"accessibility=Submit"
-118.Trip Finished,tap,,"accessibility=Done"
-119.wait,3000,,</t>
+103.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
+104.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+105.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
+106.Start Ride,tap,,"accessibility=Start"
+107.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
+108.Complete Ride,tap,,"accessibility=Complete Ride"
+109.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
+110.Collect Payment,tap,,"accessibility=Collect Payment"
+111.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+112.Confirm Payment,tap,,"accessibility=Yes"
+113.wait,2000,,
+114.Give Rating,tap_coordinate,444:1642,
+115.Submit Rating,tap,,"accessibility=Submit"
+116.Load User App,switch_to,user,
+117.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
+118.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+119.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
+120.Pay Cash,tap,,"accessibility=Proceed To Pay"
+121.Wait for Review,wait_until_visible,,"accessibility=Give Review"
+122.Give Review,tap,,"accessibility=Give Review"
+123.wait,2000,,
+124.Give Rating,tap_coordinate,444:1642,
+125.Submit Rating,tap,,"accessibility=Submit"
+126.Wait for Done,wait_until_visible,,"accessibility=Done"
+127.Trip Finished,tap,,"accessibility=Done"</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
57th Commit : Auto Ride Test Suite Without Wallet Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47539FC-5333-44AF-92CC-212E49C09453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318B228C-283F-4921-8EB5-12253E9A8591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -21,9 +21,10 @@
     <sheet name="AddCustomer" sheetId="36" r:id="rId6"/>
     <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId7"/>
     <sheet name="AutoRideAccessTest" sheetId="41" r:id="rId8"/>
-    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId9"/>
-    <sheet name="SubscriptionPlanAccess" sheetId="40" r:id="rId10"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
+    <sheet name="AutoRideWithoutWallet" sheetId="42" r:id="rId9"/>
+    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId10"/>
+    <sheet name="SubscriptionPlanAccess" sheetId="40" r:id="rId11"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="70">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1177,9 +1178,6 @@
     <t>TC_CA_03_add_verify_auto_driver</t>
   </si>
   <si>
-    <t>TC_CA_04_Autoride_Lifecycle_Test</t>
-  </si>
-  <si>
     <t>SA_TS_6</t>
   </si>
   <si>
@@ -1189,28 +1187,10 @@
     <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.This test case uses accessibility id instead of xpath for mobile automation</t>
   </si>
   <si>
-    <t>TC_CA_05_Autoride_Access_Test</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_customer</t>
-  </si>
-  <si>
-    <t>TC_CA_07_add_approved_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_08_Subscription_Plan_Test</t>
-  </si>
-  <si>
     <t>SA_TS_9</t>
   </si>
   <si>
-    <t>TC_CA_09_Subscription_Plan_Access_Test</t>
-  </si>
-  <si>
     <t>SA_TS_10</t>
-  </si>
-  <si>
-    <t>TC_CA_10_test_data_cleanup</t>
   </si>
   <si>
     <r>
@@ -1697,6 +1677,166 @@
 141.Submit Rating,tap,,"accessibility=Submit"
 141.Wait for Done,wait_until_visible,,"accessibility=Done"
 142.Trip Finished,tap,,"accessibility=Done"</t>
+  </si>
+  <si>
+    <t>Auto Ride Complete Life Cycle Test Without Wallet</t>
+  </si>
+  <si>
+    <t>TC_CA_04_add_approved_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_05_add_customer</t>
+  </si>
+  <si>
+    <t>TC_CA_06_Autoride_Lifecycle_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_07_Autoride_Access_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Autoride_Access_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_10_Subscription_Plan_Access_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_11</t>
+  </si>
+  <si>
+    <t>TC_CA_11_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>1.Load Driver App,switch_to,driver,
+2.Wait For Notification,wait_until_visible,,"id=com.android.permissioncontroller:id/permission_allow_button"
+3.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+4.Click Agree,tap,,"accessibility=Agree"
+5.Click Get Started,tap,,"accessibility=Get Started"
+6.Click Next,tap,,"accessibility=Next"
+7.Click Mobile Number,tap,,"accessibility=Mobile Number"
+8.Click Close,tap,,"accessibility=Cancel"
+9.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+10.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+11.Click Continue,tap,,"accessibility=Continue"
+12.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+13.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+14.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+15.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+16.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+17.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+18.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+19.Drag Page Layout Upward,swipe,up,
+20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+21.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+22.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+23.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+24.Wait for Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+26.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+27.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+28.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+29.Click Hamburger,tap_coordinate ,75:209,COORDINATE_MODE
+30.Click Document,tap,,"accessibility=Documents"
+31.Wait For Document Page,wait_until_visible,,"accessibility=Add Documents"
+32.Wait For Upload,wait_until_visible,,"accessibility=Upload"
+33.Click Upload,tap,,"accessibility=Upload"
+34.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
+35.Wait For Sort,wait_until_visible,,"automator=new UiSelector().resourceId("com.google.android.documentsui:id/content").instance(0)"
+36.Click Sort,tap,,"automator=new UiSelector().resourceId("com.google.android.documentsui:id/content").instance(0)"
+37.Wait For Modified,wait_until_visible,,"automator=new UiSelector().text("Modified (newest first)")"
+38.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+39.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+40.Wait For Crop,wait_until_visible,,"accessibility=Crop"
+41.Click Crop,tap,,"accessibility=Crop"
+42.Wait For  Add Document,wait_until_visible,,"accessibility=Add Documents"
+43.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
+44.Click Month,tap,"accessibility=Next month"
+45.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
+46.Click Ok,tap,,"accessibility=OK"
+47.Click Upload,tap,,"accessibility=Upload Documents"
+48.Wait For Back,wait_until_visible,,"accessibility=Back"
+49.Click Back,tap,,"accessibility=Back"
+50.Load Admin App,switch_to,web,
+51.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+52.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+53.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+54.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+55.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+56.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+57.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+58.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+59.Click Approve Driver,click,,"//i[@title='Approve']"
+60.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+61.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+62.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+63.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+64.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+65.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+66.Load Driver App,switch_to,driver,
+67.Wait For Back,wait_until_visible,,"accessibility=Back"
+68.Click Document,tap,,"accessibility=Documents"
+69.Wait For Add Document,wait_until_visible,,"accessibility=Add Documents"
+70.Click Back,tap,,"accessibility=Back"
+71.Wait For Documents,wait_until_visible,,"accessibility=Documents"
+72.Click Back,tap,,"accessibility=Back"
+73.Click Online,tap_coordinate,986:1936,
+74.Load User App,switch_to,user,
+75.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
+76.Click Get Started,tap,,"accessibility=Get Started"
+77.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+78.Click Next,tap,,"accessibility=Next"
+79.Click Mobile Number,tap,,"accessibility=Mobile Number"
+80.Click Close,tap,,"accessibility=Cancel"
+81.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+82.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+83.Click Continue,tap,,"accessibility=Continue"
+84.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+85.Wait for Finish,wait_until_visible,,"accessibility=Finish"
+86.Click Finish,tap,,"accessibility=Finish"
+87.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+88.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
+89.Click Auto Ride,tap,,"accessibility=Auto Ride"
+90.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
+91.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
+92.Select Destination,tap_coordinate,545:1299,
+93.Click Confirm,tap,,"accessibility=Confirm"
+94.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+95.Ride Now,tap,,"accessibility=Ride Now"
+96.Load Driver App,switch_to,driver,
+97.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
+98.Accept Ride,tap_coordinate,801:2113,
+99.Wait for On My Way,wait_until_visible,,"accessibility=On My Way to Pickup"
+100.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
+101.Ride Arrived,tap,,"accessibility=Arrived"
+102.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+103.Yes Arrived,tap,,"accessibility=Yes"
+104.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
+105.Start Ride,tap,,"accessibility=Start Ride"
+106.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
+107.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+108.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
+109.Start Ride,tap,,"accessibility=Start"
+110.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
+111.Complete Ride,tap,,"accessibility=Complete Ride"
+112.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
+113.Collect Payment,tap,,"accessibility=Collect Payment"
+114.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+115.Confirm Payment,tap,,"accessibility=Yes"
+116.Give Rating,tap_coordinate,348:1545,
+117.Submit Rating,tap,,"accessibility=Submit"
+118.Load User App,switch_to,user,
+119.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
+120.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+121.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
+122.Pay Cash,tap,,"accessibility=Proceed To Pay"
+123.Wait for Review,wait_until_visible,,"accessibility=Give Review"
+124.Give Review,tap,,"accessibility=Give Review"
+125.Give Rating,tap_coordinate,348:1619,
+126.Submit Rating,tap,,"accessibility=Submit"
+127.Wait for Done,wait_until_visible,,"accessibility=Done"
+128.Trip Finished,tap,,"accessibility=Done"</t>
   </si>
 </sst>
 </file>
@@ -2144,6 +2284,84 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF6BCA45-0614-4137-B63C-BCC5F13F9786}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5DCFAC-B912-41EA-9964-A3839A72D798}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2186,19 +2404,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -2221,7 +2439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2263,13 +2481,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
@@ -2350,7 +2568,7 @@
         <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>30</v>
@@ -2501,7 +2719,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2561,19 +2779,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2634,19 +2852,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>31</v>
@@ -2710,13 +2928,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -2788,22 +3006,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2824,7 +3042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF6BCA45-0614-4137-B63C-BCC5F13F9786}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{433E6E83-0B1D-4096-828C-01F3E8739F33}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2866,22 +3084,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
58th Commit : Locators.properties Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318B228C-283F-4921-8EB5-12253E9A8591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4886925-A023-476B-9741-74C199DB1B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -25,6 +25,10 @@
     <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId10"/>
     <sheet name="SubscriptionPlanAccess" sheetId="40" r:id="rId11"/>
     <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId12"/>
+    <sheet name="SuperAdminLocator" sheetId="43" r:id="rId13"/>
+    <sheet name="AddCustomerLocator" sheetId="44" r:id="rId14"/>
+    <sheet name="AddAutoDriverLocator" sheetId="46" r:id="rId15"/>
+    <sheet name="AutoRideWithoutWalletLocator" sheetId="47" r:id="rId16"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="90">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1837,6 +1841,532 @@
 126.Submit Rating,tap,,"accessibility=Submit"
 127.Wait for Done,wait_until_visible,,"accessibility=Done"
 128.Trip Finished,tap,,"accessibility=Done"</t>
+  </si>
+  <si>
+    <t>1. Enter  Email , type , super_admin@gmail.com, "admin.login.email"
+2. Enter Password,type,R1mep@321, "admin.login.password"
+3. Click Login,click,,"admin.login.submit_btn"
+4. Verify Dashboard,verify,,"admin.dashboard.statistics_header"</t>
+  </si>
+  <si>
+    <t>Super Admin Locator</t>
+  </si>
+  <si>
+    <t>Verify successful authentication of the Super Admin role using valid credentials and Dashboard access validation using Locators</t>
+  </si>
+  <si>
+    <t>SA_TS_12</t>
+  </si>
+  <si>
+    <t>TC_CA_12_super_admin_locator</t>
+  </si>
+  <si>
+    <t>SA_TS_13</t>
+  </si>
+  <si>
+    <t>Customer Locator</t>
+  </si>
+  <si>
+    <t>TC_CA_13_add_customer_Locator</t>
+  </si>
+  <si>
+    <t>Validate the end-to-end creation of a Customer Using Locator</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLocator</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page for this configure dashboard.url as https://dev.we1.co/#/page-module/dashboard_dynamic in config.properties.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Click Dashboard  Icon,click,,"admin.menu.dashboard"
+2. Click Customer  Icon,click,,"admin.menu.customer_icon"
+3.Click  Add Customers,click,,"admin.menu.add_customers"
+4. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
+5.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "admin.customer.input_name"
+6.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "admin.customer.input_email"
+7.Enter Contact Number, type, {randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
+8.Enter Video Call Limit, type, 60, "admin.customer.input_video_limit"
+9.Open Gender,click,,"admin.customer.dropdown_gender"
+10.Select Male,click,,"admin.customer.select_gender_male"
+11.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "admin.customer.upload_profile_img"
+12.Click Submit, click, , "admin.customer.submit_btn"
+13.Verify Added Succesfully, verify, , "admin.customer.toast_info"
+14. Click Customer  Icon,click,,"admin.menu.customer_icon"
+15. Click Customer  Icon,click,,"admin.menu.customer_icon"
+16.Click  Verified Customers,click,,"admin.menu.verified_customers"
+17. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading "
+18.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin test suite must be always executed before this test.This ensures the browser is already logged in as a Super Admin. Without this step, the automation will encounter a "Redirect to Login" or "Access Denied" error. The framework is configured to automatically handle this login for you if it hasn't been done yet.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> SuperAdminLocator
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: The user is already authenticated as an Admin/Super Admin with active session permissions for Driver and Document Management.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Navigation State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The browser must be on the Dashboard page (https://dev.we1.co/#/page-module/dashboard_dynamic). The dashboard.url must be correctly mapped in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>SA_TS_14</t>
+  </si>
+  <si>
+    <t>TC_CA_14_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SuperAdminLocator,AddCustomerLocator,AddAutoDriverLocator</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Click drivers menu, click, , "admin.drivers.menu.icon"
+2.Click Add Driver menu, click, ,"admin.drivers.add_menu.link"
+3.Verify Add Driver page, verify, , "admin.drivers.add_page.header"
+4.Click Service Category Dropdown, click, , "admin.drivers.service_dropdown.select"
+5.Select Auto Ride Option, click, , "admin.drivers.autoride_option.span"
+6.Select Auto Ride Option, click, ,"admin.drivers.autoride_option.span"
+7.Wait for Auto Ride Checkbox, wait_until_visible, , "admin.drivers.autoride.checkbox"
+8.Click Auto Ride Checkbox, click, , "admin.drivers.autoride.checkbox"
+9.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+10.Enter Email, type, autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail, "admin.drivers.email.input"
+11.Enter Contact Number, type, {randomPhone} &gt;&gt; autoPhone, "admin.drivers.phone.input"
+12.Click Whatsapp Checkbox, click, , "admin.drivers.whatsapp.checkbox"
+13.Enter Whatsapp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+15.Click Select Source Dropdown, click, ,"admin.drivers.source_dropdown.select"
+16.Select From Instagram Option, click, , "admin.drivers.instagram_option.span"
+17.Select Male Gender, click, ," admin.drivers.male_gender.div"
+18.Click Vehicle Type Dropdown, click, ,"admin.drivers.vehicle_dropdown.select"
+19.Select Pink Auto Option, click, ," admin.drivers.pink_auto_option.span"
+20.Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+21.Enter Plate No, type, KL-01-AB-1234,"admin.drivers.plateno.input"
+22.Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+24.Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+25.Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
+26.Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+27.Enter Account Holder Name, type, {autoName}, "admin.drivers.accountholder.input"
+28.Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+29.Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+30.Click Submit Button, click, , "admin.drivers.submit.button"
+31.Verify Driver Added Successfully, verify, , "admin.drivers.success_toast.div"
+32.Wait for Toast to Hide, wait, 1000, 
+33.Click drivers menu to refresh, click, , "admin.drivers.menu.icon"
+34.Click drivers menu to refresh, click, , "admin.drivers.menu.icon"
+35.Click Pending Documents Menu, click, , "admin.drivers.pending_docs.link"
+36.Filter Pending Docs by Name, type, {autoName}, "admin.drivers.name_filter.input"
+37.Click Dashboard Home Icon, click, , "admin.drivers.dashboard.icon"</t>
+  </si>
+  <si>
+    <t>SA_TS_15</t>
+  </si>
+  <si>
+    <t>1. Load Driver App, switch_to, driver, 
+2. Wait For Notification, wait_until_visible, , "mobile.driver.permission_allow.btn"
+3. Click Allow Notification, tap, , "mobile.driver.permission_allow.btn"
+4. Click Agree, tap, , "mobile.driver.agree.btn"
+5. Click Get Started, tap, , "mobile.driver.get_started.btn"
+6. Click Next, tap, ," mobile.driver.next.btn"
+7. Click Mobile Number, tap, , "mobile.driver.mobile_number_field.btn"
+8. Click Close, tap, , "mobile.driver.cancel.btn"
+9. Enter Mobile Number, type, {autoPhone}, "mobile.driver.edit_text.input"
+10. Wait for Continue, wait_until_visible, ,"mobile.driver.continue.btn"
+11. Click Continue, tap, ,"mobile.driver.continue.btn"
+12. Enter OTP, type, 123456, "mobile.driver.edit_text.input"
+13. Click Allow Location, tap, , "mobile.driver.location_allow.btn"
+14. Wait For Popup, wait_until_visible, , "mobile.driver.independent_contractor.checkbox"
+15. Click Independent Contractor, tap, , "mobile.driver.independent_contractor.checkbox"
+16. Click Legal Document, tap, , "mobile.driver.legal_document.checkbox"
+17. Click Safety Conduct, tap, ,"mobile.driver.safety_conduct.checkbox"
+18. Click Subscription Model, tap, , "mobile.driver.subscription_model.checkbox"
+19. Drag Page Layout Upward, swipe, up, 
+20. Click Liability, tap, , "mobile.driver.liability.checkbox"
+21. Click Data Protection, tap, , "mobile.driver.data_protection.checkbox"
+22. Click Fitness Declaration, tap, , "mobile.driver.fitness_declaration.checkbox"
+23. Click Confirmation, tap, , "mobile.driver.confirmation.checkbox"
+24. Wait for Agree, wait_until_visible, ,"mobile.driver.agree_continue.btn"
+25. Click Agree, tap, , "mobile.driver.agree_continue.btn"
+26. Wait For OTP, wait_until_visible, , "mobile.driver.edit_text.input"
+27. Enter OTP, type, 123456,"mobile.driver.edit_text.input"
+28. Wait For Driver App, wait_until_visible, , "mobile.driver.app_header.label"
+29. Click Hamburger, tap_coordinate, 75:209, COORDINATE_MODE
+30. Click Document, tap, , "mobile.driver.documents.menu"
+31. Wait For Document Page, wait_until_visible, , "mobile.driver.add_documents.header"
+32. Wait For Upload, wait_until_visible, ," mobile.driver.upload.btn"
+33. Click Upload, tap, ,"mobile.driver.upload.btn"
+34. Upload License, uploadfile, "src/main/resources/test-data/license.JPG", "mobile.driver.upload_docs.btn"
+35. Wait For Sort, wait_until_visible, ," mobile.driver.android_content.view"
+36. Click Sort, tap, , "mobile.driver.android_content.view"
+37. Wait For Modified, wait_until_visible, , "mobile.driver.sort_modified.btn"
+38. Click Modified, tap, ,"mobile.driver.sort_modified.btn"
+39. Click License, tap, , "mobile.driver.license_thumb.icon"
+40. Wait For Crop, wait_until_visible, ,"mobile.driver.crop.btn"
+41. Click Crop, tap, , "mobile.driver.crop.btn"
+42. Wait For Add Document, wait_until_visible, ,"mobile.driver.add_documents.header"
+43. Click Calendar, tap_coordinate, 121:1539, COORDINATE_MODE
+44. Click Month, tap, ,"mobile.driver.next_month.btn"
+45. Click Date, tap_coordinate, 943:1290, COORDINATE_MODE
+46. Click Ok, tap, , "mobile.driver.ok.btn"
+47. Click Upload Submission, tap, , "mobile.driver.upload_docs.btn"
+48. Wait For Back, wait_until_visible, , "mobile.driver.back.btn"
+49. Click Back, tap, , "mobile.driver.back.btn"
+50.Load Admin App,switch_to,web,
+51.Wait For Driver Menu,wait_until_visible,,"admin.drivers.menu.icon"
+52.Click drivers menu,click,,"admin.drivers.menu.icon"
+53.Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+54.Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+55.Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+56.Click Doc Icon,click,,"admin.drivers.docs.icon"
+57.Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+58.FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+59.Click Approve Driver,click,,"admin.drivers.docs.approval"
+60.Verify Updated Succesfully, verify, , "admin.drivers.updated_toast.div"
+61.Click drivers menu,click,,"admin.drivers.menu.icon"
+62.Click drivers menu,click,,"admin.drivers.menu.icon"
+63.Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+64.Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+65.Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+66.Load Driver App,switch_to,driver,
+67.Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+68.Click Document,tap,,"mobile.driver.documents.menu"
+69.Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+70.Click Back,tap,,"mobile.driver.back.btn"
+71.Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+72.Click Back,tap,,"mobile.driver.back.btn"
+73.Click Online,tap_coordinate,986:1936,
+74. Load User App, switch_to, user, 
+75. Wait For Get Started, wait_until_visible, ,"mobile.customer.get_started.btn"
+76. Click Get Started, tap, ,"mobile.customer.get_started.btn"
+77. Click Allow Notification, tap, ,"mobile.customer.permission_allow.btn"
+78. Click Next, tap, , "mobile.customer.next.btn"
+79. Click Mobile Number, tap, ,"mobile.customer.mobile_number_field.btn"
+80. Click Close, tap, , "mobile.customer.cancel.btn"
+81. Enter Mobile Number, type, {userPhone}, "mobile.customer.edit_text.input"
+82. Wait for Continue, wait_until_visible, , "mobile.customer.continue.btn"
+83. Click Continue, tap, ,"mobile.customer.continue.btn"
+84. Enter OTP, type, 123456, "mobile.customer.edit_text.input"
+85. Wait for Finish, wait_until_visible, ,"mobile.customer.finish.btn"
+86. Click Finish, tap, ,"mobile.customer.finish.btn"
+87. Click Allow Location, tap, ,"mobile.customer.location_allow.btn"
+88. Wait For Auto Ride, wait_until_visible, ,"mobile.customer.auto_ride.btn"
+89. Click Auto Ride, tap, ,"mobile.customer.auto_ride.btn"
+90. Enter Destination, type, Parsn Manare,"mobile.customer.destination.input"
+91. Wait for Location, wait_until_visible, ,"mobile.customer.set_location_map.btn"
+92. Select Destination, tap_coordinate, 545:1299, 
+93. Click Confirm, tap, ,"mobile.customer.confirm.btn"
+94. Wait for Ride, wait_until_visible, ,"mobile.customer.ride_now.btn"
+95. Ride Now, tap, , "mobile.customer.ride_now.btn"
+96. Load Driver App, switch_to, driver, 
+97. Wait for Accept, wait_until_visible, ,"mobile.driver.auto_ride_notification.label"
+98. Accept Ride, tap_coordinate, 801:2113, 
+99. Wait for On My Way, wait_until_visible, ,"mobile.driver.on_my_way.btn"
+100. Wait for Arrived, wait_until_visible, ,"mobile.driver.arrived.btn"
+101. Ride Arrived, tap, ,"mobile.driver.arrived.btn"
+102. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
+103. Yes Arrived, tap, ,"mobile.driver.yes.btn"
+104. Wait for Start Ride, wait_until_visible, ,"mobile.driver.start_ride.btn"
+105. Start Ride, tap, ,"mobile.driver.start_ride.btn"
+106. Wait for OTP, wait_until_visible, ,"mobile.driver.otp_view.input"
+107. Enter OTP, type, 1234,"mobile.driver.otp_view.input"
+108. Wait for Start Ride Confirm, wait_until_visible, ,"mobile.driver.start.btn"
+109. Start Ride Confirm, tap, ,"mobile.driver.start.btn"
+110. Wait for Complete Ride, wait_until_visible, ,"mobile.driver.complete_ride.btn"
+111. Complete Ride, tap, ,"mobile.driver.complete_ride.btn"
+112. Wait for Collect Payment, wait_until_visible, ,"mobile.driver.collect_payment.btn"
+113. Collect Payment, tap, ,"mobile.driver.collect_payment.btn"
+114. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
+115. Confirm Payment, tap, ,"mobile.driver.yes.btn"
+116. Give Rating, tap_coordinate, 348:1545, 
+117. Submit Rating, tap, ,"mobile.driver.submit_rating.btn"
+118. Load User App, switch_to, user, 
+119. Wait for Proceed Payment, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
+120. Proceed Payment, tap, ,"mobile.customer.proceed_to_pay.btn"
+121. Wait for Proceed Pay Confirm, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
+122. Pay Cash, tap, , "mobile.customer.proceed_to_pay.btn"
+123. Wait for Review, wait_until_visible, ,"mobile.customer.give_review.btn"
+124. Give Review, tap, ,"mobile.customer.give_review.btn"
+125. Give Rating, tap_coordinate, 348:1619, 
+126. Submit Rating, tap, , "mobile.customer.submit_rating.btn"
+127. Wait for Done, wait_until_visible, ,"mobile.customer.done.btn"
+128. Trip Finished, tap, , "mobile.customer.done.btn"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto Ride Complete Life Cycle Test Without Wallet Using Locator </t>
+  </si>
+  <si>
+    <t>TC_CA_15_Autoride_Locator_Test</t>
   </si>
 </sst>
 </file>
@@ -2513,6 +3043,308 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA441742-FACE-4539-AA06-56BC1BB72A03}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="36.88671875" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E5A465-4C2B-4523-8755-30CE3021A8BD}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="31.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DE31E4-5C3B-413E-B08A-861302F9F4DC}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1895CC0E-D326-49C3-B5DA-E3C80EEAE5A9}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74DE6E4A-8100-4C1D-8A58-4E86A951B80B}">
   <dimension ref="A1:H3"/>

</xml_diff>

<commit_message>
60th Commit : Web And Emulators Side by Side Intilization Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D7DF15-9BD7-4290-AB8E-9EECC810B510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4383D7CB-E8BA-4909-A07B-FEDB535F41D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -1843,12 +1843,6 @@
 128.Trip Finished,tap,,"accessibility=Done"</t>
   </si>
   <si>
-    <t>1. Enter  Email , type , super_admin@gmail.com, "admin.login.email"
-2. Enter Password,type,R1mep@321, "admin.login.password"
-3. Click Login,click,,"admin.login.submit_btn"
-4. Verify Dashboard,verify,,"admin.dashboard.statistics_header"</t>
-  </si>
-  <si>
     <t>Super Admin Locator</t>
   </si>
   <si>
@@ -2231,6 +2225,24 @@
   </si>
   <si>
     <t>SA_TS_15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto Ride Complete Life Cycle Test Without Wallet Using Locator </t>
+  </si>
+  <si>
+    <t>TC_CA_15_Autoride_Locator_Test</t>
+  </si>
+  <si>
+    <t>1.Load User App, switch_to, user, 
+2.Wait For Get Started, wait_until_visible, ,"mobile.customer.get_started.btn"
+3.Load Driver App, switch_to, driver, 
+4.Wait For Notification, wait_until_visible, , "mobile.driver.permission_allow.btn"
+5.Load  Super Admin,switch_to,web,
+6.Wait For Admin, wait_until_visible, , "admin.login.email"
+7.Enter  Email , type , super_admin@gmail.com, "admin.login.email"
+8.Enter Password,type,R1mep@321, "admin.login.password"
+9.Click Login,click,,"admin.login.submit_btn"
+10.Verify Dashboard,verify,,"admin.dashboard.statistics_header"</t>
   </si>
   <si>
     <t>1. Load Driver App, switch_to, driver, 
@@ -2333,40 +2345,35 @@
 98. Accept Ride, tap_coordinate, 801:2113, 
 99. Wait for On My Way, wait_until_visible, ,"mobile.driver.on_my_way.btn"
 100. Wait for Arrived, wait_until_visible, ,"mobile.driver.arrived.btn"
-101. Ride Arrived, tap, ,"mobile.driver.arrived.btn"
-102. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
-103. Yes Arrived, tap, ,"mobile.driver.yes.btn"
-104. Wait for Start Ride, wait_until_visible, ,"mobile.driver.start_ride.btn"
-105. Start Ride, tap, ,"mobile.driver.start_ride.btn"
-106. Wait for OTP, wait_until_visible, ,"mobile.driver.otp_view.input"
-107. Enter OTP, type, 1234,"mobile.driver.otp_view.input"
-108. Wait for Start Ride Confirm, wait_until_visible, ,"mobile.driver.start.btn"
-109. Start Ride Confirm, tap, ,"mobile.driver.start.btn"
-110. Wait for Complete Ride, wait_until_visible, ,"mobile.driver.complete_ride.btn"
-111. Complete Ride, tap, ,"mobile.driver.complete_ride.btn"
-112. Wait for Collect Payment, wait_until_visible, ,"mobile.driver.collect_payment.btn"
-113. Collect Payment, tap, ,"mobile.driver.collect_payment.btn"
-114. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
-115. Confirm Payment, tap, ,"mobile.driver.yes.btn"
-116. Give Rating, tap_coordinate, 348:1545, 
-117. Submit Rating, tap, ,"mobile.driver.submit_rating.btn"
-118. Load User App, switch_to, user, 
-119. Wait for Proceed Payment, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
-120. Proceed Payment, tap, ,"mobile.customer.proceed_to_pay.btn"
-121. Wait for Proceed Pay Confirm, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
-122. Pay Cash, tap, , "mobile.customer.proceed_to_pay.btn"
-123. Wait for Review, wait_until_visible, ,"mobile.customer.give_review.btn"
-124. Give Review, tap, ,"mobile.customer.give_review.btn"
-125. Give Rating, tap_coordinate, 348:1619, 
-126. Submit Rating, tap, , "mobile.customer.submit_rating.btn"
-127. Wait for Done, wait_until_visible, ,"mobile.customer.done.btn"
-128. Trip Finished, tap, , "mobile.customer.done.btn"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Auto Ride Complete Life Cycle Test Without Wallet Using Locator </t>
-  </si>
-  <si>
-    <t>TC_CA_15_Autoride_Locator_Test</t>
+101. Wait for Arrived, wait_until_visible, ,"mobile.driver.arrived.btn"
+102. Ride Arrived, tap, ,"mobile.driver.arrived.btn"
+103. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
+104. Yes Arrived, tap, ,"mobile.driver.yes.btn"
+105. Wait for Start Ride, wait_until_visible, ,"mobile.driver.start_ride.btn"
+106. Start Ride, tap, ,"mobile.driver.start_ride.btn"
+107. Wait for OTP, wait_until_visible, ,"mobile.driver.otp_view.input"
+108. Enter OTP, type, 1234,"mobile.driver.otp_view.input"
+109. Wait for Start Ride Confirm, wait_until_visible, ,"mobile.driver.start.btn"
+110. Start Ride Confirm, tap, ,"mobile.driver.start.btn"
+111. Wait for Complete Ride, wait_until_visible, ,"mobile.driver.complete_ride.btn"
+112. Complete Ride, tap, ,"mobile.driver.complete_ride.btn"
+113. Wait for Collect Payment, wait_until_visible, ,"mobile.driver.collect_payment.btn"
+114. Collect Payment, tap, ,"mobile.driver.collect_payment.btn"
+115. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
+116. Confirm Payment, tap, ,"mobile.driver.yes.btn"
+117. Give Rating, tap_coordinate, 348:1545, 
+118. Submit Rating, tap, ,"mobile.driver.submit_rating.btn"
+119. Load User App, switch_to, user, 
+120. Wait for Proceed Payment, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
+121. Proceed Payment, tap, ,"mobile.customer.proceed_to_pay.btn"
+122. Wait for Proceed Pay Confirm, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
+123. Pay Cash, tap, , "mobile.customer.proceed_to_pay.btn"
+124. Wait for Review, wait_until_visible, ,"mobile.customer.give_review.btn"
+125. Give Review, tap, ,"mobile.customer.give_review.btn"
+126. Give Rating, tap_coordinate, 348:1619, 
+127. Submit Rating, tap, , "mobile.customer.submit_rating.btn"
+128. Wait for Done, wait_until_visible, ,"mobile.customer.done.btn"
+129. Trip Finished, tap, , "mobile.customer.done.btn"</t>
   </si>
 </sst>
 </file>
@@ -3084,21 +3091,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -3162,22 +3169,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3237,22 +3244,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3310,22 +3317,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
64th Commit : Browser size Flexible For Mobile and Web Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAD3C24-384F-4833-901F-439CE2D469E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0DCBE08-EEA3-4235-8BB0-0C06C0716442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2305,7 +2305,7 @@
 58. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
 59. Click Approve Driver,click,,"admin.drivers.docs.approval"
 60. Verify Updated Successfully,verify,,"web.global.toast.updated"
-61. Click drivers menu,click,,"admin.drivers.menu.icon"
+61. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 62. Click drivers menu,click,,"admin.drivers.menu.icon"
 63. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
 64. Approved Drivers List,verify,,"admin.drivers.approved_page.header"

</xml_diff>

<commit_message>
68th Commit :Auto Ride Full Test  Updated With Wait Till Visible
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A45A3B-4D3E-411B-B8CB-5883BCC3FDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEECFB57-3AE6-43A9-8664-6F945368A9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -2080,18 +2080,6 @@
     <t>TC_CA_15_Autoride_Locator_Test</t>
   </si>
   <si>
-    <t>1. Load User App,switch_to,user,
-2. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-3. Load Driver App,switch_to,driver,
-4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-5. Load Super Admin,switch_to,web,
-6. Wait For Admin,wait_until_visible,,"web.global.login.email"
-7. Enter Email,type,super_admin@gmail.com,"web.global.login.email"
-8. Enter Password,type,R1mep@321,"web.global.login.password"
-9. Click Login,click,,"web.global.login.submit_btn"
-10. Verify Dashboard,verify,,"web.global.dashboard.statistics_header"</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
@@ -2180,10 +2168,30 @@
 </t>
   </si>
   <si>
+    <t>Removed Steps</t>
+  </si>
+  <si>
+    <t>7.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+8.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+9.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"</t>
+  </si>
+  <si>
+    <t>1. Load User App,switch_to,user,
+2. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+3. Load Driver App,switch_to,driver,
+4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5. Load Super Admin,switch_to,web,
+6. Wait For Admin,wait_until_visible,,"web.global.login.email"
+7. Enter Email,type,super_admin@gmail.com,"web.global.login.email"
+8. Enter Password,type,R1mep@321,"web.global.login.password"
+9. Click Login,click,,"web.global.login.submit_btn"
+10.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"</t>
+  </si>
+  <si>
     <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 2. Click Customer Icon,click,,"admin.menu.customer_icon"
 3. Click Add Customers,click,,"admin.menu.add_customers"
-4. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
+4. Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
 5. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
 6. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
 7. Enter Contact Number,type,{randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
@@ -2192,18 +2200,18 @@
 10. Select Male,click,,"admin.customer.select_gender_male"
 11.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
 12.Click Submit,click,,"web.global.action.submit"
-13. Verify Added Successfully,verify,,"web.global.toast.info"
+13. Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
 14.Click Dashboard Icon,click,,"web.global.menu.dashboard"
 15.Click Customer Icon,click,,"admin.menu.customer_icon"
 16.Click Verified Customers,click,,"admin.menu.verified_customers"
-17. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
+17. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
 18.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
   </si>
   <si>
     <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 2. Click drivers menu,click,,"admin.drivers.menu.icon"
 3. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
-4. Verify Add Driver page,verify,,"admin.drivers.add_page.header"
+4. Wait For Add Driver page,wait_until_visible,,"admin.drivers.add_page.header"
 5. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
 6. Select Auto Ride Option,click,,"admin.drivers.service_option.autoride"
 7. Enter Driver Name,type,autodriver{randomAlpha} &gt;&gt; autoName,"admin.drivers.fullname.input"
@@ -2228,7 +2236,7 @@
 26. Enter Payment Email Address,type,{autoEmail},"admin.drivers.paymentemail.input"
 27. Enter IFSC Code,type,HDFC0001234,"admin.drivers.ifsc.input"
 28. Click Submit Button,click,,"web.global.action.submit"
-29. Verify Driver Added Successfully,verify,,"web.global.toast.success"
+29. Wait For Driver Added Successfully,wait_until_visible,,"web.global.toast.success"
 30. Wait for Toast to Hide,wait,1000,,
 31.Click Dashboard Icon,click,,"web.global.menu.dashboard"
 32. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
@@ -2295,14 +2303,14 @@
 56. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
 57. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
 58. Click Doc Icon,click,,"admin.drivers.docs.icon"
-59. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+59. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
 60. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
 61. Click Approve Driver,click,,"admin.drivers.docs.approval"
-62. Verify Updated Successfully,verify,,"web.global.toast.updated"
+62. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
 63. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 64. Click drivers menu,click,,"admin.drivers.menu.icon"
 65. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
-66. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+66.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
 67. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
 68. Load Driver App,switch_to,driver,
 69. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
@@ -2368,14 +2376,6 @@
 129. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
 130. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
 131. Trip Finished,tap,,"mobile.customer.done.btn"</t>
-  </si>
-  <si>
-    <t>Removed Steps</t>
-  </si>
-  <si>
-    <t>7.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-8.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-9.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"</t>
   </si>
 </sst>
 </file>
@@ -3093,7 +3093,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>70</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -3183,7 +3183,7 @@
         <v>75</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>76</v>
@@ -3238,7 +3238,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -3258,13 +3258,13 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>77</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3334,7 +3334,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>80</v>
@@ -3563,7 +3563,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -3635,7 +3635,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
74th Commit: Auto Ride Test Completed
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFF04D7-0A0A-4ABD-8B02-B335DB125DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4586DAD3-08FC-4A0E-BF6E-4A1B75BC6469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="98">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -2381,6 +2381,147 @@
 33. Click Pending Documents Menu,click,,"admin.drivers.pending_docs.link"
 34. Filter Pending Docs by Name,type,{autoName},"admin.drivers.name_filter.input"
 35. Click Dashboard Home Icon,click,,"web.global.menu.dashboard"</t>
+  </si>
+  <si>
+    <t>1. Load Driver App,switch_to,driver,
+2. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+3. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+4. Click Agree,tap,,"mobile.driver.agree.btn"
+5. Click Get Started,tap,,"mobile.driver.get_started.btn"
+6. Click Next,tap,,"mobile.driver.next.btn"
+7. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+8. Click Close,tap,,"mobile.driver.cancel.btn"
+9. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+10. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+11. Click Continue,tap,,"mobile.driver.continue.btn"
+12. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+13. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+14. Wait For Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+15. Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+16. Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+17. Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+18. Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+19. Drag Page Layout Upward,swipe,up,
+20. Click Liability,tap,,"mobile.driver.liability.checkbox"
+21. Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+22. Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+23. Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+24. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+25. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+26. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+27. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+28. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+29. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+30. Click Document,tap,,"mobile.driver.documents.menu"
+31. Wait For Document Page,wait_until_visible,,"mobile.driver.add_documents.header"
+32. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+33. Click Upload,tap,,"mobile.driver.upload.btn"
+34. Upload License,uploadfile,"src/main/resources/test-data/license.JPG","mobile.driver.upload_docs.btn"
+35. Wait For Sort,wait_until_visible,,"mobile.driver.android_content.view"
+36. Click Sort,tap,,"mobile.driver.android_content.view"
+37. Wait For Modified,wait_until_visible,,"mobile.driver.sort_modified.btn"
+38. Click Modified,tap,,"mobile.driver.sort_modified.btn"
+39. Click License,tap,,"mobile.driver.license_thumb.icon"
+40. Wait For Crop,wait_until_visible,,"mobile.driver.crop.btn"
+41. Click Crop,tap,,"mobile.driver.crop.btn"
+42. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+43. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+44. Click Month,tap,,"mobile.driver.next_month.btn"
+45. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+46. Click Ok,tap,,"mobile.driver.ok.btn"
+47. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+48. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+49. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+50. Click Back,tap,,"mobile.driver.back.btn"
+51. Load Admin App,switch_to,web,
+52. Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+53. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+54. Click drivers menu,click,,"admin.drivers.menu.icon"
+55. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+56. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+57. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+58. Click Doc Icon,click,,"admin.drivers.docs.icon"
+59. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
+60. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+61. Click Approve Driver,click,,"admin.drivers.docs.approval"
+62. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
+63. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+64. Click drivers menu,click,,"admin.drivers.menu.icon"
+65. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+66.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
+67. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+68. Load Driver App,switch_to,driver,
+69. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+70. Click Document,tap,,"mobile.driver.documents.menu"
+71. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+72. Click Back,tap,,"mobile.driver.back.btn"
+73. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+74. Click Back,tap,,"mobile.driver.back.btn"
+75. Click Online,tap_coordinate,986:1936,
+76. Load User App,switch_to,user,
+77. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+78. Click Get Started,tap,,"mobile.customer.get_started.btn"
+79. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+80. Click Next,tap,,"mobile.customer.next.btn"
+81. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+82. Click Close,tap,,"mobile.customer.cancel.btn"
+83. Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+84. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+85. Click Continue,tap,,"mobile.customer.continue.btn"
+86. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+87. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+88. Click Finish,tap,,"mobile.customer.finish.btn"
+89. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+90. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+91. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+92. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+93. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+94. Select Destination,tap_coordinate,545:1299,
+95. Click Confirm,tap,,"mobile.customer.confirm.btn"
+96. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+97. Ride Now,tap,,"mobile.customer.ride_now.btn"
+98. Load Driver App,switch_to,driver,
+99. Wait for Accept,wait_until_visible,,"mobile.driver.auto_ride_notification.label"
+100. Accept Ride,tap_coordinate,801:2113,
+101. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+102. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+103. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+104. Ride Arrived,tap,,"mobile.driver.arrived.btn"
+105. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+106. Yes Arrived,tap,,"mobile.driver.yes.btn"
+107. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+108. Start Ride,tap,,"mobile.driver.start_ride.btn"
+109. Wait for OTP,wait_until_visible,,"mobile.driver.otp_view.input"
+110. Enter OTP,type,1234,"mobile.driver.otp_view.input"
+111. Wait for Start Ride Confirm,wait_until_visible,,"mobile.driver.start.btn"
+112. Start Ride Confirm,tap,,"mobile.driver.start.btn"
+113. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+114. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+115. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+116. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+117. Load User App,switch_to,user,
+118. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+119. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+120. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+121. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+122. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+123. Give Review,tap,,"mobile.customer.give_review.btn"
+124. Give Rating,tap_coordinate,348:1619,
+125. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+126. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+127. Trip Finished,tap,,"mobile.customer.done.btn"</t>
+  </si>
+  <si>
+    <t>Previsous Test Steps</t>
+  </si>
+  <si>
+    <t>Deleted Test Steps</t>
+  </si>
+  <si>
+    <t>117. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+118. Confirm Payment,tap,,"mobile.driver.yes.btn"
+119. Give Rating,tap_coordinate,348:1545,
+120. Submit Rating,tap,,"mobile.driver.submit_rating.btn"</t>
   </si>
 </sst>
 </file>
@@ -3298,8 +3439,8 @@
     <col min="4" max="4" width="29.109375" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -3322,10 +3463,10 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>6</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
@@ -3342,10 +3483,16 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>80</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
77th Commit: Auto Ride Test Completed
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{782D6142-FF10-40C4-80E9-EF7763CE7F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86FB5E2-094E-4356-A449-962A8957A2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1355,7 +1355,7 @@
 125. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
 126. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
 127. Trip Finished,tap,,"mobile.customer.done.btn"
-128.Wait for Auto Ride Detial,wait_until_visible,,"mobile.customer.ride_complete.heading"
+128.Wait for Back,wait_until_visible,,"mobile.driver.back.btn"
 129.Click Back,tap,,"mobile.driver.back.btn"
 130.Wait for Profile Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
 130.Profile, tap_coordinate ,971:2102,COORDINATE_MODE

</xml_diff>

<commit_message>
78th Commit: Reload App Keyword Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86FB5E2-094E-4356-A449-962A8957A2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43545072-72FC-4B5E-B0C7-65ABABDE62D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -264,18 +264,6 @@
     <t>7.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
 8.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
 9.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"</t>
-  </si>
-  <si>
-    <t>1. Load User App,switch_to,user,
-2. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-3. Load Driver App,switch_to,driver,
-4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-5. Load Super Admin,switch_to,web,
-6. Wait For Admin,wait_until_visible,,"web.global.login.email"
-7. Enter Email,type,super_admin@gmail.com,"web.global.login.email"
-8. Enter Password,type,R1mep@321,"web.global.login.password"
-9. Click Login,click,,"web.global.login.submit_btn"
-10.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"</t>
   </si>
   <si>
     <t>1. Load Driver App,switch_to,driver,
@@ -1225,7 +1213,9 @@
 110.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
 111.Click Logout,tap,,"mobile.customer.logout.btn"
 112.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
-113.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"</t>
+113.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
+114.Reload User App Completely,reload_app,user,
+115.Reload Driver App Completely,reload_app,driver,</t>
   </si>
   <si>
     <t>1. Load Driver App,switch_to,driver,
@@ -1377,7 +1367,22 @@
 146.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
 147.Click Logout,tap,,"mobile.driver.logout.btn"
 148.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
-149.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"</t>
+149.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
+150.Reload User App Completely,reload_app,user,
+151.Reload Driver App Completely,reload_app,driver,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Load User App,switch_to,user,
+2. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+3. Load Driver App,switch_to,driver,
+4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5. Load Super Admin,switch_to,web,
+6. Wait For Admin,wait_until_visible,,"web.global.login.email"
+7. Enter Email,type,super_admin@gmail.com,"web.global.login.email"
+8. Enter Password,type,R1mep@321,"web.global.login.password"
+9. Click Login,click,,"web.global.login.submit_btn"
+10.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+</t>
   </si>
 </sst>
 </file>
@@ -1789,24 +1794,24 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1859,7 +1864,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -1870,22 +1875,22 @@
         <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1945,22 +1950,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -2020,22 +2025,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2093,22 +2098,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2163,36 +2168,36 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>28</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2254,13 +2259,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
82th Commit: Regression Test With New Apk Started & tap_if_present Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2BAE396-E242-411B-94F7-B8A56ED8C1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CF0F9F-36A5-409F-8E0A-E9CA7A1DDD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="67">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -808,119 +808,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The UserDriverWebIntialilzer, HybridAddCustomer and HybridApprovedAutoDriver test sheets must always be executed prior to running this  test
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">UserDriverWebIntialilzer,HybridAddCustomer,HybridApprovedAutoDriver
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
-  </si>
-  <si>
     <t>SA_TS_04</t>
   </si>
   <si>
@@ -931,118 +818,6 @@
   </si>
   <si>
     <t>TC_CA_05_Autoride_Complete_Test</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The UserDriverWebIntialilzer,HybridAddCustomer and  HybridUnApprovedAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>UserDriverWebIntialilzer,HybridAddCustomer,HybridUnApprovedAutoDriver</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
   </si>
   <si>
     <t>SA_TS_06</t>
@@ -1236,83 +1011,247 @@
     <t>Driver App Wallet Verification</t>
   </si>
   <si>
-    <t>1. Load Driver App,switch_to,driver,
+    <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
-3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-4. Load Super Admin,switch_to,web,
-5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
-6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-7. Click Settings Menu,click,,"web.global.menu.settings"
-8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-10.Wait For On,wait,2000,
-11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
-12. Click Submit Button,click,,"web.global.action.submit"
-13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-14. Load Driver App,switch_to,driver,
-15. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-16. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-17. Click Agree,tap,,"mobile.driver.agree.btn"
-18. Click Get Started,tap,,"mobile.driver.get_started.btn"
-19. Click Next,tap,,"mobile.driver.next.btn"
-20. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-21. Click Close,tap,,"mobile.driver.cancel.btn"
-22. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-23. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-24. Click Continue,tap,,"mobile.driver.continue.btn"
-25. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-26. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-27. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-28. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-29.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
-30.Click Wallet,tap,,"mobile.driver.wallet.btn"
-31.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
-32.Click Topup,tap,,"mobile.driver.top_up.btn"
-33.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
-34.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
-35.Click Proceed,tap,,"mobile.driver.top_up.proceed"
-36.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
-37.Enter Driver Mobile,type,regression.approved_driver.phone,"mobile.driver.top_up.contact_no_box"
-38.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
-39.Wait For Net Banking,wait,3000,
-40.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
-41.Click Bob,tap_coordinate,277:1124,
-42.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
-43.Click Success,tap,,"mobile.driver.top_up.succes_popup"
-44.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
-45.Click Back,tap,,"mobile.driver.back.btn"
-46.Drag Page Layout Upward,swipe,up,
-47.Click Back,tap,,"mobile.driver.back.btn"
-48.Reload Driver App Completely,reload_app,driver,
-49. Switch To Web Session,switch_to,web,
-50.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-51. Click Settings Menu,click,,"admin.setting.sidebar.menu"
-52. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-53. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-54.Wait For off,wait,2000,
-55. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
-56. Click Submit Button,click,,"web.global.action.submit"
-57. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-58. Switch To Driver Session,switch_to,driver,
-59. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-60. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-61. Click Agree,tap,,"mobile.driver.agree.btn"
-62. Click Get Started,tap,,"mobile.driver.get_started.btn"
-63. Click Next,tap,,"mobile.driver.next.btn"
-64. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-65. Click Close,tap,,"mobile.driver.cancel.btn"
-66. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-67. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-68. Click Continue,tap,,"mobile.driver.continue.btn"
-69. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-70. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-71. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-72.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-73.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-74.Check Wallet absent,element_absent,,"accessibility=Wallet"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+3.Load Super Admin,switch_to,web,
+4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5.Click Subscription Plan,click,,"admin.subscription.menu_link"
+6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
+8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
+9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
+12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
+14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
+15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
+16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
+17.Enter Price, type,5000, "admin.subscription.common.price.input"
+18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
+19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
+20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
+21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
+22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+23.Select On,click,,"admin.subscription.common.status.option_on"
+24.Click Submit ,click,,"web.global.action.submit"
+25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+26.Click badge,click,,"admin.subscription.badge.icon"
+27.Click Subscription Plan,click,,"admin.subscription.menu_link"
+28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
+30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+32.Select Pest Control,click,,"admin.subscription.common.category.option_pest"
+33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
+34.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+35.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+36.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
+39.Enter Price, type,5000, "admin.subscription.common.price.input"
+40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
+41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
+42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
+43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
+44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+45.Select On,click,,"admin.subscription.common.status.option_on"
+46.Click Submit ,click,,"web.global.action.submit"
+47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+48.Load User App,switch_to,user,
+49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+50.Click Get Started,tap,,"mobile.customer.get_started.btn"
+51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+52.Click Next,tap,,"mobile.customer.next.btn"
+53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+54.Click Close,tap,,"mobile.customer.cancel.btn"
+55.Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+57.Click Continue,tap,,"mobile.customer.continue.btn"
+58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+59.Click Finish,tap,,"mobile.customer.finish.btn"
+60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+62.Click Subscription,tap,,"mobile.customer.subscription.btn"
+63.Wait Customer Plan,wait_until_visible,,"mobile.customer.dynamic_subscription.plan"
+64.Click Customer Plan,tap,,"mobile.customer.dynamic_subscription.plan"
+65.Load Driver App,switch_to,driver,
+66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
+67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+68.Click Agree,tap,,"mobile.driver.agree.btn"
+69.Click Get Started,tap,,"mobile.driver.get_started.btn"
+70.Click Next,tap,,"mobile.driver.next.btn"
+71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+72.Click Close,tap,,"mobile.driver.cancel.btn"
+73.Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+75.Click Continue,tap,,"mobile.driver.continue.btn"
+76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+78.Wait for Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+79.Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+80.Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+81.Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+82.Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+83.Drag Page Layout Upward,swipe,up,
+84.Click Liability,tap,,"mobile.driver.liability.checkbox"
+85.Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+86.Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+87.Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+88.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+89.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+90.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+91.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+92.Wait Till Setting Popup,wait_if_present,,"mobile.driver.goto_settings.pop_up"
+93.Click Go To Setting Popup,tap_if_present,,"mobile.driver.goto_settings.pop_up"
+94.Wait For Mobile App,wait_if_present,,"mobile.driver.goto_settings.select_driver_app"
+95.Select Driver App,tap_if_present,,"mobile.driver.goto_settings.select_driver_app"
+96.Wait For Toggle Button,wait_if_present,,"mobile.driver.goto_settings.toggle_button"
+97.Click Allow Toggle Button,tap_if_present,,"mobile.driver.goto_settings.toggle_button"
+98.Move Back From Toggle Page,tap_if_present,,"mobile.driver.goto_settings.back_from_toggle_page"
+99.Wait For Mobile App,wait_if_present,,"mobile.driver.goto_settings.select_driver_app"
+100.Move Back From App Page,tap_if_present,,"mobile.driver.goto_settings.back_from_select_driver_app_page"
+101.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+102.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+103.Click Subscription,tap,,"mobile.driver.subscription.btn"
+104.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+105.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
+106.Click Back,tap,,"mobile.driver.back.btn"
+107.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+108.Drag Page Layout Upward,swipe,up,
+110.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+111.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
+112.Click Logout,tap,,"mobile.driver.logout.btn"
+113.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
+114.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
+115.Load User App,switch_to,user,
+116.Click Back,tap,,"mobile.driver.back.btn"
+117.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
+118.Drag Page Layout Upward,swipe,up,
+120.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+121.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
+122.Click Logout,tap,,"mobile.customer.logout.btn"
+123.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
+124.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"</t>
+  </si>
+  <si>
+    <t>Orginal Test Steps Old Apk</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The UserDriverWebIntialilzer, HybridAddCustomer and HybridApprovedAutoDriver test sheets must always be executed prior to running this  test
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">UserDriverWebIntialilzer
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3. Load Driver App,switch_to,driver,
 4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
@@ -1322,7 +1261,7 @@
 8. Click Next,tap,,"mobile.driver.next.btn"
 9. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
 10. Click Close,tap,,"mobile.driver.cancel.btn"
-11. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+11. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
 12. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
 13. Click Continue,tap,,"mobile.driver.continue.btn"
 14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
@@ -1463,11 +1402,348 @@
 149.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
 150.Click Logout,tap,,"mobile.driver.logout.btn"
 151.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
+152.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"</t>
+  </si>
+  <si>
+    <t>80.Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+81.Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+82.Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+83.Drag Page Layout Upward,swipe,up,
+84.Click Liability,tap,,"mobile.driver.liability.checkbox"
+85.Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+86.Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+87.Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+88.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+89.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+106.Click Back,tap,,"mobile.driver.back.btn"
+107.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+108.Drag Page Layout Upward,swipe,up,
+110.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+111.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
+112.Click Logout,tap,,"mobile.driver.logout.btn"
+113.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
+114.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
+115.Load User App,switch_to,user,
+116.Click Back,tap,,"mobile.driver.back.btn"
+117.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
+118.Drag Page Layout Upward,swipe,up,
+120.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+121.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
+122.Click Logout,tap,,"mobile.customer.logout.btn"
+123.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
+124.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
+---------Removed Popup Steps------------
+78.Wait for Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+79.Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+80.Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+81.Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+82.Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+83.Drag Page Layout Upward,swipe,up,
+84.Click Liability,tap,,"mobile.driver.liability.checkbox"
+85.Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+86.Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+87.Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+88.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+89.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+90.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+91.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+92.Wait Till Setting Popup,wait_if_present,,"mobile.driver.goto_settings.pop_up"
+93.Click Go To Setting Popup,tap_if_present,,"mobile.driver.goto_settings.pop_up"
+94.Wait For Mobile App,wait_if_present,,"mobile.driver.goto_settings.select_driver_app"
+95.Select Driver App,tap_if_present,,"mobile.driver.goto_settings.select_driver_app"
+96.Wait For Toggle Button,wait_if_present,,"mobile.driver.goto_settings.toggle_button"
+97.Click Allow Toggle Button,tap_if_present,,"mobile.driver.goto_settings.toggle_button"
+98.Move Back From Toggle Page,tap_if_present,,"mobile.driver.goto_settings.back_from_toggle_page"
+99.Wait For Mobile App,wait_if_present,,"mobile.driver.goto_settings.select_driver_app"
+100.Move Back From App Page,tap_if_present,,"mobile.driver.goto_settings.back_from_select_driver_app_page"</t>
+  </si>
+  <si>
+    <t>117. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+118. Confirm Payment,tap,,"mobile.driver.yes.btn"
+119. Give Rating,tap_coordinate,348:1545,
+120. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+-----Wallet Steps---------------
+66.Load Driver App,switch_to,driver,
+67.Wait For Back,wait_until_visible,,"accessibility=Back"
+68.Click Document,tap,,"accessibility=Documents"
+69.Wait For Add Document,wait_until_visible,,"accessibility=Add Documents"
+70.Click Back,tap,,"accessibility=Back"
+71.Wait For Documents,wait_until_visible,,"accessibility=Documents"
+72.Click Wallet,tap,,"accessibility=Wallet"
+73.Wait For Topup,wait_until_visible,,"accessibility=TopUp"
+74.Click Topup,tap,,"accessibility=TopUp"
+75.Wait For Topup Sum,wait_until_visible,,"accessibility=TopUp"
+76.Click Hundered,tap,,"accessibility=₹ 100.00"
+77.Click Proceed,tap,,"accessibility=Proceed"
+78.Wait For Contact No,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+79.Enter Driver Mobile,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+80.Wait For Payment Options,wait_until_visible,,"automator=new UiSelector().text("Payment Options")"
+81.Click Net Banking,tap,,"automator=new UiSelector().text("Netbanking")"
+82.Click Bob,tap_coordinate,277:1124,
+83.Wait For Success,wait_until_visible,,"automator=new UiSelector().text("Success")"
+84.Click Success,tap,,"automator=new UiSelector().text("Success")"
+85.Wait For Wallet  Back,wait_until_visible,,"accessibility=Wallet"
+86.Click Back,tap,,"accessibility=Back"
+87.Drag Page Layout Upward,swipe,up,
+88.Click Back,tap,,"accessibility=Back"
+89.Click Online,tap_coordinate,986:1936,
+------ popup steps  ------
+16. Wait For Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+17. Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+18. Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+19. Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+20. Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+21. Drag Page Layout Upward,swipe,up,
+22. Click Liability,tap,,"mobile.driver.liability.checkbox"
+23. Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+24. Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+25. Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+26. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+27. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+28. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+29. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+------Drive Upload Document Phone----
+18. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+19.Wait For Pageload,wait,3000,
+20. Click Document,tap,,"mobile.driver.documents.menu"
+21. Wait For Document Page,wait_until_visible,,"mobile.driver.add_documents.header"
+34. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+35. Click Upload,tap,,"mobile.driver.upload.btn"
+36. Upload License,uploadfile,"src/main/resources/test-data/license.JPG","mobile.driver.upload_docs.btn"
+37. Wait For Sort,wait_until_visible,,"mobile.driver.android_content.view"
+38. Click Sort,tap,,"mobile.driver.android_content.view"
+39. Wait For Modified,wait_until_visible,,"mobile.driver.sort_modified.btn"
+40. Click Modified,tap,,"mobile.driver.sort_modified.btn"
+41. Click License,tap,,"mobile.driver.license_thumb.icon"
+42. Wait For Crop,wait_until_visible,,"mobile.driver.crop.btn"
+43. Click Crop,tap,,"mobile.driver.crop.btn"
+44. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+45. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+46. Click Month,tap,,"mobile.driver.next_month.btn"
+47. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+48. Click Ok,tap,,"mobile.driver.ok.btn"
+49. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+50. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+51. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+52. Click Back,tap,,"mobile.driver.back.btn"
+---------------Documet verification Super Admin ---------------------------
+53. Load Admin App,switch_to,web,
+54. Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+55. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+56. Click drivers menu,click,,"admin.drivers.menu.icon"
+57. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+58. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+59. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+60. Click Doc Icon,click,,"admin.drivers.docs.icon"
+61. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
+62. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+63. Click Approve Driver,click,,"admin.drivers.docs.approval"
+64. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
+65. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+66. Click drivers menu,click,,"admin.drivers.menu.icon"
+67. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+68.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
+69. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+70. Load Driver App,switch_to,driver,
+71. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+72. Click Document,tap,,"mobile.driver.documents.menu"
+73. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+74. Click Back,tap,,"mobile.driver.back.btn"
+75. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+76. Click Back,tap,,"mobile.driver.back.btn"
+-------------Logout Steps----------------
+130.Wait for Back,wait_until_visible,,"mobile.driver.back.btn"
+131.Click Back,tap,,"mobile.driver.back.btn"
+132.Wait for Profile Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+133.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+134.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
+135.Drag Page Layout Upward,swipe,up,
+136.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+137.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+138.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
+139.Click Logout,tap,,"mobile.customer.logout.btn"
+140.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
+141.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
+142.Load Driver App,switch_to,driver,
+143. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+144.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+145.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+146.Drag Page Layout Upward,swipe,up,
+147.Wait For Manage Account,wait_until_visible,,"mobile.driver.manage_account.btn"
+148.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+149.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
+150.Click Logout,tap,,"mobile.driver.logout.btn"
+151.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
 152.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
+----------Online Toggle Button Cordinate-------
+18.Click Online,tap_coordinate,986:1936,
+18.Click Online Toggle Button,tap,,"mobile.driver.online_toggle.btn"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Driver App,switch_to,driver,
+4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6.Click Agree,tap,,"mobile.driver.agree.btn"
+7.Click Get Started,tap,,"mobile.driver.get_started.btn"
+8.Click Next,tap,,"mobile.driver.next.btn"
+9.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+10.Click Close,tap,,"mobile.driver.cancel.btn"
+11.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+12.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+13 Click Continue,tap,,"mobile.driver.continue.btn"
+14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+15.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+16.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+17.Wait For Pageload,wait,3000,
+18.Load User App,switch_to,user,
+19.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+20.Click Get Started,tap,,"mobile.customer.get_started.btn"
+21.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+22.Click Next,tap,,"mobile.customer.next.btn"
+23.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+24.Click Close,tap,,"mobile.customer.cancel.btn"
+25.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+26.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+27. Click Continue,tap,,"mobile.customer.continue.btn"
+28. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+29. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+30. Click Finish,tap,,"mobile.customer.finish.btn"
+31. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+32. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+33. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+34. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+35. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+36. Select Destination,tap_coordinate,545:1299,
+37. Click Confirm,tap,,"mobile.customer.confirm.btn"
+38. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+39. Ride Now,tap,,"mobile.customer.ride_now.btn"
+40. Load Driver App,switch_to,driver,
+41.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+42.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+43.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+44.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+45.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+46.Ride Arrived,tap,,"mobile.driver.arrived.btn"
+47.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+48.Yes Arrived,tap,,"mobile.driver.yes.btn"
+49.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+50.Start Ride,tap,,"mobile.driver.start_ride.btn"
+51.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+52.Enter OTP,type,1234,"mobile.driver.otp_view.input"
+53.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+54.Start Ride Button,tap,,"mobile.driver.start.btn"
+55.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+56.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+57.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+58.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+59.Load User App,switch_to,user,
+60.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+61.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+62. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+63. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+64. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+65. Give Review,tap,,"mobile.customer.give_review.btn"
+66. Give Rating,tap_coordinate,348:1619,
+67. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+68.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+69.Trip Finished,tap,,"mobile.customer.done.btn"
+70. Load Driver App,switch_to,driver,
+71.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
+72.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
+73. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+74. Confirm Payment,tap,,"mobile.driver.yes.btn"
+75.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
+76.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
+77.Wait For Rating,wait,2000,
+78. Give Rating,tap_coordinate,348:1545,
+79. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+80.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
+81.Click Complete Button,tap,,"mobile.driver.complete.btn"
+82.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
+83.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+    <t>1. Load Driver App,switch_to,driver,
+2.Reload Driver App Completely,reload_app,driver,
+3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load Driver App,switch_to,driver,
+15. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+16. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+17. Click Agree,tap,,"mobile.driver.agree.btn"
+18. Click Get Started,tap,,"mobile.driver.get_started.btn"
+19. Click Next,tap,,"mobile.driver.next.btn"
+20. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+21. Click Close,tap,,"mobile.driver.cancel.btn"
+22. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+23. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+24. Click Continue,tap,,"mobile.driver.continue.btn"
+25. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+26. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+27. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+28. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+29.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
+30.Click Wallet,tap,,"mobile.driver.wallet.btn"
+31.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
+32.Click Topup,tap,,"mobile.driver.top_up.btn"
+33.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
+34.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
+35.Click Proceed,tap,,"mobile.driver.top_up.proceed"
+36.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
+37.Enter Driver Mobile,type,regression.approved_driver.phone,"mobile.driver.top_up.contact_no_box"
+38.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
+39.Wait For Net Banking,wait,5000,
+40.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
+41.Wait For Bob,wait,5000,
+42.Click Bob,tap_coordinate,288:1325,
+43.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
+44.Click Success,tap,,"mobile.driver.top_up.succes_popup"
+45.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
+46.Click Back,tap,,"mobile.driver.back.btn"
+47.Drag Page Layout Upward,swipe,up,
+48.Click Back,tap,,"mobile.driver.back.btn"
+49.Reload Driver App Completely,reload_app,driver,
+50. Switch To Web Session,switch_to,web,
+51.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+52. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+53. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+54. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+55.Wait For off,wait,2000,
+56. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+57. Click Submit Button,click,,"web.global.action.submit"
+58. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+59. Switch To Driver Session,switch_to,driver,
+60. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+61. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+62. Click Agree,tap,,"mobile.driver.agree.btn"
+63. Click Get Started,tap,,"mobile.driver.get_started.btn"
+64. Click Next,tap,,"mobile.driver.next.btn"
+65. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+66. Click Close,tap,,"mobile.driver.cancel.btn"
+67. Enter Mobile Number,type,regression.approved_driver.phone ,"mobile.driver.edit_text.input"
+68. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+69. Click Continue,tap,,"mobile.driver.continue.btn"
+70. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+71. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+72. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+73.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+74.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3.Load Super Admin,switch_to,web,
 4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
@@ -1513,7 +1789,7 @@
 44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
 45.Select On,click,,"admin.subscription.common.status.option_on"
 46.Click Submit ,click,,"web.global.action.submit"
-47.Filter Services List,type,{custometSubscriptionName},"admin.subscription.common.filter.input"
+47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
 48.Load User App,switch_to,user,
 49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
 50.Click Get Started,tap,,"mobile.customer.get_started.btn"
@@ -1521,7 +1797,7 @@
 52.Click Next,tap,,"mobile.customer.next.btn"
 53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
 54.Click Close,tap,,"mobile.customer.cancel.btn"
-55.Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
 56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
 57.Click Continue,tap,,"mobile.customer.continue.btn"
 58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
@@ -1539,50 +1815,33 @@
 70.Click Next,tap,,"mobile.driver.next.btn"
 71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
 72.Click Close,tap,,"mobile.driver.cancel.btn"
-73.Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
 74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
 75.Click Continue,tap,,"mobile.driver.continue.btn"
 76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
 77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-78.Wait for Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
-79.Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
-80.Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
-81.Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
-82.Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
-83.Drag Page Layout Upward,swipe,up,
-84.Click Liability,tap,,"mobile.driver.liability.checkbox"
-85.Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
-86.Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
-87.Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
-88.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
-89.Click Agree,tap,,"mobile.driver.agree_continue.btn"
-90.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
-91.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-92.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-93.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-94.Click Subscription,tap,,"mobile.driver.subscription.btn"
-95.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
-96.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
-97.Click Back,tap,,"mobile.driver.back.btn"
-98.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-99.Drag Page Layout Upward,swipe,up,
-100.Wait For Manage Account,wait_until_visible,,"mobile.driver.manage_account.btn"
-101.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
-102.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
-103.Click Logout,tap,,"mobile.driver.logout.btn"
-104.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
-105.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
-106.Load User App,switch_to,user,
-107.Click Back,tap,,"mobile.driver.back.btn"
-108.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
-109.Drag Page Layout Upward,swipe,up,
-110.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-111.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-112.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
-113.Click Logout,tap,,"mobile.customer.logout.btn"
-114.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
-115.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
-</t>
+78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+79.wait for page load,wait,5000,
+80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+81.wait for page load,wait,5000,
+82.Click Subscription,tap,,"mobile.driver.subscription.btn"
+83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+84.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
+85.Load Super Admin,switch_to,web,
+86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+87.Click Subscription Plan,click,,"admin.subscription.menu_link"
+88.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+89.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+90.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
+91.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+92.Wait For Deletion,wait,2000,
+93.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+94.Click Subscription Plan,click,,"admin.subscription.menu_link"
+95.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+96.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
+98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+99.Wait For Deletion,wait,2000,</t>
   </si>
 </sst>
 </file>
@@ -2008,7 +2267,7 @@
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>33</v>
@@ -2237,7 +2496,7 @@
         <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -2266,8 +2525,8 @@
     <col min="4" max="4" width="29.109375" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="7" max="7" width="52.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -2290,15 +2549,15 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>5</v>
+        <v>59</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
@@ -2310,10 +2569,16 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2376,28 +2641,28 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="H2" s="2" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2460,22 +2725,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>22</v>
@@ -2543,13 +2808,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
83th Commit: Non Verified And Delete Customer Hybrid Test Case Added
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CF0F9F-36A5-409F-8E0A-E9CA7A1DDD45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5ECF3CE-1044-4887-BB76-7766BB729DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -20,7 +20,10 @@
     <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId5"/>
     <sheet name="AutoRideCompleteTest" sheetId="47" r:id="rId6"/>
     <sheet name="DriverAppWalletVerificaton" sheetId="48" r:id="rId7"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId8"/>
+    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId8"/>
+    <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId9"/>
+    <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId10"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -32,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="79">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1842,6 +1845,305 @@
 97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
 98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
 99.Wait For Deletion,wait,2000,</t>
+  </si>
+  <si>
+    <t>SA_TS_07</t>
+  </si>
+  <si>
+    <t>Non Verified Customer</t>
+  </si>
+  <si>
+    <t>SA_TS_09</t>
+  </si>
+  <si>
+    <t>Customer Language Check</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Customer_Language_Check</t>
+  </si>
+  <si>
+    <t>SA_TS_10</t>
+  </si>
+  <si>
+    <t>Driver Language Check</t>
+  </si>
+  <si>
+    <t>TC_CA_10_Driver_Language_Check</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3.  Switch To Web Session,switch_to,web,
+4. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5. Click drivers menu,click,,"admin.drivers.menu.icon"
+6. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+7. Verify Add Driver,verify,,"admin.drivers.add_page.header"
+8. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+9. Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+10. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+11. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
+12. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
+13. Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
+14. Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+15. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+16. Select Source,click,,"admin.drivers.source_dropdown.select"
+17. Select Instagram,click,,"admin.drivers.instagram_option.span"
+18. Select Male Gender, click, , "admin.drivers.male_gender.div"
+19. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+20. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+21. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+22. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
+23. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+24. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+25. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+26. Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
+27. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+28. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
+29. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+30. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+31. Click Submit, click, , "web.global.action.submit"
+32. Verify Driver Added, verify, , "web.global.toast.success"
+33. Click drivers menu,click,,"admin.drivers.menu.icon"
+34. Click drivers menu,click,,"admin.drivers.menu.icon"
+35. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+36. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+37. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+38. Click Doc Icon,click,,"admin.drivers.docs.icon"
+39. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+40. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+41. Add Driving License,click,,"admin.drivers.docs.edit_icon"
+42. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+43. Enter Expiry Date,type,12-12-2026,"admin.drivers.doc_expiry.input"
+44. Click Submit, click, , "web.global.action.submit"
+45. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+46. Click Approve Driver,click,,"admin.drivers.docs.approval"
+47. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+48. Click Dashboard,click,,"web.global.menu.dashboard"
+49. Click drivers menu,click,,"admin.drivers.menu.icon"
+50. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+51. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+52. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+53. Wait For Get_Started,wait_until_visible,,"admin.drivers.name_filter.input"
+54. Load Driver App,switch_to,driver,
+55. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+56. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+57. Click Agree,tap,,"mobile.driver.agree.btn"
+58. Click Get Started,tap,,"mobile.driver.get_started.btn"
+59. Click Next,tap,,"mobile.driver.next.btn"
+60. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+61. Click Close,tap,,"mobile.driver.cancel.btn"
+62. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+63. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+64. Click Continue,tap,,"mobile.driver.continue.btn"
+65. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+66. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+67. Wait for Toast to Hide,wait,3000,,
+68. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+69. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+70. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+71. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+72. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+73. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+74. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+75. Drag Page Layout Upward,swipe,up,
+76. Click Language menu,tap,,"mobile.driver.Language.btn"
+77. Wait for Language Setting option,wait,3000,,
+78. Click Select Tamil Language,tap,,"mobile.driver.Language.Tamil.button"
+79. Click Select Tamil Language Update,tap,,"mobile.driver.update.btn"
+80. Wait for Language Setting option,wait,3000,,
+81. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+82. Drag Page Layout Upward,swipe,up,
+83. Click Language menu,tap,,"mobile.driver.Language.btn"
+84. Wait for Language Setting option,wait,3000,,
+85. Click Select Hindi Language,tap,,"mobile.driver.Language.Hindi.button"
+86. Click Select Hindi Language Update,tap,,"mobile.driver.Language.Tamil.update.btn"
+87. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+88. Drag Page Layout Upward,swipe,up,
+89. Click Language menu,tap,,"mobile.driver.Language.btn"
+90. Wait for Language Setting option,wait,3000,,
+91. Click Select Tamil Language,tap,,"mobile.driver.Language.English.button"
+92. Click Select Tamil Language Update,tap,,"mobile.driver.Language.Hindi.update.btn"
+93. Wait for Language Setting option,wait,3000,,
+94. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+95. Drag Page Layout Upward,swipe,up,
+96. Wait for Manage Account Loading,wait,3000,,
+97. Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+98. Click Delete Account,tap,,"mobile.customer.delete_sure.btn"
+99. Click Delete AccountSure,tap,,"mobile.customer.delete_sure.btn"
+100. Switch To Web Session,switch_to,web,
+101. Wait for Menu,wait_until_visible,,"admin.drivers.menu.icon"
+102. Click Driver Menu,click,,"admin.drivers.menu.icon"
+103. Click Driver DropDown,click,,"admin.drivers.menu.icon"
+104. Wait for Agree,wait_until_visible,,"Global.menu.driver_deleted"
+105. Click Delete Driver,click,,"Global.menu.driver_deleted"
+106. Enter Driver Vehicele,type,Pink Auto,"Global.menu.Delete_Driver.Vehicle_Type_Filter" 
+107. scroll grid,tab,4,,”Global.menu.Delete_Driver.Contact_Type_Filter"
+108. Enter Driver Name,type,{autoName},"Global.menu.Delete_Driver.Contact_Type_Filter"
+109. Wait For Delete Driver,wait_until_visible,,"Global.menu.Delete_Driver.Contact_Type_Filter"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17. Click Customer Menu,click,,"admin.menu.customer_icon"
+18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+25. Select Male Gender,click,,"admin.customer.select_gender_male"
+26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+27. Wait for Toast to Hide,wait,3000,,
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+30. Click Customer Menu,click,,"admin.menu.customer_icon"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+33.Wait For Customer Filter,wait,3000,
+34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+35.Wait For Customer,wait,2000,
+36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+37. Load User App,switch_to,user,
+38. Reload User App Completely,reload_app,user,
+39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+42. Click Next,tap,,"mobile.customer.next.btn"
+43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+44. Click Close,tap,,"mobile.customer.cancel.btn"
+45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+46. Click Continue,tap,,"mobile.customer.continue.btn"
+47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+48. Click Finish,tap,,"mobile.customer.finish.btn"
+49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+52.Wait For Profile,wait,5000,
+53. Click Profile,tap_coordinate,558:405,COORDINATE_MODE
+54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
+55.Click Back,tap,,"mobile.customer.back.btn"
+56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+57. Drag Page Layout Upward,swipe,up,
+58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+61. Click Manage Account,tap,,"mobile.customer.delete.btn"
+62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+65. Switch To Web Session,switch_to,web,
+66. Click Customer Menu,click,,"admin.menu.customer_icon"
+67. Click Customer DropDown,click,,"admin.menu.customer_icon"
+68. Click Delete Customer,click,,"admin.menu.customer_deleted"
+69. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+70. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"
+</t>
+  </si>
+  <si>
+    <t>TC_CA_07_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17. Click Customer Menu,click,,"admin.menu.customer_icon"
+18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+25. Select Male Gender,click,,"admin.customer.select_gender_male"
+26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+27. Wait for Toast to Hide,wait,3000,,
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+30. Click Customer Menu,click,,"admin.menu.customer_icon"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+33.Wait For Customer Filter,wait,3000,
+34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+35.Wait For Customer,wait,2000,
+36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+37. Load User App,switch_to,user,
+38. Reload User App Completely,reload_app,user,
+39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+42. Click Next,tap,,"mobile.customer.next.btn"
+43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+44. Click Close,tap,,"mobile.customer.cancel.btn"
+45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+46. Click Continue,tap,,"mobile.customer.continue.btn"
+47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+48. Click Finish,tap,,"mobile.customer.finish.btn"
+49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+52.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+53. Drag Page Layout Upward,swipe,up,
+54. Click Select Language,tap,,"mobile.customer.Language.btn"
+55. Wait for Language Setting option,wait,3000,,
+56. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
+57. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
+58. Wait for Language Setting option,wait,3000,,
+59. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+60. Drag Page Layout Upward,swipe,up,
+61. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
+62. Wait for Language Setting option,wait,3000,,
+63. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
+64. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
+65. Wait for Language Setting option,wait,3000,,
+66. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+67. Drag Page Layout Upward,swipe,up,
+68. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
+69. Wait for Language Setting option,wait,3000,,
+70. Click Select english Language,tap,,"mobile.customer.Language.English.button"
+71. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
+72. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+73. Drag Page Layout Upward,swipe,up,
+74. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+75. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+76. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+77. Click Manage Account,tap,,"mobile.customer.delete.btn"
+78. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+79. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+80. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+81. Switch To Web Session,switch_to,web,
+82. Click Customer Menu,click,,"admin.menu.customer_icon"
+83. Click Customer DropDown,click,,"admin.menu.customer_icon"
+84. Click Delete Customer,click,,"admin.menu.customer_deleted"
+85. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+86. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"</t>
   </si>
 </sst>
 </file>
@@ -2288,6 +2590,164 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B31CB41-AC3C-4084-88C1-98C363B7ABCB}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="7"/>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E5A465-4C2B-4523-8755-30CE3021A8BD}">
   <dimension ref="A1:H3"/>
@@ -2767,24 +3227,25 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437C624E-95B4-48EB-A315-8931C834404A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -2800,42 +3261,135 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>51</v>
+        <v>68</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+      <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D250DB7C-844B-4BAE-BD85-886B660DFD66}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
84th Commit: Customer Language Check and SuperAdmin Transport Tests Added
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5ECF3CE-1044-4887-BB76-7766BB729DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F198C7-8137-4687-9FE2-30D186D66542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="84">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -242,9 +242,6 @@
   </si>
   <si>
     <t>Validate that the admin can successfully add a new Auto driver by entering valid driver details and vehicle details and approve him from pendind documents by adding documents and verify he is coming in on approved drivers list .</t>
-  </si>
-  <si>
-    <t>Auto Ride Complete Life Cycle Test</t>
   </si>
   <si>
     <t>This comprehensive end-to-end hybrid test validates the multi-platform orchestration and transactional workflow of the ABCD Framework by simulating a complete ride lifecycle across Web Admin, Driver, and User contexts. The execution flows sequentially from the Web Admin portal to register a new auto driver, switches to the Appium-driven Driver App to submit verification documents, and transitions back to Web Admin for regulatory approval and onboarding. The test then establishes parallel operations, shifting to the Driver App to go online, moving to the User App to dynamically book a ride, routing back to the Driver App to accept and complete the trip, and concludes with payment processing, data lifecycle validation, and transactional integrity verification across all application touchpoints.</t>
@@ -604,9 +601,6 @@
     <t>Add Customer For Hybrid Testing</t>
   </si>
   <si>
-    <t>TC_CA_01_Hybrid_Add_Customer</t>
-  </si>
-  <si>
     <t>Validate the end-to-end creation of a Customer to login for user app.</t>
   </si>
   <si>
@@ -620,15 +614,6 @@
   </si>
   <si>
     <t>SA_TS_02</t>
-  </si>
-  <si>
-    <t>TC_CA_02_Hybrid_Unapproved_Auto_Driver</t>
-  </si>
-  <si>
-    <t>TC_CA_03_Hybrid_Approved_Auto_Driver</t>
-  </si>
-  <si>
-    <t>TC_CA_04_Hybrid_Subscription_Plan_Test</t>
   </si>
   <si>
     <r>
@@ -820,13 +805,7 @@
     <t xml:space="preserve">Auto Ride Complete Life Cycle Test </t>
   </si>
   <si>
-    <t>TC_CA_05_Autoride_Complete_Test</t>
-  </si>
-  <si>
     <t>SA_TS_06</t>
-  </si>
-  <si>
-    <t>TC_CA_06_test_data_cleanup</t>
   </si>
   <si>
     <t>1.Click Dashboard Icon,click,,"web.global.menu.dashboard"
@@ -891,9 +870,6 @@
 9. Click Login,click,,"web.global.login.submit_btn"
 10.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
 </t>
-  </si>
-  <si>
-    <t>TC_CA_06_Driver_App_Wallet_Verification</t>
   </si>
   <si>
     <r>
@@ -1746,129 +1722,182 @@
 75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"</t>
   </si>
   <si>
+    <t>SA_TS_07</t>
+  </si>
+  <si>
+    <t>Non Verified Customer</t>
+  </si>
+  <si>
+    <t>Customer Language Check</t>
+  </si>
+  <si>
+    <t>Driver Language Check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17. Click Customer Menu,click,,"admin.menu.customer_icon"
+18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+25. Select Male Gender,click,,"admin.customer.select_gender_male"
+26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+27. Wait for Toast to Hide,wait,3000,,
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+30. Click Customer Menu,click,,"admin.menu.customer_icon"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+33.Wait For Customer Filter,wait,3000,
+34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+35.Wait For Customer,wait,2000,
+36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+37. Load User App,switch_to,user,
+38. Reload User App Completely,reload_app,user,
+39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+42. Click Next,tap,,"mobile.customer.next.btn"
+43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+44. Click Close,tap,,"mobile.customer.cancel.btn"
+45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+46. Click Continue,tap,,"mobile.customer.continue.btn"
+47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+48. Click Finish,tap,,"mobile.customer.finish.btn"
+49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+52.Wait For Profile,wait,5000,
+53. Click Profile,tap_coordinate,558:405,COORDINATE_MODE
+54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
+55.Click Back,tap,,"mobile.customer.back.btn"
+56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+57. Drag Page Layout Upward,swipe,up,
+58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+61. Click Manage Account,tap,,"mobile.customer.delete.btn"
+62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+65. Switch To Web Session,switch_to,web,
+66. Click Customer Menu,click,,"admin.menu.customer_icon"
+67. Click Customer DropDown,click,,"admin.menu.customer_icon"
+68. Click Delete Customer,click,,"admin.menu.customer_deleted"
+69. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+70. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"
+</t>
+  </si>
+  <si>
     <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
-3.Load Super Admin,switch_to,web,
-4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-5.Click Subscription Plan,click,,"admin.subscription.menu_link"
-6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
-8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
-9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
-11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
-12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
-14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
-15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
-16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
-17.Enter Price, type,5000, "admin.subscription.common.price.input"
-18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
-19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
-20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
-21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
-22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-23.Select On,click,,"admin.subscription.common.status.option_on"
-24.Click Submit ,click,,"web.global.action.submit"
-25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-26.Click badge,click,,"admin.subscription.badge.icon"
-27.Click Subscription Plan,click,,"admin.subscription.menu_link"
-28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
-30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
-31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-32.Select Pest Control,click,,"admin.subscription.common.category.option_pest"
-33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
-34.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-35.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
-36.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
-37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
-38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
-39.Enter Price, type,5000, "admin.subscription.common.price.input"
-40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
-41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
-42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
-43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
-44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-45.Select On,click,,"admin.subscription.common.status.option_on"
-46.Click Submit ,click,,"web.global.action.submit"
-47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-48.Load User App,switch_to,user,
-49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-50.Click Get Started,tap,,"mobile.customer.get_started.btn"
-51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-52.Click Next,tap,,"mobile.customer.next.btn"
-53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-54.Click Close,tap,,"mobile.customer.cancel.btn"
-55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-57.Click Continue,tap,,"mobile.customer.continue.btn"
-58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
-59.Click Finish,tap,,"mobile.customer.finish.btn"
-60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
-62.Click Subscription,tap,,"mobile.customer.subscription.btn"
-63.Wait Customer Plan,wait_until_visible,,"mobile.customer.dynamic_subscription.plan"
-64.Click Customer Plan,tap,,"mobile.customer.dynamic_subscription.plan"
-65.Load Driver App,switch_to,driver,
-66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
-67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-68.Click Agree,tap,,"mobile.driver.agree.btn"
-69.Click Get Started,tap,,"mobile.driver.get_started.btn"
-70.Click Next,tap,,"mobile.driver.next.btn"
-71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-72.Click Close,tap,,"mobile.driver.cancel.btn"
-73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-75.Click Continue,tap,,"mobile.driver.continue.btn"
-76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-79.wait for page load,wait,5000,
-80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-81.wait for page load,wait,5000,
-82.Click Subscription,tap,,"mobile.driver.subscription.btn"
-83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
-84.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
-85.Load Super Admin,switch_to,web,
-86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-87.Click Subscription Plan,click,,"admin.subscription.menu_link"
-88.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-89.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-90.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
-91.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-92.Wait For Deletion,wait,2000,
-93.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-94.Click Subscription Plan,click,,"admin.subscription.menu_link"
-95.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-96.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
-98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-99.Wait For Deletion,wait,2000,</t>
-  </si>
-  <si>
-    <t>SA_TS_07</t>
-  </si>
-  <si>
-    <t>Non Verified Customer</t>
-  </si>
-  <si>
-    <t>SA_TS_09</t>
-  </si>
-  <si>
-    <t>Customer Language Check</t>
-  </si>
-  <si>
-    <t>TC_CA_09_Customer_Language_Check</t>
-  </si>
-  <si>
-    <t>SA_TS_10</t>
-  </si>
-  <si>
-    <t>Driver Language Check</t>
-  </si>
-  <si>
-    <t>TC_CA_10_Driver_Language_Check</t>
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17. Click Customer Menu,click,,"admin.menu.customer_icon"
+18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+25. Select Male Gender,click,,"admin.customer.select_gender_male"
+26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+27. Wait for Toast to Hide,wait,3000,,
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+30. Click Customer Menu,click,,"admin.menu.customer_icon"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+33.Wait For Customer Filter,wait,3000,
+34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+35.Wait For Customer,wait,2000,
+36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+37. Load User App,switch_to,user,
+38. Reload User App Completely,reload_app,user,
+39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+42. Click Next,tap,,"mobile.customer.next.btn"
+43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+44. Click Close,tap,,"mobile.customer.cancel.btn"
+45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+46. Click Continue,tap,,"mobile.customer.continue.btn"
+47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+48. Click Finish,tap,,"mobile.customer.finish.btn"
+49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+52.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+53. Drag Page Layout Upward,swipe,up,
+54. Click Select Language,tap,,"mobile.customer.Language.btn"
+55. Wait for Language Setting option,wait,3000,,
+56. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
+57. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
+58. Wait for Language Setting option,wait,3000,,
+59. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+60. Wait For Page Load,wait,3000,
+61. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
+62. Wait for Language Setting option,wait,3000,,
+63. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
+64. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
+65. Wait for Profile,wait,3000,,
+66. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+67. Wait For Page Load,wait,3000
+68. Click Select Language,tap,,"mobile.customer.Language_menu.Hindi.btn"
+69. Wait for Language Setting option,wait,3000,,
+70. Click Select english Language,tap,,"mobile.customer.Language.English.button"
+71. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
+72. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+73. Drag Page Layout Upward,swipe,up,
+74. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+75. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+76. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+77. Click Manage Account,tap,,"mobile.customer.delete.btn"
+78. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+79. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+80. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+81. Switch To Web Session,switch_to,web,
+82. Click Customer Menu,click,,"admin.menu.customer_icon"
+83. Click Customer DropDown,click,,"admin.menu.customer_icon"
+84. Click Delete Customer,click,,"admin.menu.customer_deleted"
+85. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+86. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"</t>
+  </si>
+  <si>
+    <t>79.Click Language menu,tap,,"mobile.driver.Language.btn"
+86. Click Language menu,tap,,"mobile.driver.Language_menu.Tamil.btn"
+92. Click Language menu,tap,,"mobile.driver.Language_menu.Hindi.btn"</t>
   </si>
   <si>
     <t>1. Reload User App Completely,reload_app,user,
@@ -1944,206 +1973,199 @@
 71. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
 72. Enter OTP,type,123456,"mobile.driver.edit_text.input"
 73. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-74. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-75. Drag Page Layout Upward,swipe,up,
-76. Click Language menu,tap,,"mobile.driver.Language.btn"
-77. Wait for Language Setting option,wait,3000,,
-78. Click Select Tamil Language,tap,,"mobile.driver.Language.Tamil.button"
-79. Click Select Tamil Language Update,tap,,"mobile.driver.update.btn"
+74.Wait For Hamburger Menu,wait,3000
+75. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+76.Wait For Driver Profile Load,wait,3000,
+77. Drag Page Layout Upward,swipe,up,
+78.Wait For Language Menu,wait,3000,
+79. Click Language menu,tap_coordinate,394:1631,COORDINATE_MODE
 80. Wait for Language Setting option,wait,3000,,
-81. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-82. Drag Page Layout Upward,swipe,up,
-83. Click Language menu,tap,,"mobile.driver.Language.btn"
-84. Wait for Language Setting option,wait,3000,,
-85. Click Select Hindi Language,tap,,"mobile.driver.Language.Hindi.button"
-86. Click Select Hindi Language Update,tap,,"mobile.driver.Language.Tamil.update.btn"
-87. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-88. Drag Page Layout Upward,swipe,up,
-89. Click Language menu,tap,,"mobile.driver.Language.btn"
-90. Wait for Language Setting option,wait,3000,,
-91. Click Select Tamil Language,tap,,"mobile.driver.Language.English.button"
-92. Click Select Tamil Language Update,tap,,"mobile.driver.Language.Hindi.update.btn"
-93. Wait for Language Setting option,wait,3000,,
-94. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-95. Drag Page Layout Upward,swipe,up,
-96. Wait for Manage Account Loading,wait,3000,,
-97. Click Manage Account,tap,,"mobile.driver.manage_account.btn"
-98. Click Delete Account,tap,,"mobile.customer.delete_sure.btn"
-99. Click Delete AccountSure,tap,,"mobile.customer.delete_sure.btn"
-100. Switch To Web Session,switch_to,web,
-101. Wait for Menu,wait_until_visible,,"admin.drivers.menu.icon"
-102. Click Driver Menu,click,,"admin.drivers.menu.icon"
-103. Click Driver DropDown,click,,"admin.drivers.menu.icon"
-104. Wait for Agree,wait_until_visible,,"Global.menu.driver_deleted"
-105. Click Delete Driver,click,,"Global.menu.driver_deleted"
-106. Enter Driver Vehicele,type,Pink Auto,"Global.menu.Delete_Driver.Vehicle_Type_Filter" 
-107. scroll grid,tab,4,,”Global.menu.Delete_Driver.Contact_Type_Filter"
-108. Enter Driver Name,type,{autoName},"Global.menu.Delete_Driver.Contact_Type_Filter"
-109. Wait For Delete Driver,wait_until_visible,,"Global.menu.Delete_Driver.Contact_Type_Filter"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
-14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
-16. Switch To Web Session,switch_to,web,
-17. Click Customer Menu,click,,"admin.menu.customer_icon"
-18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
-19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
-20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
-21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
-22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
-24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
-25. Select Male Gender,click,,"admin.customer.select_gender_male"
-26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-27. Wait for Toast to Hide,wait,3000,,
-28. Click Submit Button,click,,"web.global.action.submit"
-29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
-30. Click Customer Menu,click,,"admin.menu.customer_icon"
-31. Click Customer Menu,click,,"admin.menu.customer_icon"
-32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-33.Wait For Customer Filter,wait,3000,
-34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-35.Wait For Customer,wait,2000,
-36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-37. Load User App,switch_to,user,
-38. Reload User App Completely,reload_app,user,
-39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
-41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
-42. Click Next,tap,,"mobile.customer.next.btn"
-43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-44. Click Close,tap,,"mobile.customer.cancel.btn"
-45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
-46. Click Continue,tap,,"mobile.customer.continue.btn"
-47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-48. Click Finish,tap,,"mobile.customer.finish.btn"
-49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
-52.Wait For Profile,wait,5000,
-53. Click Profile,tap_coordinate,558:405,COORDINATE_MODE
-54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
-55.Click Back,tap,,"mobile.customer.back.btn"
-56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-57. Drag Page Layout Upward,swipe,up,
-58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
-61. Click Manage Account,tap,,"mobile.customer.delete.btn"
-62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
-63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
-64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
-65. Switch To Web Session,switch_to,web,
-66. Click Customer Menu,click,,"admin.menu.customer_icon"
-67. Click Customer DropDown,click,,"admin.menu.customer_icon"
-68. Click Delete Customer,click,,"admin.menu.customer_deleted"
-69. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-70. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"
-</t>
-  </si>
-  <si>
-    <t>TC_CA_07_Non_Verified_And_Deleted_Customer</t>
+81. Click Select Tamil Language,tap,,"mobile.driver.Language.Tamil.button"
+82. Click Select Tamil Language Update,tap,,"mobile.driver.menu.Language.save_changes.btn"
+83. Wait for Language Setting option,wait,3000,,
+84. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+85. Drag Page Layout Upward,swipe,up,
+86.Wait For Page Load,wait,3000,
+87. Click Language menu,tap_coordinate,394:1631,COORDINATE_MODE
+88. Wait for Language Setting option,wait,3000,,
+89. Click Select Hindi Language,tap,,"mobile.driver.Language.Hindi.button"
+90. Click Select Hindi Language Update,tap,,"mobile.driver.menu.Language_Tamil.save_changes.btn"
+91. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+92. Drag Page Layout Upward,swipe,up,
+93.Wait For Page Load,wait,3000,
+94. Click Language menu,tap_coordinate,394:1631,COORDINATE_MODE
+95. Wait for Language Setting option,wait,3000,,
+96. Click Select English Language,tap,,"mobile.driver.Language.English.button"
+97. Click Select English Language Update,tap,,"mobile.driver.menu.Language_Hindi.save_changes.btn"
+98. Wait for Language Setting option,wait,3000,,
+99. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+100. Drag Page Layout Upward,swipe,up,
+101. Wait for Manage Account Loading,wait,3000,,
+102. Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+103. Click Delete Account,tap,,"mobile.driver.delete.btn"
+104. Click Delete Account Sure,tap,,"mobile.driver.delete_sure.btn"
+105. Switch To Web Session,switch_to,web,
+106. Wait for Menu,wait_until_visible,,"admin.drivers.menu.icon"
+107. Click Driver Menu,click,,"admin.drivers.menu.icon"
+108. Click Driver DropDown,click,,"admin.drivers.menu.icon"
+109. Wait for Agree,wait_until_visible,,"Global.menu.driver_deleted"
+110. Click Delete Driver,click,,"Global.menu.driver_deleted"
+111. Enter Driver Vehicele,type,Pink Auto,"Global.menu.Delete_Driver.Vehicle_Type_Filter" 
+112. scroll grid,tab,4,,”Global.menu.Delete_Driver.Contact_Type_Filter"
+113. Enter Driver Name,type,{autoName},"Global.menu.Delete_Driver.Contact_Type_Filter"
+114. Wait For Delete Driver,wait_until_visible,,"Global.menu.Delete_Driver.Contact_Type_Filter"</t>
+  </si>
+  <si>
+    <t>SA_TS_0A</t>
+  </si>
+  <si>
+    <t>TC_CA_0A_Hybrid_Add_Customer</t>
+  </si>
+  <si>
+    <t>SA_TS_0B</t>
+  </si>
+  <si>
+    <t>TC_CA_0B_Hybrid_Unapproved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>SA_TS_0D</t>
+  </si>
+  <si>
+    <t>TC_CA_0D_Hybrid_Approved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>TC_CA_01_Hybrid_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>Subscriptin Plan Complete Test</t>
+  </si>
+  <si>
+    <t>TC_CA_02_Autoride_Complete_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_03_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <t>TC_CA_04_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>This comprehensive, cross-platform regression test suite validates the entire lifecycle of a customer account by seamlessly orchestrating actions between native mobile applications and the centralized web administration portal. The test sequence begins by initializing a fresh mobile session using the reload_app utility, executing a new user registration flow via dynamic device permissions, randomized phone generation, and OTP simulation. The execution then seamlessly switches context to the web portal to locate the newly created profile under the Non-Verified Customers matrix, populates missing metadata (including automated profile image uploads and randomized alpha naming strings), and submits the profile to trigger status escalation. After confirming the user's migration into the Verified Customers data grid, the execution switches back to the mobile application instance to verify verified account access. Finally, the test validates data-compliance workflows by triggering a native Delete Account chain from the mobile device settings and cross-verifying that the user profile is immediately and correctly relocated to the web admin’s Deleted Customers repository.</t>
+  </si>
+  <si>
+    <t>TC_CA_05_Customer_Language_Check</t>
+  </si>
+  <si>
+    <t>This comprehensive, cross-platform regression test suite validates the customer onboarding lifecycle, profile verification, and dynamic UI localization capabilities across both native mobile environments and the centralized web admin portal. The script begins by orchestrating an initial mobile registration and OTP verification sequence, shifts context to the web portal to escalate the profile from the Non-Verified Customers grid to the Verified Customers list via metadata injection and profile image uploads, and logs back into the mobile app to verify access. It then comprehensively audits the localization subsystem by performing sequential runtime dialect switches—transitioning the interface dynamically from English to Tamil, Tamil to Hindi, and back to English—while verifying that language save triggers update the UI element bounds properly without memory leaks. Finally, the suite executes a clean teardown flow by triggering a native Delete Account action from the mobile settings drawer and cross-verifying that the profile records are accurately reassigned to the web admin's Deleted Customers master repository.</t>
+  </si>
+  <si>
+    <t>TC_CA_06_Driver_Language_Check</t>
+  </si>
+  <si>
+    <t>This end-to-end, cross-platform regression test suite orchestrates a complex testing lifecycle for driver management by coordinating operations between the central web administration portal and native mobile driver application runtimes. The execution flow begins by initializing clean device environments using the reload_app keyword and shifts context to the web portal to register a new driver profile with comprehensive metadata mapping—including automated profile picture uploads, customized vehicle specifications ("Pink Auto"), and corporate banking infrastructure parameters. The test then executes a multi-tiered regulatory validation pipeline by locating the profile in the Pending Documents grid, uploading a simulated driving license file with an active expiry date, and escalating the profile to the official Approved Drivers registry. Transitioning into the native mobile engine environment, the suite authenticates the newly approved driver using dynamic OTP routing, processes specialized compliance checkboxes, and thoroughly audits the application's localization subsystem by executing dynamic runtime language shifts—transitioning the interface seamlessly from English to Tamil, Tamil to Hindi, and back to English. Finally, the suite tests legal compliance and lifecycle termination rules by triggering a native Delete Account flow from the driver app interface and verifying that the record instantly relocates to the web admin's Deleted Drivers repository under localized filtering conditions.</t>
+  </si>
+  <si>
+    <t>TC_CA_07_test_data_cleanup</t>
   </si>
   <si>
     <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
-14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
-16. Switch To Web Session,switch_to,web,
-17. Click Customer Menu,click,,"admin.menu.customer_icon"
-18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
-19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
-20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
-21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
-22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
-24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
-25. Select Male Gender,click,,"admin.customer.select_gender_male"
-26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-27. Wait for Toast to Hide,wait,3000,,
-28. Click Submit Button,click,,"web.global.action.submit"
-29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
-30. Click Customer Menu,click,,"admin.menu.customer_icon"
-31. Click Customer Menu,click,,"admin.menu.customer_icon"
-32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-33.Wait For Customer Filter,wait,3000,
-34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-35.Wait For Customer,wait,2000,
-36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-37. Load User App,switch_to,user,
-38. Reload User App Completely,reload_app,user,
-39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
-41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
-42. Click Next,tap,,"mobile.customer.next.btn"
-43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-44. Click Close,tap,,"mobile.customer.cancel.btn"
-45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
-46. Click Continue,tap,,"mobile.customer.continue.btn"
-47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-48. Click Finish,tap,,"mobile.customer.finish.btn"
-49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
-52.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-53. Drag Page Layout Upward,swipe,up,
-54. Click Select Language,tap,,"mobile.customer.Language.btn"
-55. Wait for Language Setting option,wait,3000,,
-56. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
-57. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
-58. Wait for Language Setting option,wait,3000,,
-59. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-60. Drag Page Layout Upward,swipe,up,
-61. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
-62. Wait for Language Setting option,wait,3000,,
-63. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
-64. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
-65. Wait for Language Setting option,wait,3000,,
-66. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-67. Drag Page Layout Upward,swipe,up,
-68. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
-69. Wait for Language Setting option,wait,3000,,
-70. Click Select english Language,tap,,"mobile.customer.Language.English.button"
-71. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
-72. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-73. Drag Page Layout Upward,swipe,up,
-74. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-75. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-76. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
-77. Click Manage Account,tap,,"mobile.customer.delete.btn"
-78. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
-79. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
-80. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
-81. Switch To Web Session,switch_to,web,
-82. Click Customer Menu,click,,"admin.menu.customer_icon"
-83. Click Customer DropDown,click,,"admin.menu.customer_icon"
-84. Click Delete Customer,click,,"admin.menu.customer_deleted"
-85. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-86. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"</t>
+3.Load Super Admin,switch_to,web,
+4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5.Click Subscription Plan,click,,"admin.subscription.menu_link"
+6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
+8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
+9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
+12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
+14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
+15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
+16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
+17.Enter Price, type,5000, "admin.subscription.common.price.input"
+18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
+19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
+20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
+21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
+22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+23.Select On,click,,"admin.subscription.common.status.option_on"
+24.Click Submit ,click,,"web.global.action.submit"
+25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+26.Click badge,click,,"admin.subscription.badge.icon"
+27.Click Subscription Plan,click,,"admin.subscription.menu_link"
+28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
+30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+32.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
+34.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+35.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+36.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
+39.Enter Price, type,5000, "admin.subscription.common.price.input"
+40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
+41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
+42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
+43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
+44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+45.Select On,click,,"admin.subscription.common.status.option_on"
+46.Click Submit ,click,,"web.global.action.submit"
+47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+48.Load User App,switch_to,user,
+49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+50.Click Get Started,tap,,"mobile.customer.get_started.btn"
+51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+52.Click Next,tap,,"mobile.customer.next.btn"
+53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+54.Click Close,tap,,"mobile.customer.cancel.btn"
+55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+57.Click Continue,tap,,"mobile.customer.continue.btn"
+58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+59.Click Finish,tap,,"mobile.customer.finish.btn"
+60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+62.Click Subscription,tap,,"mobile.customer.subscription.btn"
+63.Wait Customer Plan,wait_until_visible,,"mobile.customer.dynamic_subscription.plan"
+64.Click Customer Plan,tap,,"mobile.customer.dynamic_subscription.plan"
+65.Load Driver App,switch_to,driver,
+66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
+67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+68.Click Agree,tap,,"mobile.driver.agree.btn"
+69.Click Get Started,tap,,"mobile.driver.get_started.btn"
+70.Click Next,tap,,"mobile.driver.next.btn"
+71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+72.Click Close,tap,,"mobile.driver.cancel.btn"
+73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+75.Click Continue,tap,,"mobile.driver.continue.btn"
+76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+79.wait for page load,wait,5000,
+80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+81.wait for page load,wait,5000,
+82.Click Subscription,tap,,"mobile.driver.subscription.btn"
+83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+84.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
+85.Load Super Admin,switch_to,web,
+86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+87.Click Subscription Plan,click,,"admin.subscription.menu_link"
+88.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+89.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+90.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
+91.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+92.Wait For Deletion,wait,2000,
+93.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+94.Click Subscription Plan,click,,"admin.subscription.menu_link"
+95.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+96.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
+98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+99.Wait For Deletion,wait,2000,</t>
   </si>
 </sst>
 </file>
@@ -2557,22 +2579,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2625,37 +2647,35 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -2663,7 +2683,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -2716,13 +2736,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>
@@ -2783,7 +2803,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -2791,25 +2811,25 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2861,7 +2881,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -2869,25 +2889,25 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2944,22 +2964,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3009,36 +3029,36 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3047,7 +3067,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -3093,36 +3113,36 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3131,7 +3151,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -3177,36 +3197,36 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3215,7 +3235,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -3261,36 +3281,36 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3299,7 +3319,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -3345,36 +3365,36 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3383,7 +3403,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>

</xml_diff>

<commit_message>
88th Commit: Hover Keyword Added In ABCD Framwork For Element Hovering
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D0F3CD-37E1-4054-B8E3-45FFC72A06DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F20D60A-A21C-4341-8B9F-43BDF7D103B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -1820,107 +1820,6 @@
     <t>TC_CA_04_Autoride_Complete_Test</t>
   </si>
   <si>
-    <t>1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3.Load Super Admin,switch_to,web,
-4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-5.Click Subscription Plan,click,,"admin.subscription.menu_link"
-6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
-8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
-9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
-11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
-12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
-14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
-15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
-16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
-17.Enter Price, type,5000, "admin.subscription.common.price.input"
-18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
-19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
-20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
-21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
-22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-23.Select On,click,,"admin.subscription.common.status.option_on"
-24.Click Submit ,click,,"web.global.action.submit"
-25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-26.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-27.Click Subscription Plan,click,,"admin.subscription.menu_link"
-28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
-30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
-31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-32.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
-33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
-34.Enter Customer Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-35.Enter Customer Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
-36.Enter Customer Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
-37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
-38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
-39.Enter Price, type,5000, "admin.subscription.common.price.input"
-40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
-41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
-42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
-43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
-44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-45.Select On,click,,"admin.subscription.common.status.option_on"
-46.Click Submit ,click,,"web.global.action.submit"
-47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-48.Load User App,switch_to,user,
-49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-50.Click Get Started,tap,,"mobile.customer.get_started.btn"
-51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-52.Click Next,tap,,"mobile.customer.next.btn"
-53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-54.Click Close,tap,,"mobile.customer.cancel.btn"
-55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-57.Click Continue,tap,,"mobile.customer.continue.btn"
-58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
-59.Click Finish,tap,,"mobile.customer.finish.btn"
-60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
-62.Click Subscription,tap,,"mobile.customer.subscription.btn"
-63.Wait Customer Plan,wait_until_visible,,"mobile.customer.dynamic_subscription.plan"
-64.Click Customer Plan,tap,,"mobile.customer.dynamic_subscription.plan"
-65.Load Driver App,switch_to,driver,
-66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
-67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-68.Click Agree,tap,,"mobile.driver.agree.btn"
-69.Click Get Started,tap,,"mobile.driver.get_started.btn"
-70.Click Next,tap,,"mobile.driver.next.btn"
-71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-72.Click Close,tap,,"mobile.driver.cancel.btn"
-73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-75.Click Continue,tap,,"mobile.driver.continue.btn"
-76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-79.wait for page load,wait,5000,
-80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-81.wait for page load,wait,5000,
-82.Click Subscription,tap,,"mobile.driver.subscription.btn"
-83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
-84.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
-85.Load Super Admin,switch_to,web,
-86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-87.Click Subscription Plan,click,,"admin.subscription.menu_link"
-88.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-89.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-90.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
-91.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-92.Wait For Deletion,wait,2000,
-93.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-94.Click Subscription Plan,click,,"admin.subscription.menu_link"
-95.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-96.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
-98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-99.Wait For Deletion,wait,2000,</t>
-  </si>
-  <si>
     <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3.Load Driver App,switch_to,driver,
@@ -2170,6 +2069,107 @@
 86.Wait For Delete Cusotmer,wait,3000,
 86. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
 87. Wait For Delete Cusotmer,wait,3000,</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Super Admin,switch_to,web,
+4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5.Click Subscription Plan,click,,"admin.subscription.menu_link"
+6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
+8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
+9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
+12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
+14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
+15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
+16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
+17.Enter Price, type,5000, "admin.subscription.common.price.input"
+18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
+19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
+20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
+21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
+22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+23.Select On,click,,"admin.subscription.common.status.option_on"
+24.Click Submit ,click,,"web.global.action.submit"
+25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+26.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+27.Click Subscription Plan,click,,"admin.subscription.menu_link"
+28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
+30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+32.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
+34.Enter Customer Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+35.Enter Customer Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+36.Enter Customer Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
+39.Enter Price, type,5000, "admin.subscription.common.price.input"
+40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
+41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
+42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
+43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
+44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+45.Select On,click,,"admin.subscription.common.status.option_on"
+46.Click Submit ,click,,"web.global.action.submit"
+47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+48.Load User App,switch_to,user,
+49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+50.Click Get Started,tap,,"mobile.customer.get_started.btn"
+51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+52.Click Next,tap,,"mobile.customer.next.btn"
+53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+54.Click Close,tap,,"mobile.customer.cancel.btn"
+55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+57.Click Continue,tap,,"mobile.customer.continue.btn"
+58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+59.Click Finish,tap,,"mobile.customer.finish.btn"
+60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+62.Click Subscription,tap_if_present,,"mobile.customer.subscription.btn"
+63.Wait Customer Plan,wait_if_present,,"mobile.customer.dynamic_subscription.plan"
+64.Click Customer Plan,tap_if_present,,"mobile.customer.dynamic_subscription.plan"
+65.Load Driver App,switch_to,driver,
+66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
+67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+68.Click Agree,tap,,"mobile.driver.agree.btn"
+69.Click Get Started,tap,,"mobile.driver.get_started.btn"
+70.Click Next,tap,,"mobile.driver.next.btn"
+71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+72.Click Close,tap,,"mobile.driver.cancel.btn"
+73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+75.Click Continue,tap,,"mobile.driver.continue.btn"
+76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+79.wait for page load,wait,5000,
+80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+81.wait for page load,wait,5000,
+82.Click Subscription,tap,,"mobile.driver.subscription.btn"
+83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+84.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
+85.Load Super Admin,switch_to,web,
+86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+87.Click Subscription Plan,click,,"admin.subscription.menu_link"
+88.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+89.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+90.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
+91.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+92.Wait For Deletion,wait,2000,
+93.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+94.Click Subscription Plan,click,,"admin.subscription.menu_link"
+95.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+96.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
+98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+99.Wait For Deletion,wait,2000,</t>
   </si>
 </sst>
 </file>
@@ -3053,7 +3053,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>52</v>
@@ -3221,7 +3221,7 @@
         <v>71</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -3305,7 +3305,7 @@
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -3389,7 +3389,7 @@
         <v>73</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
Draw Polygon And Variable Data Comparing Keyword Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89234CCC-3091-490C-BA71-9CAB72755CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828ED715-67AD-4306-9110-259869EB71C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -22,12 +22,14 @@
     <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId7"/>
     <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId8"/>
     <sheet name="RideCustomerReportIssue" sheetId="58" r:id="rId9"/>
-    <sheet name="AutoRideTestOtpUi" sheetId="57" r:id="rId10"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
-    <sheet name="AutoRideTestOtpDb" sheetId="54" r:id="rId12"/>
-    <sheet name="HybridAddCustomer" sheetId="44" r:id="rId13"/>
-    <sheet name="HybridUnApprovedAutoDriver" sheetId="46" r:id="rId14"/>
-    <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId15"/>
+    <sheet name="GeoFencingVerification" sheetId="59" r:id="rId10"/>
+    <sheet name="AutoRideTestOtpUi" sheetId="57" r:id="rId11"/>
+    <sheet name="DriverRegistrationMobileApp" sheetId="60" r:id="rId12"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId13"/>
+    <sheet name="AutoRideTestOtpDb" sheetId="54" r:id="rId14"/>
+    <sheet name="HybridAddCustomer" sheetId="44" r:id="rId15"/>
+    <sheet name="HybridUnApprovedAutoDriver" sheetId="46" r:id="rId16"/>
+    <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId17"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="115">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1344,11 +1346,6 @@
     <t>Driver Language Check</t>
   </si>
   <si>
-    <t>79.Click Language menu,tap,,"mobile.driver.Language.btn"
-86. Click Language menu,tap,,"mobile.driver.Language_menu.Tamil.btn"
-92. Click Language menu,tap,,"mobile.driver.Language_menu.Hindi.btn"</t>
-  </si>
-  <si>
     <t>SA_TS_0A</t>
   </si>
   <si>
@@ -1972,100 +1969,6 @@
     <t>TC_CA_07_Driver_Language_Check</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3.Load Driver App,switch_to,driver,
-4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-6.Click Agree,tap,,"mobile.driver.agree.btn"
-7.Click Get Started,tap,,"mobile.driver.get_started.btn"
-8.Click Next,tap,,"mobile.driver.next.btn"
-9.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-10.Click Close,tap,,"mobile.driver.cancel.btn"
-11.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-12.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-13 Click Continue,tap,,"mobile.driver.continue.btn"
-14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-15.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-16.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-17.Wait For Pageload,wait,3000,
-18.Click Online Toggle,tap_coordinate,982:1932,
-19.Load User App,switch_to,user,
-20.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-21.Click Get Started,tap,,"mobile.customer.get_started.btn"
-22.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-23.Click Next,tap,,"mobile.customer.next.btn"
-24.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-25.Click Close,tap,,"mobile.customer.cancel.btn"
-26.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-27.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-28. Click Continue,tap,,"mobile.customer.continue.btn"
-29. Enter OTP,type,123456,"mobile.customer.otp_input"
-30. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-31. Click Finish,tap,,"mobile.customer.finish.btn"
-32. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-33. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
-34. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
-35. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
-36. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
-37. Select Destination,tap,,"mobile.customer.destination_suggestion_first"
-38.Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
-39.Click Entrance,tap,,"mobile.customer.destination_entrance_location"
-40. Click Confirm,tap,,"mobile.customer.confirm.btn"
-41.Wait For Ride,wait,5000,
-42. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
-43. Ride Now,tap,,"mobile.customer.ride_now.btn"
-44. Load Driver App,switch_to,driver,
-45.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
-46.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
-47.Load User App,switch_to,user,
-48.Wait for OTP Layout to Load,wait_until_visible,,"mobile.customer.otp_display_element"
-49.Extract OTP from Screen,store_text,ride_otp,"mobile.customer.otp_display_element"
-50.Load Driver App,switch_to,driver,
-51.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
-52.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-53.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-54.Ride Arrived,tap,,"mobile.driver.arrived.btn"
-55.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-56.Yes Arrived,tap,,"mobile.driver.yes.btn"
-57.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
-58.Start Ride,tap,,"mobile.driver.start_ride.btn"
-59.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
-60.Enter  Extracted OTP,type,{ride_otp},"mobile.driver.otp_view.input"
-61.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
-62.Start Ride Button,tap,,"mobile.driver.start.btn"
-63.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
-64.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
-65.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
-66.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
-67.Load User App,switch_to,user,
-68.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-69.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
-70. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-71. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
-72. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
-73. Give Review,tap,,"mobile.customer.give_review.btn"
-74. Give Rating,tap_coordinate,348:1619,
-75. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
-76.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
-77.Trip Finished,tap,,"mobile.customer.done.btn"
-78. Load Driver App,switch_to,driver,
-79.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
-80.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
-81. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-82. Confirm Payment,tap,,"mobile.driver.yes.btn"
-83.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
-84.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
-85.Wait For Rating,wait,2000,
-86. Give Rating,tap_coordinate,348:1545,
-87. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
-88.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
-89.Click Complete Button,tap,,"mobile.driver.complete.btn"
-90.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
-91.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
-</t>
-  </si>
-  <si>
     <t>Auto Ride Complete Life Cycle Test With Otp Fetched From DB</t>
   </si>
   <si>
@@ -2073,71 +1976,6 @@
   </si>
   <si>
     <t>SA_TS_10</t>
-  </si>
-  <si>
-    <t>TC_CA_10_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>1.Load User App,switch_to,user,
-2.Reload User App Completely,reload_app,user,
-3.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-4. Load Super Admin,switch_to,web,
-5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
-6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-7. Click Settings Menu,click,,"web.global.menu.settings"
-8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-10.Wait For On,wait,2000,
-11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
-12. Click Submit Button,click,,"web.global.action.submit"
-13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-14. Load User App,switch_to,user,
-15.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-16.Click Get Started,tap,,"mobile.customer.get_started.btn"
-17.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-18.Click Next,tap,,"mobile.customer.next.btn"
-19.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-20.Click Close,tap,,"mobile.customer.cancel.btn"
-21.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-22.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-23.Click Continue,tap,,"mobile.customer.continue.btn"
-24.Enter OTP,type,123456,"mobile.customer.otp_input"
-25.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-26.Click Finish,tap,,"mobile.customer.finish.btn"
-27.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-28. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
-29. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
-30.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-31.wait for Wallet,wait_until_visible,"mobile.customer.wallet.btn"
-32.Check Wallet Present,element_present,,"mobile.customer.wallet.btn"
-33.Reload User App Completely,reload_app,user,
-34. Switch To Web Session,switch_to,web,
-35.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-36. Click Settings Menu,click,,"admin.setting.sidebar.menu"
-37. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-38. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-39.Wait For off,wait,2000,
-40. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
-41. Click Submit Button,click,,"web.global.action.submit"
-42. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-43. Load User App,switch_to,user,
-44.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-45.Click Get Started,tap,,"mobile.customer.get_started.btn"
-46.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-47.Click Next,tap,,"mobile.customer.next.btn"
-48.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-49.Click Close,tap,,"mobile.customer.cancel.btn"
-50.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-51.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-52.Click Continue,tap,,"mobile.customer.continue.btn"
-53.Enter OTP,type,123456,"mobile.customer.otp_input"
-54.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-55.Click Finish,tap,,"mobile.customer.finish.btn"
-56.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-57. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
-58. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
-59.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-60.Check Wallet absent,element_absent,,"mobile.customer.wallet.btn"</t>
   </si>
   <si>
     <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
@@ -2305,48 +2143,6 @@
 </t>
   </si>
   <si>
-    <t>1. Reload User App Completely,reload_app,user,
-2. Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.otp_input"
-14. Enter OTP,type,123456,"mobile.customer.otp_input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.register_customer.name"
-16. Enter Customer Name,type,customer{randomAlpha}&gt;&gt;customerName,"mobile.customer.register_customer.name"
-17. Enter Customer Email,type,customer{timestamp}@gmail.com&gt;&gt;customerEmail,"mobile.customer.register_customer.email"
-18. Select gender male,tap,,"mobile.customer.register_customer.gender.female"
-19. Click the checkbox,tap,,"mobile.customer.register_customer.checkbox"
-20. Click sign_up button,tap,,"mobile.customer.register_customer.sign_up"
-21 Click the while using the app,tap,,"mobile.customer.location_allow.btn"
-22. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
-23. Click Emergency Contact,tap,,"mobile.customer.menu.Emergency"
-24. Click Add Emergency Contact,tap,,"mobile.customer.menu.Emergency.Emergency_Add_Number"
-25. Enter Emergency Number,type,{randomPhone}&gt;&gt;emergencyPhone,"mobile.customer.menu.Emergency.Emergency_Number_Field"
-26. Click update button in profile,tap,,"mobile.customer.menu.profile_edit.update"
-27. Click Back button in profile,tap,,"mobile.customer.back.btn"
-28. Wait For Emergency Call Button,wait_until_visible,,"mobile.customer.menu.emergency.Emergency_call"
-29. Click Emergency Call Button,tap,,"mobile.customer.menu.emergency.Emergency_call"
-30. Switch To Web Session,switch_to,web,
-31. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-32. Click Customer Icon,click,,"admin.menu.customer_icon"
-33. Click Verified Customers,click,,"admin.menu.verified_customers"
-34. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
-35. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
-36. Scroll Grid,tab,7,"admin.customer.filter_name"
-37. Click Pencil Button,click,,"admin.customer.pencil_edit.btn"
-38.Wait For Popup,wait,1000,
-39.Verify Emergeny Number Matches,verify,{emergencyPhone},"admin.customer.input_Emergency_phone"
-40.Wait For Emergency Number,wait,3000,</t>
-  </si>
-  <si>
     <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3. Load User App,switch_to,user,
@@ -2527,6 +2323,39 @@
 85.Wait For Resolved Issue To Load,wait,5000,</t>
   </si>
   <si>
+    <t>TC_CA_0A_Autoride_Test_Otp_DB</t>
+  </si>
+  <si>
+    <t>TC_CA_0B_Hybrid_Add_Customer</t>
+  </si>
+  <si>
+    <t>TC_CA_0C_Hybrid_Unapproved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>SA_TS_0D</t>
+  </si>
+  <si>
+    <t>TC_CA_0D_Hybrid_Approved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Completed_Ride_Customer_Report_Issue</t>
+  </si>
+  <si>
+    <t>SA_TS_11</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Geo_Fencing_Verification</t>
+  </si>
+  <si>
+    <t>TC_CA_10_Autoride_Test_Otp_Ui</t>
+  </si>
+  <si>
+    <t>This test case validates the platform's ability to enforce active geo-fencing restrictions by automatically blocking mobile ride requests initiated from within a prohibited geographical zone. The automated workflow begins in the web administration panel, where the draw_polygon keyword is used to map and activate a restricted area around "Officers Training Academy Chennai." Execution then switches to the native Driver and Customer mobile applications sequentially, utilizing the set_location keyword to inject matching restricted GPS coordinates into both emulator sessions mid-execution. The test concludes by attempting to book an active ride from the customer application and executing a final timeout validation to confirm that the platform successfully intercepts and blocks the order request due to the active boundary constraint.</t>
+  </si>
+  <si>
+    <t>35.Click Online Toggle,tap_coordinate,982:1932,</t>
+  </si>
+  <si>
     <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3.Load Super Admin,switch_to,web,
@@ -2591,47 +2420,57 @@
 62.Click Subscription,tap_if_present,,"mobile.customer.subscription.btn"
 63.Wait Customer Plan,wait_if_present,,"mobile.customer.dynamic_subscription.plan"
 64.Click Customer Plan,tap_if_present,,"mobile.customer.dynamic_subscription.plan"
-65.Load Driver App,switch_to,driver,
-66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
-67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-68.Click Agree,tap,,"mobile.driver.agree.btn"
-69.Click Get Started,tap,,"mobile.driver.get_started.btn"
-70.Click Next,tap,,"mobile.driver.next.btn"
-71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-72.Click Close,tap,,"mobile.driver.cancel.btn"
-73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-75.Click Continue,tap,,"mobile.driver.continue.btn"
-76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-79.wait for page load,wait,5000,
-80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-81.wait for page load,wait,5000,
-82.Click Subscription,tap,,"mobile.driver.subscription.btn"
-83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
-84.Click Driver Plan,tap_if_present,,"mobile.driver.dynamic_subscription.plan"
-85.Click Pay Button,tap,,"mobile.diver.subscription.pay_btn"
-86.Select Wallet Payment,tap,,"mobile.diver.subscription.select_wallet"
-87.Click Proceed to Pay,tap,,"mobile.diver.subscription.proceed_to_pay"
-88.Wait For Payment,wait,5000,
-89.Cancel Subscription,tap_coordinate ,971:362,COORDINATE_MODE
-90.Confirm Cancel Subscrption,tap,,"mobile.diver.subscription.confirm_cancel_subscription"
-88.Load Super Admin,switch_to,web,
-89.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-90.Click Subscription Plan,click,,"admin.subscription.menu_link"
-91.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-92.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-93.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
-94.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-95.Wait For Deletion,wait,2000,
-96.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-97.Click Subscription Plan,click,,"admin.subscription.menu_link"
-98.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-99.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-100.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
-101.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-102.Wait For Deletion,wait,2000,</t>
+65.Load Super Admin,switch_to,web,
+66.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+67.Click Settings Menu,click,,"web.global.menu.settings"
+68.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+69.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+70.Wait For On,wait,2000,
+71.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+72.Click Submit Button,click,,"web.global.action.submit"
+73.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+74.Wait For Toast To Hide,wait,3000,
+75.Load Driver App,switch_to,driver,
+76.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
+77.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+78.Click Agree,tap,,"mobile.driver.agree.btn"
+79.Click Get Started,tap,,"mobile.driver.get_started.btn"
+80.Click Next,tap,,"mobile.driver.next.btn"
+81.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+82.Click Close,tap,,"mobile.driver.cancel.btn"
+83.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+84.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+85.Click Continue,tap,,"mobile.driver.continue.btn"
+86.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+87.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+88.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+89.wait for page load,wait,5000,
+90.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+91.wait for page load,wait,5000,
+92.Click Subscription,tap,,"mobile.driver.subscription.btn"
+93.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+94.Click Driver Plan,tap_if_present,,"mobile.driver.dynamic_subscription.plan"
+95.Click Pay Button,tap,,"mobile.diver.subscription.pay_btn"
+96.Select Wallet Payment,tap,,"mobile.diver.subscription.select_wallet"
+97.Click Proceed to Pay,tap,,"mobile.diver.subscription.proceed_to_pay"
+98.Wait For Payment,wait,5000,
+99.Cancel Subscription,tap_coordinate ,971:362,COORDINATE_MODE
+100.Confirm Cancel Subscrption,tap,,"mobile.diver.subscription.confirm_cancel_subscription"
+101.Load Super Admin,switch_to,web,
+102.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+103.Click Subscription Plan,click,,"admin.subscription.menu_link"
+104.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+105.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+106.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
+107.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+108.Wait For Deletion,wait,2000,
+109.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+110.Click Subscription Plan,click,,"admin.subscription.menu_link"
+111.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+112.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+113.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
+114.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+115.Wait For Deletion,wait,2000,</t>
   </si>
   <si>
     <t>1. Load Driver App,switch_to,driver,
@@ -2708,28 +2547,648 @@
 72. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
 73.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
 74.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"</t>
-  </si>
-  <si>
-    <t>TC_CA_0A_Autoride_Test_Otp_DB</t>
-  </si>
-  <si>
-    <t>TC_CA_0B_Hybrid_Add_Customer</t>
-  </si>
-  <si>
-    <t>TC_CA_0C_Hybrid_Unapproved_Auto_Driver</t>
-  </si>
-  <si>
-    <t>SA_TS_0D</t>
-  </si>
-  <si>
-    <t>TC_CA_0D_Hybrid_Approved_Auto_Driver</t>
-  </si>
-  <si>
-    <t>TC_CA_08_Completed_Ride_Customer_Report_Issue</t>
-  </si>
-  <si>
-    <t>TC_CA_09_Autoride_Test_Otp_Ui</t>
+75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"
+76.Load Super Admin,switch_to,web,
+77.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+78.Click Settings Menu,click,,"web.global.menu.settings"
+79.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+80.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+81.Wait For On,wait,2000,
+82.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+83.Click Submit Button,click,,"web.global.action.submit"
+84.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+85.Wait For Toast To Hide,wait,3000,</t>
+  </si>
+  <si>
+    <t>1.Load User App,switch_to,user,
+2.Reload User App Completely,reload_app,user,
+3.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load User App,switch_to,user,
+15.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+16.Click Get Started,tap,,"mobile.customer.get_started.btn"
+17.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+18.Click Next,tap,,"mobile.customer.next.btn"
+19.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+20.Click Close,tap,,"mobile.customer.cancel.btn"
+21.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+22.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+23.Click Continue,tap,,"mobile.customer.continue.btn"
+24.Enter OTP,type,123456,"mobile.customer.otp_input"
+25.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+26.Click Finish,tap,,"mobile.customer.finish.btn"
+27.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+28. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+29. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+30.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+31.wait for Wallet,wait_until_visible,"mobile.customer.wallet.btn"
+32.Check Wallet Present,element_present,,"mobile.customer.wallet.btn"
+33.Reload User App Completely,reload_app,user,
+34. Switch To Web Session,switch_to,web,
+35.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+37. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+38. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+39.Wait For off,wait,2000,
+40. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+41. Click Submit Button,click,,"web.global.action.submit"
+42. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+43. Load User App,switch_to,user,
+44.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+45.Click Get Started,tap,,"mobile.customer.get_started.btn"
+46.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+47.Click Next,tap,,"mobile.customer.next.btn"
+48.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+49.Click Close,tap,,"mobile.customer.cancel.btn"
+50.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+51.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+52.Click Continue,tap,,"mobile.customer.continue.btn"
+53.Enter OTP,type,123456,"mobile.customer.otp_input"
+54.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+55.Click Finish,tap,,"mobile.customer.finish.btn"
+56.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+57. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+58. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+59.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+60.Check Wallet absent,element_absent,,"mobile.customer.wallet.btn"
+61.Load Super Admin,switch_to,web,
+62.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+63.Click Settings Menu,click,,"web.global.menu.settings"
+64.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+65.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+66.Wait For On,wait,2000,
+67.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+68.Click Submit Button,click,,"web.global.action.submit"
+69.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+70.Wait For Toast To Hide,wait,3000,</t>
+  </si>
+  <si>
+    <t>1. Load Driver App,switch_to,driver,
+2.Reload Driver App Completely,reload_app,driver,
+3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load Driver App,switch_to,driver,
+15. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+16. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+17. Click Agree,tap,,"mobile.driver.agree.btn"
+18. Click Get Started,tap,,"mobile.driver.get_started.btn"
+19. Click Next,tap,,"mobile.driver.next.btn"
+20. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+21. Click Close,tap,,"mobile.driver.cancel.btn"
+22. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+23. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+24. Click Continue,tap,,"mobile.driver.continue.btn"
+25. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+26. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+27. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+28. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+29.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
+30.Click Wallet,tap,,"mobile.driver.wallet.btn"
+31.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
+32.Click Topup,tap,,"mobile.driver.top_up.btn"
+33.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
+34.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
+35.Click Proceed,tap,,"mobile.driver.top_up.proceed"
+36.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
+37.Enter Driver Mobile,type,regression.approved_driver.phone,"mobile.driver.top_up.contact_no_box"
+38.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
+39.Wait For Net Banking,wait_until_visible,,"mobile.driver.top_up.net_banking"
+40.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
+41.Wait For Bob,wait_until_visible,,"mobile.driver.top_up.bob_bank"
+42.Click Bob,tap,,"mobile.driver.top_up.bob_bank"
+43.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
+44.Click Success,tap,,"mobile.driver.top_up.succes_popup"
+45.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
+46.Click Back,tap,,"mobile.driver.back.btn"
+47.Drag Page Layout Upward,swipe,up,
+48.Click Back,tap,,"mobile.driver.back.btn"
+49.Reload Driver App Completely,reload_app,driver,
+50. Switch To Web Session,switch_to,web,
+51.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+52. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+53. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+54. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+55.Wait For off,wait,2000,
+56. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+57. Click Submit Button,click,,"web.global.action.submit"
+58. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+59. Switch To Driver Session,switch_to,driver,
+60. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+61. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+62. Click Agree,tap,,"mobile.driver.agree.btn"
+63. Click Get Started,tap,,"mobile.driver.get_started.btn"
+64. Click Next,tap,,"mobile.driver.next.btn"
+65. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+66. Click Close,tap,,"mobile.driver.cancel.btn"
+67. Enter Mobile Number,type,regression.approved_driver.phone ,"mobile.driver.edit_text.input"
+68. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+69. Click Continue,tap,,"mobile.driver.continue.btn"
+70. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+71. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+72. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+73.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+74.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"
+76.Load Super Admin,switch_to,web,
+77.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+78.Click Settings Menu,click,,"web.global.menu.settings"
+79.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+80.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+81.Wait For On,wait,2000,
+82.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+83.Click Submit Button,click,,"web.global.action.submit"
+84.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+85.Wait For Toast To Hide,wait,3000,</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.otp_input"
+14. Enter OTP,type,123456,"mobile.customer.otp_input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.register_customer.name"
+16. Enter Customer Name,type,customer{randomAlpha}&gt;&gt;customerName,"mobile.customer.register_customer.name"
+17. Enter Customer Email,type,customer{timestamp}@gmail.com&gt;&gt;customerEmail,"mobile.customer.register_customer.email"
+18. Select gender male,tap,,"mobile.customer.register_customer.gender.female"
+19. Click the checkbox,tap,,"mobile.customer.register_customer.checkbox"
+20. Click sign_up button,tap,,"mobile.customer.register_customer.sign_up"
+21 Click the while using the app,tap,,"mobile.customer.location_allow.btn"
+22.Wait For Profile,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+23. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+24.Swipe Profile Page,swipe,up,
+25.Wait For Page Load,wait,3000,
+26.Click Emergency Contact,tap,,"mobile.customer.menu.Emergency"
+27.Click Add Emergency Contact,tap,,"mobile.customer.menu.Emergency.Emergency_Add_Number"
+28.Enter Emergency Number,type,{randomPhone}&gt;&gt;emergencyPhone,"mobile.customer.menu.Emergency.Emergency_Number_Field"
+29.Click update button in profile,tap,,"mobile.customer.menu.profile_edit.update"
+30.Click Back button in profile,tap,,"mobile.customer.back.btn"
+31.Wait For Emergency Call Button,wait_until_visible,,"mobile.customer.menu.emergency.Emergency_call"
+32.Click Emergency Call Button,tap,,"mobile.customer.menu.emergency.Emergency_call"
+33.Switch To Web Session,switch_to,web,
+34.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+35.Click Customer Icon,click,,"admin.menu.customer_icon"
+36.Click Verified Customers,click,,"admin.menu.verified_customers"
+37.Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+38.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+39.Scroll Grid,tab,7,"admin.customer.filter_name"
+40.Click Pencil Button,click,,"admin.customer.pencil_edit.btn"
+41.Wait For Popup,wait,1000,
+42.Extract Emergency Contact Saved from Screen,store_text,stored_emergency_number,"admin.customer.input_Emergency_phone"
+43.Wait For Extraction,wait,5000,
+44.Verify Emergeny Number Matches,verify_variables_match,emergencyPhone,stored_emergency_number
+45.Wait For Emergency Number,wait,3000,</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3.  Switch To Web Session,switch_to,web,
+4. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5. Click drivers menu,click,,"admin.drivers.menu.icon"
+6. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+7. Verify Add Driver,verify,,"admin.drivers.add_page.header"
+8. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+9. Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+10.Click Driver Type Dropdown,click,,"admin.drivers.driver_type.dropdown"
+11.Select pilot Option,click,,"admin.drivers.driver_type.dropdown_pilot"
+12. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+13. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
+14. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
+15. Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
+16. Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+17. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+18. Select Source,click,,"admin.drivers.source_dropdown.select"
+19. Select Instagram,click,,"admin.drivers.instagram_option.span"
+20. Select Male Gender, click, , "admin.drivers.male_gender.div"
+21. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+22. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+23. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+24. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
+25. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+26. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+27. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+28. Enter Bank Location, type, PARK STREET, "admin.drivers.banklocation.input"
+29. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+30. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
+31. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+32. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+33. Click Submit, click, , "web.global.action.submit"
+34. Verify Driver Added, verify,, "web.global.toast.success"
+35. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click drivers menu,click,,"admin.drivers.menu.icon"
+37. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+38. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+39. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+40. Click Doc Icon,click,,"admin.drivers.docs.icon"
+41. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+42. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+43. Add Driving License,click,,"admin.drivers.docs.edit_icon"
+44. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+45. Enter Expiry Date,set_date,2026-12-12,"admin.drivers.doc_expiry.input"
+46. Click Submit, click, , "web.global.action.submit"
+47. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+48. Click Approve Driver,click,,"admin.drivers.docs.approval"
+49. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+50. Click Dashboard,click,,"web.global.menu.dashboard"
+51. Click drivers menu,click,,"admin.drivers.menu.icon"
+52. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+53. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+54. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+55. Wait For Get_Started,wait_until_visible,,"admin.drivers.name_filter.input"
+56. Load Driver App,switch_to,driver,
+57. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+58. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+59. Click Agree,tap,,"mobile.driver.agree.btn"
+60. Click Get Started,tap,,"mobile.driver.get_started.btn"
+61. Click Next,tap,,"mobile.driver.next.btn"
+62. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+63. Click Close,tap,,"mobile.driver.cancel.btn"
+64. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+65. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+66. Click Continue,tap,,"mobile.driver.continue.btn"
+67. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+68.Enter Account Holder,type,{autoName},"mobile.driver.bank_details.account_holder_name"
+69.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+70.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+71.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+72.Wait For Keyboard Minimises,hide_keyboard,,
+73.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+74.Wait For Keyboard Minimises,hide_keyboard,,
+75.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+76. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+77. Wait for Toast to Hide,wait,3000,,
+78. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+79. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+80. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+81. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+82. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+83. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+84.Wait For Hamburger Menu,wait,3000
+85. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+86.Wait For Driver Profile Load,wait,3000,
+87. Drag Page Layout Upward,swipe,up,
+88.Wait For Language Menu,wait,3000,
+89.Click Language Button,tap_coordinate,546:1624,COORDINATE_MODE
+90. Wait for Language Setting option,wait,3000,,
+91. Click Select Tamil Language,tap,,"mobile.driver.Language.Tamil.button"
+92. Click Select Tamil Language Update,tap,,"mobile.driver.menu.Language.save_changes.btn"
+93. Wait for Language Setting option,wait,3000,,
+94. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+95. Drag Page Layout Upward,swipe,up,
+96.Wait For Page Load,wait,3000,
+97.Click Language Button,tap_coordinate,546:1624,COORDINATE_MODE
+98. Wait for Language Setting option,wait,3000,,
+99. Click Select Hindi Language,tap,,"mobile.driver.Language.Hindi.button"
+100. Click Select Hindi Language Update,tap,,"mobile.driver.menu.Language_Tamil.save_changes.btn"
+101.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+102.Drag Page Layout Upward,swipe,up,
+103.Wait For Page Load,wait,3000,
+104.Click Language Button,tap_coordinate,546:1624,COORDINATE_MODE
+105.Wait for Language Setting option,wait,3000,,
+106.Click Select English Language,tap,,"mobile.driver.Language.English.button"
+107.Click Select English Language Update,tap,,"mobile.driver.menu.Language_Hindi.save_changes.btn"
+108. Wait for Language Setting option,wait,3000,,
+109.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+110.Drag Page Layout Upward,swipe,up,
+111.Wait for Manage Account Loading,wait,3000,,
+112.Click Manage Account,tap_coordinate,503:2084,COORDINATE_MODE
+113.Click Delete Account,tap,,"mobile.driver.delete.btn"
+114.Click Delete Account Sure,tap,,"mobile.driver.delete_sure.btn"
+115.Switch To Web Session,switch_to,web,
+116. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+117. Click drivers menu,click,,"admin.drivers.menu.icon"
+118.Click Delete Driver,click,,"admin.drivers.delete_drivers.menu"
+119.Wait For Load,wait,1000,
+120. Enter Driver Name,type,{autoName},"admin.drivers.name_filter.input" 
+121.Wait For Load,wait,3000,</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3.  Switch To Web Session,switch_to,web,
+4.Click Dashboard,Click,,"web.global.menu.dashboard"
+5.Click Setting Button,click,,"admin.setting.sidebar.menu"
+6.Click Geo Fencing,click,,"admin.setting.geo_fencing.sidebar_menu"
+7.Add Restrict Area,click,,"admin.setting.geo_fencing.add_restricted_area_btn"
+8.Enter Restricted Area Name,type,officers training academy chennai,"admin.setting.geo_fencing.area_name_input_field"
+9.Click The Status Button On,click,,"admin.setting.geo_fencing.status_toggle_button"
+10. Enter Search Location,type,officers training academy chennai,"admin.city_area.input_search_location"
+11.Wait For Options To Load,wait,3000,
+12. Select First Option,arrow_down,,"admin.city_area.input_search_location"
+13. Confirm Option,press_enter,,"admin.city_area.input_search_location"
+14. Wait For Map To Load,wait,3000,
+15.Map Polygon,draw polygon,"-60;-60 : 60;-60 : 60;60 : -60;60","//div[@class='ol-layer']//canvas"
+16.Wait For Polygon Draw,wait,3000,
+17.Click Submit Button,click,,"admin.setting.geo_fencing.form_submit_button"
+18.Wait For Submit,wait,2000,
+19.Load Driver App,switch_to,driver,
+20.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+21.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+22.Force Driver Location Officers Academy Chennai,set_location,12.998359;80.192347,
+23.Click Agree,tap,,"mobile.driver.agree.btn"
+24.Click Get Started,tap,,"mobile.driver.get_started.btn"
+25.Click Next,tap,,"mobile.driver.next.btn"
+26.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+27.Click Close,tap,,"mobile.driver.cancel.btn"
+28.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+29.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+30. Click Continue,tap,,"mobile.driver.continue.btn"
+31. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+32.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+33.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+34.Wait For Pageload,wait,5000,
+35.Load User App,switch_to,user,
+36.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+37.Click Get Started,tap,,"mobile.customer.get_started.btn"
+38.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+39.Force User Location Officers Academy Chennai,set_location,12.998359;80.192347,
+40.Click Next,tap,,"mobile.customer.next.btn"
+41.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+42.Click Close,tap,,"mobile.customer.cancel.btn"
+43.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+44.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+45.Click Continue,tap,,"mobile.customer.continue.btn"
+46.Enter OTP,type,123456,"mobile.customer.otp_input"
+47.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+48.Click Finish,tap,,"mobile.customer.finish.btn"
+49.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50.Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+51. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+52. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+53. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+54. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+55. Select Destination,tap,,"mobile.customer.destination_suggestion_first"
+56.Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
+57.Click Entrance,tap,,"mobile.customer.destination_entrance_location"
+58. Click Confirm,tap,,"mobile.customer.confirm.btn"
+59.Wait For Ride,wait,5000,
+60. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+61. Ride Now,tap,,"mobile.customer.ride_now.btn"
+62.Wait For Geo Fencing Message,wait,5000,
+63. Load Driver App,switch_to,driver,
+64.Wait For Drive App,wait,5000 
+65.Verify Driver App Didnot Recieve Ride From Geo Fenced Area,element_absent,,"mobie.driver.auto_ride_accept.button"
+66.Wait For Checking,wait,3000,
+67.Switch To Web Session,switch_to,web,
+68.Click Dashboard,Click,,"web.global.menu.dashboard"
+69.Click Setting Button,click,,"admin.setting.sidebar.menu"
+70.Click Geo Fencing,click,,"admin.setting.geo_fencing.sidebar_menu"
+71.Enter Search Area,type,officers training academy chennai,"admin.setting.geo_fencing.area_search_filter"
+72.Wait For Load,wait,2000,
+73.Click Delete Button,click,,"admin.setting.geo_fencing.delete_button"
+74.Click Yes Delete It Button,click,,"admin.setting.geo_fencing.confirm_delete_button"
+75.Wait For Delete,wait,2000,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Driver App,switch_to,driver,
+4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6.Force Driver Location To Perambur,set_location,13.121030;80.232578,
+7.Click Agree,tap,,"mobile.driver.agree.btn"
+8.Click Get Started,tap,,"mobile.driver.get_started.btn"
+9.Click Next,tap,,"mobile.driver.next.btn"
+10.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+11.Click Close,tap,,"mobile.driver.cancel.btn"
+12.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+13.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+14.Click Continue,tap,,"mobile.driver.continue.btn"
+15.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+16.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+17.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+18.Wait For Driver App Toggle On,wait,3000,
+19.Load User App,switch_to,user,
+20.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+21.Click Get Started,tap,,"mobile.customer.get_started.btn"
+22.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+23.Force User Location To Perambur,set_location,13.121030;80.232578,
+24.Click Next,tap,,"mobile.customer.next.btn"
+25.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+26.Click Close,tap,,"mobile.customer.cancel.btn"
+27.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+28.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+29. Click Continue,tap,,"mobile.customer.continue.btn"
+30. Enter OTP,type,123456,"mobile.customer.otp_input"
+31. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+32. Click Finish,tap,,"mobile.customer.finish.btn"
+33. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+34. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+35.Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+36.Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+37.Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+38.Select Destination,tap,,"mobile.customer.destination_suggestion_first"
+39.Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
+40.Click Entrance,tap,,"mobile.customer.destination_entrance_location"
+41. Click Confirm,tap,,"mobile.customer.confirm.btn"
+42.Wait For Ride,wait,5000,
+43.Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+44.Ride Now,tap,,"mobile.customer.ride_now.btn"
+45.Load Driver App,switch_to,driver,
+46.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+47.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+48.Load User App,switch_to,user,
+49.Wait for OTP Layout to Load,wait_until_visible,,"mobile.customer.otp_display_element"
+50.Extract OTP from Screen,store_text,ride_otp,"mobile.customer.otp_display_element"
+51.Load Driver App,switch_to,driver,
+52.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+53.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+54.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+55.Ride Arrived,tap,,"mobile.driver.arrived.btn"
+56.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+57.Yes Arrived,tap,,"mobile.driver.yes.btn"
+58.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+59.Start Ride,tap,,"mobile.driver.start_ride.btn"
+60.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+61.Enter  Extracted OTP,type,{ride_otp},"mobile.driver.otp_view.input"
+62.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+63.Start Ride Button,tap,,"mobile.driver.start.btn"
+64.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+65.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+66.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+67.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+68.Load User App,switch_to,user,
+69.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+70.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+71. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+72. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+73. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+74. Give Review,tap,,"mobile.customer.give_review.btn"
+75. Give Rating,tap_coordinate,348:1619,
+76. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+77.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+78.Trip Finished,tap,,"mobile.customer.done.btn"
+79. Load Driver App,switch_to,driver,
+80.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
+81.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
+82. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+83. Confirm Payment,tap,,"mobile.driver.yes.btn"
+84.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
+85.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
+86.Wait For Rating,wait,2000,
+87. Give Rating,tap_coordinate,348:1545,
+88. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+89.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
+90.Click Complete Button,tap,,"mobile.driver.complete.btn"
+91.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
+92.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3. Load Driver App,switch_to,driver,
+4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6. Click Agree,tap,,"mobile.driver.agree.btn"
+7. Click Get Started,tap,,"mobile.driver.get_started.btn"
+8. Click Next,tap,,"mobile.driver.next.btn"
+9. Click Mobile Number Button,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap_if_present,,"mobile.driver.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;driverNumber,"mobile.driver.edit_text.input"
+12.Wait For Continue,wait_until_visible,,"mobile.driver.continue.btn"
+13.Click on Continue,tap,,"mobile.driver.continue.btn"
+14. wait for OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+15. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+16. Wait for Finish,wait_until_visible,,"mobile.driver.finish.btn"
+17. Click on Finish,tap,"mobile.driver.finish.btn"
+18.Wait For Profile Registation Page,wait_until_visible,"mobile.driver.Register.profile.pen_icon"
+19.Click on ProfileImage,tap,,"mobile.driver.Register.profile.pen_icon"
+20.Wait For Camera,wait_until_visible,"mobile.driver.Camera.btn"
+21.Click on camera,tap,,"mobile.driver.Camera.btn"
+22.Click while using this app Notification,tap,,"mobile.driver.camera_allow.btn"
+23.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+24.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+25.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+26.Type Driver Name,type,autoDriver{randomAlpha}&gt;&gt;driverName,"mobile.driver.driver_name_input"
+27.Wait For Keyboard Minimises,hide_keyboard,,
+28.Click Whatapp Checkbox,tap_coordinate ,165:1097,COORDINATE_MODE
+29.Enter Email,type,{driverName}@gmail.com&gt;&gt;driverEmail,"mobile.driver.driver_email_input"
+30.Wait For Keyboard Minimises,hide_keyboard,,
+31.Click  Gender Box Male,tap,,"mobile.driver.select_gender_male"
+32.Scroll Screen,swipe,up,
+33.Click  Social Media,tap,,"mobile.driver.how_did_you_hear_about_us"
+34.Select Instagram,tap,,"mobile.driver.select_option_instagram"
+35.Click Terms And Conditions,tap_coordinate ,124:1758,COORDINATE_MODE
+36.Click Sign Up,tap,,"mobile.driver.sign_up_btn"
+37.Wait For Vehicle Type,wait_until_visible,"mobile.driver.Service_vehicle_Type_heading"
+38.Select Auto Ride,tap,,"mobile.driver.select_auto_ride"
+39.Click Next,tap,,"mobile.driver.auto_ride_next_btn"
+40.Wait for Pop Up,wait_if_present,,"mobile.driver.driver_location_allow.btn"
+41.Click While Using This App Notification,tap_if_present,,"mobile.driver.driver_location_allow.btn"
+42.Click Upload image Icon,tap,,"mobile.driver.vehicle_image_upload_icon"
+43.Click on camera,tap,,"mobile.driver.Camera.btn"
+44.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+45.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+46.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+47.Click Select Vehicle Type Dropdown,tap,,"mobile.driver.vehicle_type_dropdown"
+48.Select Option Pink Auto,tap,,"mobile.driver.vehicle_type_option.pink_auto"
+49.Type Model Name,type,petrol,"mobile.driver.vehicle_model_name.input_box"
+50.Click Vehicle Model Year,tap,,"mobile.driver.vehicle_type_model_year.dropdown"
+51.Select Year,tap,,"mobile.driver.vehicle_type_model_year.option_year"
+52..Type Vehicle Plate No,type,TN22CL5170,"mobile.driver.Vehicle_plate_number"
+53.Click the Seat Number,tap,,"mobile.driver.select_seat_number.drop_down"
+54.Select Number Of Seat,tap,"mobile.driver.select_seat_number.option_three"
+55.Scroll Screen,swipe,up,
+56.Type Vehicle Color,type,Pink,"mobile.driver.Vehicle_colour"
+57.Save Vehicle Detaills,tap,,"mobile.drivers_vehicle_details.save_btn"
+58. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+59. Click Upload,tap,,"mobile.driver.upload.btn"
+60. Upload License,tap,,"mobile.driver.upload_docs.btn"
+61.Click on camera,tap,,"mobile.driver.Camera.btn"
+62.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+63.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+64.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+65. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+66. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+67. Click Month,tap,,"mobile.driver.next_month.btn"
+68. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+69. Click Ok,tap,,"mobile.driver.ok.btn"
+70. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+71.Click Next Button,tap,,"mobile.drivers.after_upload_doc.next_btn"
+72.Enter Account Holder,type,{driverName},"mobile.driver.bank_details.account_holder_name"
+73.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+74.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+75.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+76.Wait For Keyboard Minimises,hide_keyboard,,
+77.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+78.Wait For Keyboard Minimises,hide_keyboard,,
+79.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+80.Wait For Logout,wait_until_visible,"mobile.drivers.after_upload_doc.logout_btn"
+81.Click Logout,tap,,"mobile.drivers.after_upload_doc.logout_btn"
+82.Click Confirm Logout,tap,,"mobile.drivers.after_upload_doc.logout_confirm_btn"
+83.Reload Driver App Completely,reload_app,driver,
+84.Load Admin App,switch_to,web,
+85.Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+87.Click drivers menu,click,,"admin.drivers.menu.icon"
+88.Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+89.Filter by Name,type,{driverName},"admin.drivers.name_filter.input"
+90.Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+91. Click Doc Icon,click,,"admin.drivers.docs.icon"
+92. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
+93. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+94. Click Approve Driver,click,,"admin.drivers.docs.approval"
+95. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
+96. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+97. Click drivers menu,click,,"admin.drivers.menu.icon"
+98. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+99.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
+100. Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
+101. Load Driver App,switch_to,driver,
+102.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+103.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+104.Click Agree,tap,,"mobile.driver.agree.btn"
+105.Click Get Started,tap,,"mobile.driver.get_started.btn"
+106.Click Next,tap,,"mobile.driver.next.btn"
+107.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+108.Click Close,tap,,"mobile.driver.cancel.btn"
+109.Enter Mobile Number,type,{driverNumber},"mobile.driver.edit_text.input"
+110.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+111.Click Continue,tap,,"mobile.driver.continue.btn"
+112.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+113.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+114.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+115.Wait For Pageload,wait,3000,
+</t>
+  </si>
+  <si>
+    <t>This test case validates the end-to-end onboarding, registration, and administrative approval pipeline for new service providers on the platform. The automated workflow begins on the native Driver Mobile App, executing a complete registration sequence that includes mobile OTP verification, profile selfie uploads, detailed vehicle configuration (such as selecting a "Pink Auto" model), document submission with dynamic expiration dates, and bank account onboarding. Execution then switches context to the Web Admin Portal, where the script acts as a system administrator to filter the pending queues by the dynamically generated driver name, verify the uploaded driving license, and formally authorize the profile status. The test concludes by switching back to the mobile simulator to confirm that the newly approved driver can successfully bypass onboarding restrictions and authenticate into the active service dashboard</t>
+  </si>
+  <si>
+    <t>SA_TS_12</t>
+  </si>
+  <si>
+    <t>TC_CA_12_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>TC_CA_11_Driver_Registration_Mobile_App</t>
   </si>
 </sst>
 </file>
@@ -3177,6 +3636,88 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D336680-5C86-4607-94FA-F265347A7E84}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77578C42-408B-4BD1-8455-A36E9774F1FD}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3219,22 +3760,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>109</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>50</v>
@@ -3260,7 +3801,87 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91EB8016-EA4B-41B6-8140-24B0AE352F99}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3302,13 +3923,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>
@@ -3334,7 +3955,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A659562-16FE-472A-9348-C2754F8B87F9}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3377,22 +3998,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>50</v>
@@ -3418,7 +4039,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E5A465-4C2B-4523-8755-30CE3021A8BD}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3461,13 +4082,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>34</v>
@@ -3497,7 +4118,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DE31E4-5C3B-413E-B08A-861302F9F4DC}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3539,13 +4160,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>37</v>
@@ -3572,7 +4193,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3614,13 +4235,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
@@ -3690,19 +4311,19 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>48</v>
@@ -3777,23 +4398,21 @@
         <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>46</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -3858,25 +4477,25 @@
         <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3942,19 +4561,19 @@
         <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -4026,19 +4645,19 @@
         <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -4113,16 +4732,16 @@
         <v>54</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -4197,19 +4816,19 @@
         <v>55</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -4218,9 +4837,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -4273,22 +4890,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>50</v>

</xml_diff>

<commit_message>
99th Commit: All Test Cases Foramtted to  New Excel Format
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828ED715-67AD-4306-9110-259869EB71C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1011925-D054-4851-9273-BF99E6AFCC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -41,18 +41,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="150">
   <si>
     <t>Requirement Title</t>
   </si>
   <si>
-    <t>Test Case ID(s)</t>
-  </si>
-  <si>
     <t>Test Case Description</t>
-  </si>
-  <si>
-    <t>Test Step Description</t>
   </si>
   <si>
     <t>Precondition</t>
@@ -506,9 +500,6 @@
   </si>
   <si>
     <t>User Driver Web Intialilzer</t>
-  </si>
-  <si>
-    <t>TC_CA_00_User_Driver_Web_Intializer</t>
   </si>
   <si>
     <t>This test case loads user app in emulator 5554  and loads driver app in emulator 5556 and login as superadmin in web.</t>
@@ -1352,9 +1343,6 @@
     <t>SA_TS_0B</t>
   </si>
   <si>
-    <t>TC_CA_01_Hybrid_Subscription_Plan_Test</t>
-  </si>
-  <si>
     <t>This comprehensive, cross-platform regression test suite validates the entire lifecycle of a customer account by seamlessly orchestrating actions between native mobile applications and the centralized web administration portal. The test sequence begins by initializing a fresh mobile session using the reload_app utility, executing a new user registration flow via dynamic device permissions, randomized phone generation, and OTP simulation. The execution then seamlessly switches context to the web portal to locate the newly created profile under the Non-Verified Customers matrix, populates missing metadata (including automated profile image uploads and randomized alpha naming strings), and submits the profile to trigger status escalation. After confirming the user's migration into the Verified Customers data grid, the execution switches back to the mobile application instance to verify verified account access. Finally, the test validates data-compliance workflows by triggering a native Delete Account chain from the mobile device settings and cross-verifying that the user profile is immediately and correctly relocated to the web admin’s Deleted Customers repository.</t>
   </si>
   <si>
@@ -1364,13 +1352,7 @@
     <t>This end-to-end, cross-platform regression test suite orchestrates a complex testing lifecycle for driver management by coordinating operations between the central web administration portal and native mobile driver application runtimes. The execution flow begins by initializing clean device environments using the reload_app keyword and shifts context to the web portal to register a new driver profile with comprehensive metadata mapping—including automated profile picture uploads, customized vehicle specifications ("Pink Auto"), and corporate banking infrastructure parameters. The test then executes a multi-tiered regulatory validation pipeline by locating the profile in the Pending Documents grid, uploading a simulated driving license file with an active expiry date, and escalating the profile to the official Approved Drivers registry. Transitioning into the native mobile engine environment, the suite authenticates the newly approved driver using dynamic OTP routing, processes specialized compliance checkboxes, and thoroughly audits the application's localization subsystem by executing dynamic runtime language shifts—transitioning the interface seamlessly from English to Tamil, Tamil to Hindi, and back to English. Finally, the suite tests legal compliance and lifecycle termination rules by triggering a native Delete Account flow from the driver app interface and verifying that the record instantly relocates to the web admin's Deleted Drivers repository under localized filtering conditions.</t>
   </si>
   <si>
-    <t>TC_CA_02_Driver_App_Wallet_Verification</t>
-  </si>
-  <si>
     <t>Customer App Wallet Check</t>
-  </si>
-  <si>
-    <t>TC_CA_03_Customer_App_Wallet_Check</t>
   </si>
   <si>
     <t>This end-to-end hybrid regression test verifies the runtime visibility and functionality of the mobile Customer Wallet module based on configurations managed within the Super Admin Web Portal. The execution workflow first activates the wallet feature via the admin portal's site settings, logs into the customer application, and executes a full simulated wallet top-up transaction using Net Banking to confirm operational stability. It then reverts to the web panel to toggle the wallet status to "OFF," restarts the mobile application context to clear active sessions, re-authenticates the customer, and explicitly asserts that the Wallet option is completely absent from the side menu hierarchy.</t>
@@ -1717,9 +1699,6 @@
   </si>
   <si>
     <t>Non Verified And Delete Customer</t>
-  </si>
-  <si>
-    <t>TC_CA_04_Non_Verified_And_Deleted_Customer</t>
   </si>
   <si>
     <t>SA_TS_08</t>
@@ -1826,9 +1805,6 @@
   </si>
   <si>
     <t>Add Customer App Emergency Number</t>
-  </si>
-  <si>
-    <t>TC_CA_05_Add_Customer_App_Emergency_Number</t>
   </si>
   <si>
     <t>This end-to-end regression test suite validates native customer onboarding workflows and profile property mutations across mobile and web runtime interfaces. The test sequence begins by executing a clean app initialization loop, walking through device access configuration, and utilizing dynamic runtime token generation to process mobile OTP verification steps. It then completes native in-app self-registration by populating customer metadata fields (name strings, email structures, gender flags, and legal checklists) before interacting with coordinate boundaries to locate the account drawer profiles. Crucially, the script provisions an active fallback record inside the native Emergency Contact subsystem, saves the payload, and tests intent handling by triggering the emergency alert call mechanism. Finally, the test switches to the web administration platform to locate the freshly synchronized account record inside the Verified Customers data matrix, opening the admin's inline panel to execute data-integrity lookups against the updated emergency phone element bounds.</t>
@@ -1963,12 +1939,6 @@
 121.Wait For Load,wait,3000,</t>
   </si>
   <si>
-    <t>TC_CA_06_Customer_Language_Check</t>
-  </si>
-  <si>
-    <t>TC_CA_07_Driver_Language_Check</t>
-  </si>
-  <si>
     <t>Auto Ride Complete Life Cycle Test With Otp Fetched From DB</t>
   </si>
   <si>
@@ -2323,31 +2293,10 @@
 85.Wait For Resolved Issue To Load,wait,5000,</t>
   </si>
   <si>
-    <t>TC_CA_0A_Autoride_Test_Otp_DB</t>
-  </si>
-  <si>
-    <t>TC_CA_0B_Hybrid_Add_Customer</t>
-  </si>
-  <si>
-    <t>TC_CA_0C_Hybrid_Unapproved_Auto_Driver</t>
-  </si>
-  <si>
     <t>SA_TS_0D</t>
   </si>
   <si>
-    <t>TC_CA_0D_Hybrid_Approved_Auto_Driver</t>
-  </si>
-  <si>
-    <t>TC_CA_08_Completed_Ride_Customer_Report_Issue</t>
-  </si>
-  <si>
     <t>SA_TS_11</t>
-  </si>
-  <si>
-    <t>TC_CA_09_Geo_Fencing_Verification</t>
-  </si>
-  <si>
-    <t>TC_CA_10_Autoride_Test_Otp_Ui</t>
   </si>
   <si>
     <t>This test case validates the platform's ability to enforce active geo-fencing restrictions by automatically blocking mobile ride requests initiated from within a prohibited geographical zone. The automated workflow begins in the web administration panel, where the draw_polygon keyword is used to map and activate a restricted area around "Officers Training Academy Chennai." Execution then switches to the native Driver and Customer mobile applications sequentially, utilizing the set_location keyword to inject matching restricted GPS coordinates into both emulator sessions mid-execution. The test concludes by attempting to book an active ride from the customer application and executing a final timeout validation to confirm that the platform successfully intercepts and blocks the order request due to the active boundary constraint.</t>
@@ -3185,10 +3134,311 @@
     <t>SA_TS_12</t>
   </si>
   <si>
-    <t>TC_CA_12_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>TC_CA_11_Driver_Registration_Mobile_App</t>
+    <t>Test Case ID [Manual]</t>
+  </si>
+  <si>
+    <t>Test Case ID [Regression]</t>
+  </si>
+  <si>
+    <t>TC_RG_00_User_Driver_Web_Intializer</t>
+  </si>
+  <si>
+    <t>TC_HY_00_User_Driver_Web_Intializer</t>
+  </si>
+  <si>
+    <t>Manual Test  Steps</t>
+  </si>
+  <si>
+    <t>Regression Test Steps</t>
+  </si>
+  <si>
+    <t>1. Launch the User mobile application and wait for the "Get Started" screen to appear.
+2. Launch the Driver mobile application and wait for the notification permission prompt.
+3. Launch the Super Admin web portal and wait for the login page to load.
+4. Enter the Super Admin credentials (Email: super_admin@gmail.com and Password) and click the Login button.
+5. Verify that the Super Admin successfully logs in and the main Dashboard page is displayed.</t>
+  </si>
+  <si>
+    <t>TC_RG_01_Hybrid_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>TC_RY_01_Hybrid_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Subscription Plan &gt; Driver Subscription Plan and click "Add New Subscription".
+2. Create a Driver Subscription Plan:
+   - Select Service Category ("Auto Ride").
+   - Enter Plan Name in English, Arabic, Tamil, and Hindi.
+   - Enter Validity (100 days), Free Rides (2), Price (50), and multi-language Descriptions.
+   - Set Status to On and submit.
+3. Navigate to Subscription Plan &gt; Customer Subscription Plan and click "Add New Subscription".
+4. Create a Customer Subscription Plan:
+   - Select Service Category ("Auto Ride").
+   - Enter Plan Name in English, Arabic, Tamil, and Hindi.
+   - Enter Validity (100 days), Free Rides (2), Price (50), and multi-language Descriptions.
+   - Set Status to On and submit.
+5. Launch the Customer Mobile App, log in via phone number and OTP, navigate to Profile &gt; Subscription, and verify that the newly created customer subscription plan is displayed.
+6. In Super Admin, go to Settings &gt; Site Settings and ensure the Wallet Status is set to ON.
+7. Launch the Driver Mobile App, log in via phone number and OTP, open the side menu, and navigate to Subscription.
+8. Select the newly created driver subscription plan, pay and activate the plan using Wallet Payment, and then test canceling the active subscription.
+9. In Super Admin, navigate back to Customer Subscription Plan, search for the created plan, and delete it.
+10. Navigate to Driver Subscription Plan, search for the created plan, and delete it.</t>
+  </si>
+  <si>
+    <t>TC_RG_02_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <t>TC_HY_02_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Settings &gt; Site Settings, set the Wallet Status dropdown to ON, and save the settings.
+2. Launch and set up the Driver Mobile App, log in using phone number and OTP, and navigate to the Wallet section via the side menu.
+3. Initiate a wallet top-up by selecting an amount (100) and complete the transaction using Net Banking (BOB).
+4. Verify top-up success, navigate back, and reload the Driver App.
+5. Return to Super Admin Site Settings, change the Wallet Status dropdown to OFF, and save the changes.
+6. Re-launch and log into the Driver App, open the side menu, and verify that the Wallet option is no longer visible/present.
+7. In Super Admin, revert the Wallet Status setting back to ON and save changes to restore wallet functionality.</t>
+  </si>
+  <si>
+    <t>TC_RG_03_Customer_App_Wallet_Check</t>
+  </si>
+  <si>
+    <t>TC_HY_03_Customer_App_Wallet_Check</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Settings &gt; Site Settings, set the Wallet Status dropdown to ON, and save the settings.
+2. Launch and set up the User Mobile App, log in using phone number and OTP, navigate to Profile, and verify that the Wallet button is present.
+3. Reload the User App.
+4. Return to Super Admin Site Settings, change the Wallet Status dropdown to OFF, and save the changes.
+5. Re-launch and log into the User App, navigate to Profile, and verify that the Wallet option is no longer visible/present.
+6. In Super Admin, revert the Wallet Status setting back to ON and save changes to restore wallet functionality.</t>
+  </si>
+  <si>
+    <t>TC_RG_04_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>TC_HY_04_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>1. Launch the User Mobile App, register a new account using a random phone number, and enter the OTP to reach the landing page.
+2. Open the Super Admin portal, navigate to Non-Verified Customers, filter by the registered phone number, and click Edit.
+3. Complete the profile details (Full Name, Email, Emergency Contact, Gender: Male, Profile Image) and submit to update the customer account.
+4. Navigate to Verified Customers in Super Admin and verify that the updated customer is listed under verified users.
+5. Re-launch the User Mobile App and log in with the verified phone number and OTP.
+6. Navigate to Profile &gt; Manage Account, select Delete Account, and confirm account deletion.
+7. Return to Super Admin, navigate to Deleted Customers, filter by the Customer Name, and verify that the account appears in the deleted customers list.</t>
+  </si>
+  <si>
+    <t>TC_RG_05_Add_Customer_App_Emergency_Number</t>
+  </si>
+  <si>
+    <t>TC_HY_05_Add_Customer_App_Emergency_Number</t>
+  </si>
+  <si>
+    <t>1. Launch the User Mobile App and initiate registration using a random phone number and OTP.
+2. Complete customer registration in the app by entering Full Name, Email, Gender (Male), accepting terms, and granting location permissions to reach the home screen.
+3. Navigate to Profile &gt; Emergency Contact and select "Add Emergency Contact".
+4. Enter a random Emergency Phone Number, click Update, and trigger the Emergency Call button.
+5. Open the Super Admin portal, navigate to Customer Icon &gt; Verified Customers, and filter the list by Customer Name.
+6. Open the customer edit modal via the Pencil (Edit) button to view saved customer details.
+7. Verify that the Emergency Contact Number stored in Super Admin matches the emergency number updated in the User App.</t>
+  </si>
+  <si>
+    <t>TC_RG_06_Customer_Language_Check</t>
+  </si>
+  <si>
+    <t>TC_HY_06_Customer_Language_Check</t>
+  </si>
+  <si>
+    <t>1. Launch the User Mobile App, register a new account using a random phone number, and enter the OTP to reach the landing page.
+2. Open the Super Admin portal, navigate to Non-Verified Customers, filter by the registered phone number, and click Edit.
+3. Complete profile details (Full Name, Email, Emergency Contact, Gender: Male, Profile Image) and submit to verify the customer.
+4. Verify that the updated customer is listed under Verified Customers in Super Admin.
+5. Re-launch the User Mobile App, log in with the verified phone number and OTP, and navigate to Profile &gt; Language Settings.
+6. Test multi-language updates in the User App:
+   - Switch language to Tamil and save changes.
+   - Switch language to Hindi and save changes.
+   - Switch language back to English and save changes.
+7. Navigate to Profile &gt; Manage Account, select Delete Account, and confirm account deletion.
+8. Open Super Admin, navigate to Deleted Customers, filter by Customer Name, and verify that the account appears in the deleted list.</t>
+  </si>
+  <si>
+    <t>TC_RG_07_Driver_Language_Check</t>
+  </si>
+  <si>
+    <t>TC_HY_07_Driver_Language_Check</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Drivers &gt; Add Driver and enter all required driver details (Service Category: Auto Ride, Driver Type: Pilot, Full Name, Email, Phone Number, WhatsApp Number, Profile Image, Source: Instagram, Gender: Male).
+2. Enter Vehicle details (Vehicle Type: Auto, Model Year: 2013, Plate Number, Model Name: Petrol, Vehicle Image) and Bank details (Bank Name: HDFC Bank, Location, Account Number, Holder Name, Payment Email, IFSC Code), then submit to create the driver.
+3. Navigate to Pending Documents, filter for the created Driver Name, upload the Driving License with an expiry date, and approve the driver document.
+4. Navigate to Approved Drivers and confirm the driver is listed in the approved state.
+5. Launch the Driver Mobile App, log in with the registered phone number and OTP, and enter the bank/UPI details to complete setup.
+6. Grant location permissions, accept the Independent Contractor agreement, and enter the OTP to reach the driver home screen.
+7. Open the Driver App side menu, navigate to Language Settings, and verify multi-language functionality by switching through Tamil, Hindi, and back to English.
+8. Navigate to Manage Account, select Delete Account, and confirm account deletion in the Driver App.
+9. Return to Super Admin, navigate to Drivers &gt; Deleted Drivers, filter by Driver Name, and verify that the deleted driver account appears in the list.</t>
+  </si>
+  <si>
+    <t>TC_RG_08_Completed_Ride_Customer_Report_Issue</t>
+  </si>
+  <si>
+    <t>TC_HY_08_Completed_Ride_Customer_Report_Issue</t>
+  </si>
+  <si>
+    <t>1. Launch the User Mobile App, log in using phone number and OTP, and navigate to Profile &gt; My Orders.
+2. Filter orders using the "All" orders option and navigate to the Completed Rides tab.
+3. Select a completed ride, open the options menu (three dots), and select "Report Issue".
+4. Enter the issue description ("Bad Behaviour Of Driver"), attach a photo captured via camera, and submit the ticket.
+5. Note the generated Ticket ID, open the Report Issue Chat, send a follow-up message to Support, and switch session to Web.
+6. In Super Admin, navigate to Report Issue &gt; Customer Report Issues.
+7. Filter by Customer Name and Unresolved status, view issue details, and open the Chat module.
+8. Send a support reply to the customer and update the issue status to Resolved.
+9. Return to the User Mobile App, navigate back to Profile &gt; Report Issue, and verify that the ticket appears in the Resolved Issues list.</t>
+  </si>
+  <si>
+    <t>TC_RG_09_Geo_Fencing_Verification</t>
+  </si>
+  <si>
+    <t>TC_HY_09_Geo_Fencing_Verification</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Settings &gt; Geo Fencing and click "Add Restricted Area".
+2. Enter the restricted area name ("Officers Training Academy Chennai"), enable the status toggle, search for the location, and draw a polygon on the map to define the restricted area.
+3. Submit and save the new Geo Fencing restricted area.
+4. Launch the Driver Mobile App, log in, and set the driver's mock location inside the restricted area (Officers Training Academy Chennai).
+5. Launch the User Mobile App, log in, set the user's location inside the restricted area, and attempt to book an Auto Ride to a specified destination ("Parsn Manere").
+6. Request a ride ("Ride Now") from within the Geo-fenced restricted area.
+7. Switch to the Driver App and verify that the driver does NOT receive any ride request coming from the restricted Geo-fenced zone.
+8. Return to Super Admin, navigate to Settings &gt; Geo Fencing, filter for the created restricted area, and delete it to clean up configuration.</t>
+  </si>
+  <si>
+    <t>1. Launch the Driver Mobile App, log in using phone number and OTP, set location to Perambur, and switch status to Online.
+2. Launch the User Mobile App, log in using phone number and OTP, and set location to Perambur.
+3. Select "Auto Ride", enter destination ("Parsn Manere"), select entrance location, confirm booking, and request a ride ("Ride Now").
+4. Switch to the Driver App and accept the incoming ride request.
+5. Switch to the User App, view the generated Ride OTP, and store it.
+6. Switch to the Driver App, update ride status to "Arrived", confirm arrival, and initiate "Start Ride".
+7. Enter the retrieved Ride OTP in the Driver App to verify and start the trip.
+8. Drive to the destination, click "Complete Ride", and initiate payment collection.
+9. Switch to the User App, select Cash Payment via "Proceed to Pay", rate the driver, submit feedback, and complete the trip.
+10. Switch back to the Driver App, confirm cash payment collection, rate the user, and submit the final ride completion form.</t>
+  </si>
+  <si>
+    <t>TC_RG_11_Driver_Registration_Mobile_App</t>
+  </si>
+  <si>
+    <t>TC_HY_11_Driver_Registration_Mobile_App</t>
+  </si>
+  <si>
+    <t>1. Launch the Driver Mobile App, enter a random phone number and OTP to initiate new driver registration.
+2. Complete profile registration:
+   - Upload a profile picture captured via camera (with crop).
+   - Enter Full Name, Email, Gender (Male), Source (Instagram), and accept Terms &amp; Conditions.
+3. Select Service Category ("Auto Ride") and upload vehicle information:
+   - Upload a vehicle photo.
+   - Select Vehicle Type ("Pink Auto"), enter Model Name, Model Year, Plate Number, Seat Count (3), and Color ("Pink").
+4. Upload required documents (Driving License with expiry date) and enter Bank/UPI details (Account Holder Name, Account Number, IFSC Code, UPI ID).
+5. Log out of the Driver App once registration is submitted.
+6. Open Super Admin portal, navigate to Drivers &gt; Pending Documents, filter by Driver Name, and approve the submitted Driving License document.
+7. Verify that the driver appears in the Approved Drivers list in Super Admin.
+8. Re-launch the Driver App, log in with the registered phone number and OTP, grant location permissions, and verify direct access to the driver home screen.</t>
+  </si>
+  <si>
+    <t>TC_RG_12_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>TC_HY_12_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>This is Data Clean Up sheet no manual test steps for it</t>
+  </si>
+  <si>
+    <t>TC_RG_0A_Autoride_Test_Otp_DB</t>
+  </si>
+  <si>
+    <t>1. Launch the Driver Mobile App, log in using phone number and OTP, turn the Online Status toggle ON, and keep the app ready.
+2. Launch the User Mobile App, log in using phone number and OTP, select "Auto Ride", enter destination ("Parsn Manere"), select entrance location, confirm booking, and request a ride ("Ride Now").
+3. Switch to the Driver App, accept the ride request, and fetch the Ride OTP directly from the database query.
+4. Update driver status to "Arrived", confirm arrival, initiate "Start Ride", and enter the fetched Ride OTP to start the trip.
+5. Complete the trip in the Driver App and click "Collect Payment".
+6. Switch to the User App, select Cash Payment via "Proceed to Pay", rate the driver, submit feedback, and finish the trip.
+7. Switch back to the Driver App, confirm cash payment collection, rate the customer, and submit the final ride completion details.</t>
+  </si>
+  <si>
+    <t>TC_RG_0B_Hybrid_Add_Customer</t>
+  </si>
+  <si>
+    <t>TC_SA_0B_Hybrid_Add_Custome</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Customer Icon &gt; Add Customers.
+2. Enter the new customer details:
+   - Full Name (e.g., customer + random string)
+   - Email Address
+   - Contact Phone Number
+   - Gender (Male)
+   - Profile Image
+3. Click Submit and wait for the success toast message ("Added Successfully").
+4. Navigate to Customer Icon &gt; Verified Customers.
+5. Filter the Verified Customers list by the newly created Customer Name to confirm successful registration and verification.</t>
+  </si>
+  <si>
+    <t>TC_RG_0C_Hybrid_Unapproved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>TC_HY_0C_Hybrid_Unapproved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Drivers &gt; Add Driver and ensure the Add Driver page loads.
+2. Select "Auto Ride" from the Service Category dropdown.
+3. Complete the driver profile details:
+   - Full Name (e.g., autodriver + random string)
+   - Email Address &amp; Contact Number
+   - WhatsApp Number (enable WhatsApp checkbox and reuse phone number)
+   - Upload Profile Image
+   - Select Source ("Instagram") and Gender ("Male")
+4. Complete the vehicle details:
+   - Select Vehicle Type ("Pink Auto")
+   - Enter Model Year (2013), Plate Number (KL-01-AB-1234), and Model Name ("petrol")
+   - Upload Vehicle Image
+5. Complete the bank details:
+   - Bank Name ("HDFC Bank"), Location ("Chennai"), Account Number, Account Holder Name, Payment Email, and IFSC Code
+6. Click Submit and wait for the success toast message confirming the driver has been added.
+7. Navigate to Drivers &gt; Pending Documents and filter the list by the newly created Driver Name to verify their application is pending document approval.</t>
+  </si>
+  <si>
+    <t>TC_RG_0D_Hybrid_Approved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>TC_HY_0D_Hybrid_Approved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>1. In Super Admin, navigate to Drivers &gt; Add Driver and verify that the Add Driver header displays.
+2. Select "Auto Ride" from the Service Category dropdown.
+3. Fill in the driver profile details:
+   - Full Name (e.g., autodriver + random string)
+   - Email Address &amp; Contact Phone Number
+   - WhatsApp Number (enable WhatsApp checkbox and reuse phone number)
+   - Profile Image upload
+   - Source ("Instagram") &amp; Gender ("Male")
+4. Fill in the vehicle details:
+   - Select Vehicle Type ("Pink Auto")
+   - Enter Model Year (2013), Plate Number (KL-01-AB-1234), and Model Name ("petrol")
+   - Upload Vehicle Image
+5. Fill in the bank details:
+   - Bank Name ("HDFC Bank"), Location ("Chennai"), Account Number, Account Holder Name, Payment Email, and IFSC Code
+6. Click Submit and verify the "Driver Added" success toast message.
+7. Navigate to Drivers &gt; Pending Documents and filter the list by the Driver Name.
+8. Click the Document icon, filter for "Driving Licence", upload the license file, enter the expiry date (12-12-2026), and submit.
+9. Click "Approve Driver" and verify the update success toast message.
+10. Navigate to Drivers &gt; Approved Drivers and filter by Driver Name to verify that the driver is listed as approved.</t>
+  </si>
+  <si>
+    <t>TC_RG_10_Autoride_Test_Otp_Ui</t>
+  </si>
+  <si>
+    <t>TC_HY_10_Autoride_Test_Otp_Ui</t>
   </si>
 </sst>
 </file>
@@ -3254,7 +3504,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3277,9 +3527,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3561,74 +3808,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA441742-FACE-4539-AA06-56BC1BB72A03}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="36.88671875" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="26.6640625" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" customWidth="1"/>
+    <col min="7" max="7" width="53.21875" customWidth="1"/>
+    <col min="8" max="8" width="36.88671875" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>32</v>
-      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3637,80 +3899,96 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D336680-5C86-4607-94FA-F265347A7E84}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="24.77734375" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="41.88671875" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" s="2"/>
+        <v>129</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="H2" s="2" t="s">
-        <v>101</v>
+        <v>62</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3719,82 +3997,97 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77578C42-408B-4BD1-8455-A36E9774F1FD}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="37.44140625" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>99</v>
+        <v>149</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>148</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>109</v>
+        <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>92</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3803,78 +4096,94 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91EB8016-EA4B-41B6-8140-24B0AE352F99}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="29.109375" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="46.33203125" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>114</v>
+        <v>132</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>111</v>
+        <v>131</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+        <v>133</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3883,70 +4192,85 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" customWidth="1"/>
+    <col min="4" max="4" width="26.77734375" customWidth="1"/>
+    <col min="5" max="6" width="34.109375" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" customWidth="1"/>
+    <col min="8" max="8" width="31.77734375" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="C2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="7"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
@@ -3957,82 +4281,98 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A659562-16FE-472A-9348-C2754F8B87F9}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="27.44140625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="40.109375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>91</v>
+        <v>137</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>137</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>138</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4041,77 +4381,91 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E5A465-4C2B-4523-8755-30CE3021A8BD}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="7" width="42.44140625" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="6" width="31.6640625" customWidth="1"/>
+    <col min="7" max="7" width="53.21875" customWidth="1"/>
+    <col min="8" max="8" width="29" customWidth="1"/>
+    <col min="9" max="9" width="42.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
+      <c r="H2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4120,73 +4474,89 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DE31E4-5C3B-413E-B08A-861302F9F4DC}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
-    <col min="4" max="4" width="35.5546875" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="29.6640625" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="3" max="3" width="33.109375" customWidth="1"/>
+    <col min="4" max="4" width="30.88671875" customWidth="1"/>
+    <col min="5" max="5" width="35.5546875" customWidth="1"/>
+    <col min="6" max="6" width="38.109375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="29.6640625" customWidth="1"/>
+    <col min="9" max="9" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>20</v>
+      <c r="I2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4195,70 +4565,84 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
-    <col min="4" max="4" width="35.5546875" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="29.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="30.88671875" customWidth="1"/>
+    <col min="5" max="6" width="35.5546875" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="29.6640625" customWidth="1"/>
+    <col min="9" max="9" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>145</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>40</v>
+        <v>147</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4267,82 +4651,97 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5DCFAC-B912-41EA-9964-A3839A72D798}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="52.44140625" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="51" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
     <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="52.44140625" customWidth="1"/>
+    <col min="10" max="10" width="40.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>19</v>
+      <c r="I1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>58</v>
+        <v>104</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>102</v>
+        <v>16</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>51</v>
-      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4351,80 +4750,96 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2DD3E8-3167-4AD5-B95A-26FB801D55E0}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="28.44140625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="45.77734375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4433,82 +4848,97 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0586A9D0-0ABC-41A4-8FF3-8503F348B496}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="6" width="29.109375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>74</v>
+      <c r="I2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4517,82 +4947,98 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437C624E-95B4-48EB-A315-8931C834404A}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="28.44140625" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="36.77734375" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4601,82 +5047,98 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0962450F-C7D8-41FC-90CD-CAAFB127F74F}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="3" max="3" width="27.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="39.21875" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4685,82 +5147,97 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D250DB7C-844B-4BAE-BD85-886B660DFD66}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="39.5546875" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4769,78 +5246,93 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B31CB41-AC3C-4084-88C1-98C363B7ABCB}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>82</v>
+        <v>122</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>61</v>
+        <v>121</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>107</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>123</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4849,82 +5341,97 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0BD74F5-8D47-475E-A6FE-D0E5567AC0D3}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="2" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="28.77734375" customWidth="1"/>
+    <col min="5" max="5" width="29.109375" customWidth="1"/>
+    <col min="6" max="6" width="41.5546875" customWidth="1"/>
+    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="8" max="8" width="40.44140625" customWidth="1"/>
+    <col min="9" max="9" width="61.88671875" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
+      <c r="I1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>124</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>52</v>
+        <v>62</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
100th Commit: Epic Wise Test Cases Created
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1011925-D054-4851-9273-BF99E6AFCC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70061456-D10C-451E-88BA-47961BBA076F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>

</xml_diff>